<commit_message>
doc(md): correcion del isa.md para instrucciones tipo T + otras correcciones para mayor claridad
</commit_message>
<xml_diff>
--- a/res/isa.xlsx
+++ b/res/isa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\workbench\repos\CE4301--p2_fobando_isa--\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DACEB4D-82D0-4DC9-8607-393D9ECB9FD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE3D8480-BDDA-4C64-87D7-B3C83CFA299D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{EC7525CD-E51C-4E61-B306-9CBCE090E85A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EC7525CD-E51C-4E61-B306-9CBCE090E85A}"/>
   </bookViews>
   <sheets>
     <sheet name="Encode" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="36">
   <si>
     <t>R</t>
   </si>
@@ -217,7 +217,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -277,11 +277,108 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -307,6 +404,12 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -319,8 +422,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -661,7 +788,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{173FC0BC-28E0-4D62-8DDD-273D10319523}">
-  <dimension ref="A2:AG12"/>
+  <dimension ref="A2:AG13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="33" width="3.109375" customWidth="1"/>
@@ -769,49 +896,49 @@
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="10" t="s">
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="10" t="s">
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="10" t="s">
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
+      <c r="R3" s="14"/>
+      <c r="S3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="T3" s="11"/>
-      <c r="U3" s="11"/>
-      <c r="V3" s="11"/>
-      <c r="W3" s="12"/>
-      <c r="X3" s="10" t="s">
+      <c r="T3" s="13"/>
+      <c r="U3" s="13"/>
+      <c r="V3" s="13"/>
+      <c r="W3" s="14"/>
+      <c r="X3" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="Y3" s="11"/>
-      <c r="Z3" s="11"/>
-      <c r="AA3" s="12"/>
-      <c r="AB3" s="10" t="s">
+      <c r="Y3" s="13"/>
+      <c r="Z3" s="13"/>
+      <c r="AA3" s="14"/>
+      <c r="AB3" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="AC3" s="11"/>
-      <c r="AD3" s="11"/>
-      <c r="AE3" s="11"/>
-      <c r="AF3" s="12"/>
+      <c r="AC3" s="13"/>
+      <c r="AD3" s="13"/>
+      <c r="AE3" s="13"/>
+      <c r="AF3" s="14"/>
       <c r="AG3" s="3" t="s">
         <v>16</v>
       </c>
@@ -820,47 +947,47 @@
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="12"/>
-      <c r="N4" s="10" t="s">
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
+      <c r="L4" s="13"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
-      <c r="R4" s="12"/>
-      <c r="S4" s="10" t="s">
+      <c r="O4" s="13"/>
+      <c r="P4" s="13"/>
+      <c r="Q4" s="13"/>
+      <c r="R4" s="14"/>
+      <c r="S4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="T4" s="11"/>
-      <c r="U4" s="11"/>
-      <c r="V4" s="11"/>
-      <c r="W4" s="12"/>
-      <c r="X4" s="10" t="s">
+      <c r="T4" s="13"/>
+      <c r="U4" s="13"/>
+      <c r="V4" s="13"/>
+      <c r="W4" s="14"/>
+      <c r="X4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="Y4" s="11"/>
-      <c r="Z4" s="11"/>
-      <c r="AA4" s="12"/>
-      <c r="AB4" s="10" t="s">
+      <c r="Y4" s="13"/>
+      <c r="Z4" s="13"/>
+      <c r="AA4" s="14"/>
+      <c r="AB4" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="AC4" s="11"/>
-      <c r="AD4" s="11"/>
-      <c r="AE4" s="11"/>
-      <c r="AF4" s="12"/>
+      <c r="AC4" s="13"/>
+      <c r="AD4" s="13"/>
+      <c r="AE4" s="13"/>
+      <c r="AF4" s="14"/>
       <c r="AG4" s="3" t="s">
         <v>16</v>
       </c>
@@ -869,34 +996,34 @@
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="12"/>
-      <c r="N5" s="10" t="s">
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="12"/>
-      <c r="S5" s="10" t="s">
+      <c r="O5" s="13"/>
+      <c r="P5" s="13"/>
+      <c r="Q5" s="13"/>
+      <c r="R5" s="14"/>
+      <c r="S5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="T5" s="11"/>
-      <c r="U5" s="11"/>
-      <c r="V5" s="11"/>
-      <c r="W5" s="12"/>
+      <c r="T5" s="13"/>
+      <c r="U5" s="13"/>
+      <c r="V5" s="13"/>
+      <c r="W5" s="14"/>
       <c r="X5" s="3" t="s">
         <v>19</v>
       </c>
@@ -909,13 +1036,13 @@
       <c r="AA5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AB5" s="10" t="s">
+      <c r="AB5" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="AC5" s="11"/>
-      <c r="AD5" s="11"/>
-      <c r="AE5" s="11"/>
-      <c r="AF5" s="12"/>
+      <c r="AC5" s="13"/>
+      <c r="AD5" s="13"/>
+      <c r="AE5" s="13"/>
+      <c r="AF5" s="14"/>
       <c r="AG5" s="3" t="s">
         <v>16</v>
       </c>
@@ -924,49 +1051,49 @@
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="10" t="s">
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="12"/>
-      <c r="N6" s="10" t="s">
+      <c r="J6" s="13"/>
+      <c r="K6" s="13"/>
+      <c r="L6" s="13"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="12"/>
-      <c r="S6" s="10" t="s">
+      <c r="O6" s="13"/>
+      <c r="P6" s="13"/>
+      <c r="Q6" s="13"/>
+      <c r="R6" s="14"/>
+      <c r="S6" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="T6" s="11"/>
-      <c r="U6" s="11"/>
-      <c r="V6" s="11"/>
-      <c r="W6" s="12"/>
-      <c r="X6" s="10" t="s">
+      <c r="T6" s="13"/>
+      <c r="U6" s="13"/>
+      <c r="V6" s="13"/>
+      <c r="W6" s="14"/>
+      <c r="X6" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="Y6" s="11"/>
-      <c r="Z6" s="11"/>
-      <c r="AA6" s="12"/>
-      <c r="AB6" s="10" t="s">
+      <c r="Y6" s="13"/>
+      <c r="Z6" s="13"/>
+      <c r="AA6" s="14"/>
+      <c r="AB6" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="AC6" s="11"/>
-      <c r="AD6" s="11"/>
-      <c r="AE6" s="11"/>
-      <c r="AF6" s="12"/>
+      <c r="AC6" s="13"/>
+      <c r="AD6" s="13"/>
+      <c r="AE6" s="13"/>
+      <c r="AF6" s="14"/>
       <c r="AG6" s="3" t="s">
         <v>16</v>
       </c>
@@ -975,45 +1102,45 @@
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
-      <c r="R7" s="12"/>
-      <c r="S7" s="10" t="s">
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="13"/>
+      <c r="Q7" s="13"/>
+      <c r="R7" s="14"/>
+      <c r="S7" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="T7" s="11"/>
-      <c r="U7" s="11"/>
-      <c r="V7" s="11"/>
-      <c r="W7" s="12"/>
-      <c r="X7" s="10" t="s">
+      <c r="T7" s="13"/>
+      <c r="U7" s="13"/>
+      <c r="V7" s="13"/>
+      <c r="W7" s="14"/>
+      <c r="X7" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="Y7" s="11"/>
-      <c r="Z7" s="11"/>
-      <c r="AA7" s="12"/>
-      <c r="AB7" s="10" t="s">
+      <c r="Y7" s="13"/>
+      <c r="Z7" s="13"/>
+      <c r="AA7" s="14"/>
+      <c r="AB7" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="AC7" s="11"/>
-      <c r="AD7" s="11"/>
-      <c r="AE7" s="11"/>
-      <c r="AF7" s="12"/>
+      <c r="AC7" s="13"/>
+      <c r="AD7" s="13"/>
+      <c r="AE7" s="13"/>
+      <c r="AF7" s="14"/>
       <c r="AG7" s="3" t="s">
         <v>16</v>
       </c>
@@ -1022,47 +1149,47 @@
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="11"/>
-      <c r="R8" s="11"/>
-      <c r="S8" s="11"/>
-      <c r="T8" s="11"/>
-      <c r="U8" s="12"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="13"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="13"/>
+      <c r="Q8" s="13"/>
+      <c r="R8" s="13"/>
+      <c r="S8" s="13"/>
+      <c r="T8" s="13"/>
+      <c r="U8" s="14"/>
       <c r="V8" s="3">
         <v>0</v>
       </c>
       <c r="W8" s="3">
         <v>0</v>
       </c>
-      <c r="X8" s="10" t="s">
+      <c r="X8" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="Y8" s="11"/>
-      <c r="Z8" s="11"/>
-      <c r="AA8" s="12"/>
-      <c r="AB8" s="10" t="s">
+      <c r="Y8" s="13"/>
+      <c r="Z8" s="13"/>
+      <c r="AA8" s="14"/>
+      <c r="AB8" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="AC8" s="11"/>
-      <c r="AD8" s="11"/>
-      <c r="AE8" s="11"/>
-      <c r="AF8" s="12"/>
+      <c r="AC8" s="13"/>
+      <c r="AD8" s="13"/>
+      <c r="AE8" s="13"/>
+      <c r="AF8" s="14"/>
       <c r="AG8" s="3" t="s">
         <v>16</v>
       </c>
@@ -1071,34 +1198,34 @@
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="12"/>
-      <c r="R9" s="10" t="s">
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13"/>
+      <c r="L9" s="13"/>
+      <c r="M9" s="13"/>
+      <c r="N9" s="13"/>
+      <c r="O9" s="13"/>
+      <c r="P9" s="13"/>
+      <c r="Q9" s="14"/>
+      <c r="R9" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="S9" s="11"/>
-      <c r="T9" s="12"/>
-      <c r="U9" s="10" t="s">
+      <c r="S9" s="13"/>
+      <c r="T9" s="14"/>
+      <c r="U9" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="V9" s="11"/>
-      <c r="W9" s="12"/>
+      <c r="V9" s="13"/>
+      <c r="W9" s="14"/>
       <c r="X9" s="3" t="s">
         <v>19</v>
       </c>
@@ -1111,13 +1238,13 @@
       <c r="AA9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AB9" s="10" t="s">
+      <c r="AB9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="AC9" s="11"/>
-      <c r="AD9" s="11"/>
-      <c r="AE9" s="11"/>
-      <c r="AF9" s="12"/>
+      <c r="AC9" s="13"/>
+      <c r="AD9" s="13"/>
+      <c r="AE9" s="13"/>
+      <c r="AF9" s="14"/>
       <c r="AG9" s="3" t="s">
         <v>16</v>
       </c>
@@ -1126,53 +1253,53 @@
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="10" t="s">
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="J10" s="11"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="10" t="s">
+      <c r="J10" s="13"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="M10" s="11"/>
-      <c r="N10" s="12"/>
-      <c r="O10" s="10" t="s">
+      <c r="M10" s="13"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="12"/>
-      <c r="R10" s="10" t="s">
+      <c r="P10" s="13"/>
+      <c r="Q10" s="14"/>
+      <c r="R10" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="S10" s="11"/>
-      <c r="T10" s="12"/>
-      <c r="U10" s="10" t="s">
+      <c r="S10" s="13"/>
+      <c r="T10" s="14"/>
+      <c r="U10" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="V10" s="11"/>
-      <c r="W10" s="12"/>
-      <c r="X10" s="10" t="s">
+      <c r="V10" s="13"/>
+      <c r="W10" s="14"/>
+      <c r="X10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="Y10" s="11"/>
-      <c r="Z10" s="11"/>
-      <c r="AA10" s="12"/>
-      <c r="AB10" s="10" t="s">
+      <c r="Y10" s="13"/>
+      <c r="Z10" s="13"/>
+      <c r="AA10" s="14"/>
+      <c r="AB10" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="AC10" s="11"/>
-      <c r="AD10" s="11"/>
-      <c r="AE10" s="11"/>
-      <c r="AF10" s="12"/>
+      <c r="AC10" s="13"/>
+      <c r="AD10" s="13"/>
+      <c r="AE10" s="13"/>
+      <c r="AF10" s="14"/>
       <c r="AG10" s="3" t="s">
         <v>16</v>
       </c>
@@ -1181,53 +1308,53 @@
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="12"/>
-      <c r="R11" s="10" t="s">
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="13"/>
+      <c r="O11" s="13"/>
+      <c r="P11" s="13"/>
+      <c r="Q11" s="14"/>
+      <c r="R11" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="S11" s="11"/>
-      <c r="T11" s="12"/>
-      <c r="U11" s="10" t="s">
+      <c r="S11" s="13"/>
+      <c r="T11" s="14"/>
+      <c r="U11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="V11" s="11"/>
-      <c r="W11" s="12"/>
-      <c r="X11" s="10" t="s">
+      <c r="V11" s="13"/>
+      <c r="W11" s="14"/>
+      <c r="X11" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="Y11" s="11"/>
-      <c r="Z11" s="11"/>
-      <c r="AA11" s="12"/>
-      <c r="AB11" s="10" t="s">
+      <c r="Y11" s="13"/>
+      <c r="Z11" s="13"/>
+      <c r="AA11" s="14"/>
+      <c r="AB11" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="AC11" s="11"/>
-      <c r="AD11" s="11"/>
-      <c r="AE11" s="11"/>
-      <c r="AF11" s="12"/>
+      <c r="AC11" s="13"/>
+      <c r="AD11" s="13"/>
+      <c r="AE11" s="13"/>
+      <c r="AF11" s="14"/>
       <c r="AG11" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="3">
@@ -1266,71 +1393,123 @@
       <c r="M12" s="3">
         <v>0</v>
       </c>
-      <c r="N12" s="10" t="s">
+      <c r="N12" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="11"/>
-      <c r="R12" s="12"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="13"/>
+      <c r="Q12" s="13"/>
+      <c r="R12" s="14"/>
       <c r="S12" s="3">
         <v>0</v>
       </c>
       <c r="T12" s="3">
         <v>0</v>
       </c>
-      <c r="U12" s="10" t="s">
+      <c r="U12" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="V12" s="11"/>
-      <c r="W12" s="12"/>
-      <c r="X12" s="10" t="s">
+      <c r="V12" s="13"/>
+      <c r="W12" s="14"/>
+      <c r="X12" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="Y12" s="11"/>
-      <c r="Z12" s="11"/>
-      <c r="AA12" s="12"/>
-      <c r="AB12" s="10" t="s">
+      <c r="Y12" s="17"/>
+      <c r="Z12" s="17"/>
+      <c r="AA12" s="18"/>
+      <c r="AB12" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="AC12" s="11"/>
-      <c r="AD12" s="11"/>
-      <c r="AE12" s="11"/>
-      <c r="AF12" s="12"/>
-      <c r="AG12" s="3" t="s">
+      <c r="AC12" s="17"/>
+      <c r="AD12" s="17"/>
+      <c r="AE12" s="17"/>
+      <c r="AF12" s="18"/>
+      <c r="AG12" s="22" t="s">
         <v>16</v>
       </c>
+    </row>
+    <row r="13" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A13" s="15"/>
+      <c r="B13" s="3">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3">
+        <v>0</v>
+      </c>
+      <c r="F13" s="3">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3">
+        <v>0</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3">
+        <v>0</v>
+      </c>
+      <c r="L13" s="3">
+        <v>0</v>
+      </c>
+      <c r="M13" s="3">
+        <v>0</v>
+      </c>
+      <c r="N13" s="3">
+        <v>0</v>
+      </c>
+      <c r="O13" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="P13" s="13"/>
+      <c r="Q13" s="14"/>
+      <c r="R13" s="9">
+        <v>0</v>
+      </c>
+      <c r="S13" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="T13" s="13"/>
+      <c r="U13" s="13"/>
+      <c r="V13" s="13"/>
+      <c r="W13" s="14"/>
+      <c r="X13" s="19"/>
+      <c r="Y13" s="20"/>
+      <c r="Z13" s="20"/>
+      <c r="AA13" s="21"/>
+      <c r="AB13" s="19"/>
+      <c r="AC13" s="20"/>
+      <c r="AD13" s="20"/>
+      <c r="AE13" s="20"/>
+      <c r="AF13" s="21"/>
+      <c r="AG13" s="23"/>
     </row>
   </sheetData>
-  <mergeCells count="49">
-    <mergeCell ref="AB3:AF3"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="N3:R3"/>
-    <mergeCell ref="S3:W3"/>
-    <mergeCell ref="X3:AA3"/>
-    <mergeCell ref="AB4:AF4"/>
-    <mergeCell ref="B5:M5"/>
-    <mergeCell ref="N5:R5"/>
-    <mergeCell ref="S5:W5"/>
-    <mergeCell ref="AB5:AF5"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B4:M4"/>
-    <mergeCell ref="N4:R4"/>
-    <mergeCell ref="S4:W4"/>
-    <mergeCell ref="X4:AA4"/>
-    <mergeCell ref="AB6:AF6"/>
-    <mergeCell ref="X6:AA6"/>
-    <mergeCell ref="I6:M6"/>
-    <mergeCell ref="N6:R6"/>
-    <mergeCell ref="S6:W6"/>
-    <mergeCell ref="AB7:AF7"/>
-    <mergeCell ref="X7:AA7"/>
-    <mergeCell ref="S7:W7"/>
-    <mergeCell ref="B7:R7"/>
-    <mergeCell ref="X8:AA8"/>
-    <mergeCell ref="AB8:AF8"/>
-    <mergeCell ref="B8:U8"/>
+  <mergeCells count="53">
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="X12:AA13"/>
+    <mergeCell ref="AB12:AF13"/>
+    <mergeCell ref="AG12:AG13"/>
+    <mergeCell ref="S13:W13"/>
+    <mergeCell ref="O13:Q13"/>
+    <mergeCell ref="B11:Q11"/>
+    <mergeCell ref="U12:W12"/>
+    <mergeCell ref="N12:R12"/>
+    <mergeCell ref="R11:T11"/>
+    <mergeCell ref="U11:W11"/>
+    <mergeCell ref="X11:AA11"/>
+    <mergeCell ref="AB11:AF11"/>
     <mergeCell ref="AB9:AF9"/>
     <mergeCell ref="U9:W9"/>
     <mergeCell ref="R9:T9"/>
@@ -1342,16 +1521,35 @@
     <mergeCell ref="O10:Q10"/>
     <mergeCell ref="I10:K10"/>
     <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B11:Q11"/>
-    <mergeCell ref="AB12:AF12"/>
-    <mergeCell ref="X12:AA12"/>
-    <mergeCell ref="U12:W12"/>
-    <mergeCell ref="N12:R12"/>
-    <mergeCell ref="R11:T11"/>
-    <mergeCell ref="U11:W11"/>
-    <mergeCell ref="X11:AA11"/>
-    <mergeCell ref="AB11:AF11"/>
     <mergeCell ref="L10:N10"/>
+    <mergeCell ref="AB7:AF7"/>
+    <mergeCell ref="X7:AA7"/>
+    <mergeCell ref="S7:W7"/>
+    <mergeCell ref="B7:R7"/>
+    <mergeCell ref="X8:AA8"/>
+    <mergeCell ref="AB8:AF8"/>
+    <mergeCell ref="B8:U8"/>
+    <mergeCell ref="AB6:AF6"/>
+    <mergeCell ref="X6:AA6"/>
+    <mergeCell ref="I6:M6"/>
+    <mergeCell ref="N6:R6"/>
+    <mergeCell ref="S6:W6"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="N4:R4"/>
+    <mergeCell ref="S4:W4"/>
+    <mergeCell ref="X4:AA4"/>
+    <mergeCell ref="AB4:AF4"/>
+    <mergeCell ref="B5:M5"/>
+    <mergeCell ref="N5:R5"/>
+    <mergeCell ref="S5:W5"/>
+    <mergeCell ref="AB5:AF5"/>
+    <mergeCell ref="AB3:AF3"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="N3:R3"/>
+    <mergeCell ref="S3:W3"/>
+    <mergeCell ref="X3:AA3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1362,7 +1560,7 @@
   <dimension ref="A2:AM8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="13"/>
+    <col min="1" max="1" width="8.88671875" style="10"/>
     <col min="2" max="2" width="19.44140625" customWidth="1"/>
     <col min="3" max="34" width="3.44140625" customWidth="1"/>
     <col min="35" max="38" width="4.21875" customWidth="1"/>
@@ -1466,18 +1664,18 @@
       <c r="AH2" s="5">
         <v>0</v>
       </c>
-      <c r="AI2" s="9" t="s">
+      <c r="AI2" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="AJ2" s="9"/>
-      <c r="AK2" s="9"/>
-      <c r="AL2" s="9"/>
+      <c r="AJ2" s="11"/>
+      <c r="AK2" s="11"/>
+      <c r="AL2" s="11"/>
       <c r="AM2" s="4" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:39" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="10" t="s">
         <v>35</v>
       </c>
       <c r="B3" s="2" t="s">

</xml_diff>

<commit_message>
feat(sv): unidad de extension de inmediatos + testbench
</commit_message>
<xml_diff>
--- a/res/isa.xlsx
+++ b/res/isa.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frede\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\workbench\repos\CE4301--p2_fobando_isa--\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F5D958B-2496-4DC8-9A20-AA8D0B55C417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{120388A2-2551-4D62-8CAE-7210F7BC860E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{EC7525CD-E51C-4E61-B306-9CBCE090E85A}"/>
   </bookViews>
@@ -441,7 +441,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -473,6 +473,27 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -498,36 +519,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -978,49 +969,49 @@
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="20" t="s">
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="20" t="s">
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="17"/>
+      <c r="N3" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="O3" s="21"/>
-      <c r="P3" s="21"/>
-      <c r="Q3" s="21"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="20" t="s">
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="17"/>
+      <c r="S3" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="T3" s="21"/>
-      <c r="U3" s="21"/>
-      <c r="V3" s="21"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="20" t="s">
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
+      <c r="V3" s="16"/>
+      <c r="W3" s="17"/>
+      <c r="X3" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="Y3" s="21"/>
-      <c r="Z3" s="21"/>
-      <c r="AA3" s="22"/>
-      <c r="AB3" s="20" t="s">
+      <c r="Y3" s="16"/>
+      <c r="Z3" s="16"/>
+      <c r="AA3" s="17"/>
+      <c r="AB3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC3" s="21"/>
-      <c r="AD3" s="21"/>
-      <c r="AE3" s="21"/>
-      <c r="AF3" s="22"/>
+      <c r="AC3" s="16"/>
+      <c r="AD3" s="16"/>
+      <c r="AE3" s="16"/>
+      <c r="AF3" s="17"/>
       <c r="AG3" s="3" t="s">
         <v>16</v>
       </c>
@@ -1029,47 +1020,47 @@
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="20" t="s">
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="17"/>
+      <c r="N4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="O4" s="21"/>
-      <c r="P4" s="21"/>
-      <c r="Q4" s="21"/>
-      <c r="R4" s="22"/>
-      <c r="S4" s="20" t="s">
+      <c r="O4" s="16"/>
+      <c r="P4" s="16"/>
+      <c r="Q4" s="16"/>
+      <c r="R4" s="17"/>
+      <c r="S4" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="T4" s="21"/>
-      <c r="U4" s="21"/>
-      <c r="V4" s="21"/>
-      <c r="W4" s="22"/>
-      <c r="X4" s="20" t="s">
+      <c r="T4" s="16"/>
+      <c r="U4" s="16"/>
+      <c r="V4" s="16"/>
+      <c r="W4" s="17"/>
+      <c r="X4" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="Y4" s="21"/>
-      <c r="Z4" s="21"/>
-      <c r="AA4" s="22"/>
-      <c r="AB4" s="20" t="s">
+      <c r="Y4" s="16"/>
+      <c r="Z4" s="16"/>
+      <c r="AA4" s="17"/>
+      <c r="AB4" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC4" s="21"/>
-      <c r="AD4" s="21"/>
-      <c r="AE4" s="21"/>
-      <c r="AF4" s="22"/>
+      <c r="AC4" s="16"/>
+      <c r="AD4" s="16"/>
+      <c r="AE4" s="16"/>
+      <c r="AF4" s="17"/>
       <c r="AG4" s="3" t="s">
         <v>16</v>
       </c>
@@ -1078,34 +1069,34 @@
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
-      <c r="H5" s="21"/>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="20" t="s">
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="17"/>
+      <c r="N5" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="O5" s="21"/>
-      <c r="P5" s="21"/>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="20" t="s">
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
+      <c r="Q5" s="16"/>
+      <c r="R5" s="17"/>
+      <c r="S5" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="T5" s="21"/>
-      <c r="U5" s="21"/>
-      <c r="V5" s="21"/>
-      <c r="W5" s="22"/>
+      <c r="T5" s="16"/>
+      <c r="U5" s="16"/>
+      <c r="V5" s="16"/>
+      <c r="W5" s="17"/>
       <c r="X5" s="3" t="s">
         <v>19</v>
       </c>
@@ -1118,13 +1109,13 @@
       <c r="AA5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AB5" s="20" t="s">
+      <c r="AB5" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC5" s="21"/>
-      <c r="AD5" s="21"/>
-      <c r="AE5" s="21"/>
-      <c r="AF5" s="22"/>
+      <c r="AC5" s="16"/>
+      <c r="AD5" s="16"/>
+      <c r="AE5" s="16"/>
+      <c r="AF5" s="17"/>
       <c r="AG5" s="3" t="s">
         <v>16</v>
       </c>
@@ -1133,49 +1124,49 @@
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="20" t="s">
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="20" t="s">
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="O6" s="21"/>
-      <c r="P6" s="21"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="22"/>
-      <c r="S6" s="20" t="s">
+      <c r="O6" s="16"/>
+      <c r="P6" s="16"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="T6" s="21"/>
-      <c r="U6" s="21"/>
-      <c r="V6" s="21"/>
-      <c r="W6" s="22"/>
-      <c r="X6" s="20" t="s">
+      <c r="T6" s="16"/>
+      <c r="U6" s="16"/>
+      <c r="V6" s="16"/>
+      <c r="W6" s="17"/>
+      <c r="X6" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="Y6" s="21"/>
-      <c r="Z6" s="21"/>
-      <c r="AA6" s="22"/>
-      <c r="AB6" s="20" t="s">
+      <c r="Y6" s="16"/>
+      <c r="Z6" s="16"/>
+      <c r="AA6" s="17"/>
+      <c r="AB6" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC6" s="21"/>
-      <c r="AD6" s="21"/>
-      <c r="AE6" s="21"/>
-      <c r="AF6" s="22"/>
+      <c r="AC6" s="16"/>
+      <c r="AD6" s="16"/>
+      <c r="AE6" s="16"/>
+      <c r="AF6" s="17"/>
       <c r="AG6" s="3" t="s">
         <v>16</v>
       </c>
@@ -1184,45 +1175,45 @@
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="22"/>
-      <c r="S7" s="20" t="s">
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="17"/>
+      <c r="S7" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="T7" s="21"/>
-      <c r="U7" s="21"/>
-      <c r="V7" s="21"/>
-      <c r="W7" s="22"/>
-      <c r="X7" s="20" t="s">
+      <c r="T7" s="16"/>
+      <c r="U7" s="16"/>
+      <c r="V7" s="16"/>
+      <c r="W7" s="17"/>
+      <c r="X7" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="Y7" s="21"/>
-      <c r="Z7" s="21"/>
-      <c r="AA7" s="22"/>
-      <c r="AB7" s="20" t="s">
+      <c r="Y7" s="16"/>
+      <c r="Z7" s="16"/>
+      <c r="AA7" s="17"/>
+      <c r="AB7" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC7" s="21"/>
-      <c r="AD7" s="21"/>
-      <c r="AE7" s="21"/>
-      <c r="AF7" s="22"/>
+      <c r="AC7" s="16"/>
+      <c r="AD7" s="16"/>
+      <c r="AE7" s="16"/>
+      <c r="AF7" s="17"/>
       <c r="AG7" s="3" t="s">
         <v>16</v>
       </c>
@@ -1231,47 +1222,47 @@
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="21"/>
-      <c r="J8" s="21"/>
-      <c r="K8" s="21"/>
-      <c r="L8" s="21"/>
-      <c r="M8" s="21"/>
-      <c r="N8" s="21"/>
-      <c r="O8" s="21"/>
-      <c r="P8" s="21"/>
-      <c r="Q8" s="21"/>
-      <c r="R8" s="21"/>
-      <c r="S8" s="21"/>
-      <c r="T8" s="21"/>
-      <c r="U8" s="22"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="16"/>
+      <c r="P8" s="16"/>
+      <c r="Q8" s="16"/>
+      <c r="R8" s="16"/>
+      <c r="S8" s="16"/>
+      <c r="T8" s="16"/>
+      <c r="U8" s="17"/>
       <c r="V8" s="3">
         <v>0</v>
       </c>
       <c r="W8" s="3">
         <v>0</v>
       </c>
-      <c r="X8" s="20" t="s">
+      <c r="X8" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="Y8" s="21"/>
-      <c r="Z8" s="21"/>
-      <c r="AA8" s="22"/>
-      <c r="AB8" s="20" t="s">
+      <c r="Y8" s="16"/>
+      <c r="Z8" s="16"/>
+      <c r="AA8" s="17"/>
+      <c r="AB8" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC8" s="21"/>
-      <c r="AD8" s="21"/>
-      <c r="AE8" s="21"/>
-      <c r="AF8" s="22"/>
+      <c r="AC8" s="16"/>
+      <c r="AD8" s="16"/>
+      <c r="AE8" s="16"/>
+      <c r="AF8" s="17"/>
       <c r="AG8" s="3" t="s">
         <v>16</v>
       </c>
@@ -1280,34 +1271,34 @@
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21"/>
-      <c r="I9" s="21"/>
-      <c r="J9" s="21"/>
-      <c r="K9" s="21"/>
-      <c r="L9" s="21"/>
-      <c r="M9" s="21"/>
-      <c r="N9" s="21"/>
-      <c r="O9" s="21"/>
-      <c r="P9" s="21"/>
-      <c r="Q9" s="22"/>
-      <c r="R9" s="20" t="s">
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="S9" s="21"/>
-      <c r="T9" s="22"/>
-      <c r="U9" s="20" t="s">
+      <c r="S9" s="16"/>
+      <c r="T9" s="17"/>
+      <c r="U9" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="V9" s="21"/>
-      <c r="W9" s="22"/>
+      <c r="V9" s="16"/>
+      <c r="W9" s="17"/>
       <c r="X9" s="3" t="s">
         <v>19</v>
       </c>
@@ -1320,13 +1311,13 @@
       <c r="AA9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AB9" s="20" t="s">
+      <c r="AB9" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC9" s="21"/>
-      <c r="AD9" s="21"/>
-      <c r="AE9" s="21"/>
-      <c r="AF9" s="22"/>
+      <c r="AC9" s="16"/>
+      <c r="AD9" s="16"/>
+      <c r="AE9" s="16"/>
+      <c r="AF9" s="17"/>
       <c r="AG9" s="3" t="s">
         <v>16</v>
       </c>
@@ -1335,53 +1326,53 @@
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="20" t="s">
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="J10" s="21"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="20" t="s">
+      <c r="J10" s="16"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="M10" s="21"/>
-      <c r="N10" s="22"/>
-      <c r="O10" s="20" t="s">
+      <c r="M10" s="16"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="22"/>
-      <c r="R10" s="20" t="s">
+      <c r="P10" s="16"/>
+      <c r="Q10" s="17"/>
+      <c r="R10" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="S10" s="21"/>
-      <c r="T10" s="22"/>
-      <c r="U10" s="20" t="s">
+      <c r="S10" s="16"/>
+      <c r="T10" s="17"/>
+      <c r="U10" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="V10" s="21"/>
-      <c r="W10" s="22"/>
-      <c r="X10" s="20" t="s">
+      <c r="V10" s="16"/>
+      <c r="W10" s="17"/>
+      <c r="X10" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="Y10" s="21"/>
-      <c r="Z10" s="21"/>
-      <c r="AA10" s="22"/>
-      <c r="AB10" s="20" t="s">
+      <c r="Y10" s="16"/>
+      <c r="Z10" s="16"/>
+      <c r="AA10" s="17"/>
+      <c r="AB10" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC10" s="21"/>
-      <c r="AD10" s="21"/>
-      <c r="AE10" s="21"/>
-      <c r="AF10" s="22"/>
+      <c r="AC10" s="16"/>
+      <c r="AD10" s="16"/>
+      <c r="AE10" s="16"/>
+      <c r="AF10" s="17"/>
       <c r="AG10" s="3" t="s">
         <v>16</v>
       </c>
@@ -1390,53 +1381,53 @@
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="21"/>
-      <c r="L11" s="21"/>
-      <c r="M11" s="21"/>
-      <c r="N11" s="21"/>
-      <c r="O11" s="21"/>
-      <c r="P11" s="21"/>
-      <c r="Q11" s="22"/>
-      <c r="R11" s="20" t="s">
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="16"/>
+      <c r="N11" s="16"/>
+      <c r="O11" s="16"/>
+      <c r="P11" s="16"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="S11" s="21"/>
-      <c r="T11" s="22"/>
-      <c r="U11" s="20" t="s">
+      <c r="S11" s="16"/>
+      <c r="T11" s="17"/>
+      <c r="U11" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="V11" s="21"/>
-      <c r="W11" s="22"/>
-      <c r="X11" s="20" t="s">
+      <c r="V11" s="16"/>
+      <c r="W11" s="17"/>
+      <c r="X11" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="Y11" s="21"/>
-      <c r="Z11" s="21"/>
-      <c r="AA11" s="22"/>
-      <c r="AB11" s="20" t="s">
+      <c r="Y11" s="16"/>
+      <c r="Z11" s="16"/>
+      <c r="AA11" s="17"/>
+      <c r="AB11" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC11" s="21"/>
-      <c r="AD11" s="21"/>
-      <c r="AE11" s="21"/>
-      <c r="AF11" s="22"/>
+      <c r="AC11" s="16"/>
+      <c r="AD11" s="16"/>
+      <c r="AE11" s="16"/>
+      <c r="AF11" s="17"/>
       <c r="AG11" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="18" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="3">
@@ -1475,43 +1466,43 @@
       <c r="M12" s="3">
         <v>0</v>
       </c>
-      <c r="N12" s="20" t="s">
+      <c r="N12" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="O12" s="21"/>
-      <c r="P12" s="21"/>
-      <c r="Q12" s="21"/>
-      <c r="R12" s="22"/>
+      <c r="O12" s="16"/>
+      <c r="P12" s="16"/>
+      <c r="Q12" s="16"/>
+      <c r="R12" s="17"/>
       <c r="S12" s="3">
         <v>0</v>
       </c>
       <c r="T12" s="3">
         <v>0</v>
       </c>
-      <c r="U12" s="20" t="s">
+      <c r="U12" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="V12" s="21"/>
-      <c r="W12" s="22"/>
-      <c r="X12" s="12" t="s">
+      <c r="V12" s="16"/>
+      <c r="W12" s="17"/>
+      <c r="X12" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="Y12" s="13"/>
-      <c r="Z12" s="13"/>
-      <c r="AA12" s="14"/>
-      <c r="AB12" s="12" t="s">
+      <c r="Y12" s="20"/>
+      <c r="Z12" s="20"/>
+      <c r="AA12" s="21"/>
+      <c r="AB12" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="AC12" s="13"/>
-      <c r="AD12" s="13"/>
-      <c r="AE12" s="13"/>
-      <c r="AF12" s="14"/>
-      <c r="AG12" s="18" t="s">
+      <c r="AC12" s="20"/>
+      <c r="AD12" s="20"/>
+      <c r="AE12" s="20"/>
+      <c r="AF12" s="21"/>
+      <c r="AG12" s="25" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A13" s="11"/>
+      <c r="A13" s="18"/>
       <c r="B13" s="3">
         <v>0</v>
       </c>
@@ -1551,62 +1542,50 @@
       <c r="N13" s="3">
         <v>0</v>
       </c>
-      <c r="O13" s="20" t="s">
+      <c r="O13" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="P13" s="21"/>
-      <c r="Q13" s="22"/>
+      <c r="P13" s="16"/>
+      <c r="Q13" s="17"/>
       <c r="R13" s="9">
         <v>0</v>
       </c>
-      <c r="S13" s="20" t="s">
+      <c r="S13" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="T13" s="21"/>
-      <c r="U13" s="21"/>
-      <c r="V13" s="21"/>
-      <c r="W13" s="22"/>
-      <c r="X13" s="15"/>
-      <c r="Y13" s="16"/>
-      <c r="Z13" s="16"/>
-      <c r="AA13" s="17"/>
-      <c r="AB13" s="15"/>
-      <c r="AC13" s="16"/>
-      <c r="AD13" s="16"/>
-      <c r="AE13" s="16"/>
-      <c r="AF13" s="17"/>
-      <c r="AG13" s="19"/>
+      <c r="T13" s="16"/>
+      <c r="U13" s="16"/>
+      <c r="V13" s="16"/>
+      <c r="W13" s="17"/>
+      <c r="X13" s="22"/>
+      <c r="Y13" s="23"/>
+      <c r="Z13" s="23"/>
+      <c r="AA13" s="24"/>
+      <c r="AB13" s="22"/>
+      <c r="AC13" s="23"/>
+      <c r="AD13" s="23"/>
+      <c r="AE13" s="23"/>
+      <c r="AF13" s="24"/>
+      <c r="AG13" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="AB3:AF3"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="N3:R3"/>
-    <mergeCell ref="S3:W3"/>
-    <mergeCell ref="X3:AA3"/>
-    <mergeCell ref="AB4:AF4"/>
-    <mergeCell ref="B5:M5"/>
-    <mergeCell ref="N5:R5"/>
-    <mergeCell ref="S5:W5"/>
-    <mergeCell ref="AB5:AF5"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B4:M4"/>
-    <mergeCell ref="N4:R4"/>
-    <mergeCell ref="S4:W4"/>
-    <mergeCell ref="X4:AA4"/>
-    <mergeCell ref="AB6:AF6"/>
-    <mergeCell ref="X6:AA6"/>
-    <mergeCell ref="I6:M6"/>
-    <mergeCell ref="N6:R6"/>
-    <mergeCell ref="S6:W6"/>
-    <mergeCell ref="AB7:AF7"/>
-    <mergeCell ref="X7:AA7"/>
-    <mergeCell ref="S7:W7"/>
-    <mergeCell ref="B7:R7"/>
-    <mergeCell ref="X8:AA8"/>
-    <mergeCell ref="AB8:AF8"/>
-    <mergeCell ref="B8:U8"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="X12:AA13"/>
+    <mergeCell ref="AB12:AF13"/>
+    <mergeCell ref="AG12:AG13"/>
+    <mergeCell ref="S13:W13"/>
+    <mergeCell ref="O13:Q13"/>
+    <mergeCell ref="B11:Q11"/>
+    <mergeCell ref="U12:W12"/>
+    <mergeCell ref="N12:R12"/>
+    <mergeCell ref="R11:T11"/>
+    <mergeCell ref="U11:W11"/>
+    <mergeCell ref="X11:AA11"/>
+    <mergeCell ref="AB11:AF11"/>
+    <mergeCell ref="AB9:AF9"/>
+    <mergeCell ref="U9:W9"/>
+    <mergeCell ref="R9:T9"/>
     <mergeCell ref="B9:Q9"/>
     <mergeCell ref="X10:AA10"/>
     <mergeCell ref="AB10:AF10"/>
@@ -1616,22 +1595,34 @@
     <mergeCell ref="I10:K10"/>
     <mergeCell ref="B10:H10"/>
     <mergeCell ref="L10:N10"/>
-    <mergeCell ref="X11:AA11"/>
-    <mergeCell ref="AB11:AF11"/>
-    <mergeCell ref="AB9:AF9"/>
-    <mergeCell ref="U9:W9"/>
-    <mergeCell ref="R9:T9"/>
-    <mergeCell ref="B11:Q11"/>
-    <mergeCell ref="U12:W12"/>
-    <mergeCell ref="N12:R12"/>
-    <mergeCell ref="R11:T11"/>
-    <mergeCell ref="U11:W11"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="X12:AA13"/>
-    <mergeCell ref="AB12:AF13"/>
-    <mergeCell ref="AG12:AG13"/>
-    <mergeCell ref="S13:W13"/>
-    <mergeCell ref="O13:Q13"/>
+    <mergeCell ref="AB7:AF7"/>
+    <mergeCell ref="X7:AA7"/>
+    <mergeCell ref="S7:W7"/>
+    <mergeCell ref="B7:R7"/>
+    <mergeCell ref="X8:AA8"/>
+    <mergeCell ref="AB8:AF8"/>
+    <mergeCell ref="B8:U8"/>
+    <mergeCell ref="AB6:AF6"/>
+    <mergeCell ref="X6:AA6"/>
+    <mergeCell ref="I6:M6"/>
+    <mergeCell ref="N6:R6"/>
+    <mergeCell ref="S6:W6"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="N4:R4"/>
+    <mergeCell ref="S4:W4"/>
+    <mergeCell ref="X4:AA4"/>
+    <mergeCell ref="AB4:AF4"/>
+    <mergeCell ref="B5:M5"/>
+    <mergeCell ref="N5:R5"/>
+    <mergeCell ref="S5:W5"/>
+    <mergeCell ref="AB5:AF5"/>
+    <mergeCell ref="AB3:AF3"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="N3:R3"/>
+    <mergeCell ref="S3:W3"/>
+    <mergeCell ref="X3:AA3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1746,12 +1737,12 @@
       <c r="AH2" s="5">
         <v>0</v>
       </c>
-      <c r="AI2" s="23" t="s">
+      <c r="AI2" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="AJ2" s="23"/>
-      <c r="AK2" s="23"/>
-      <c r="AL2" s="23"/>
+      <c r="AJ2" s="14"/>
+      <c r="AK2" s="14"/>
+      <c r="AL2" s="14"/>
       <c r="AM2" s="4" t="s">
         <v>33</v>
       </c>
@@ -1763,100 +1754,100 @@
       <c r="B3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="24">
-        <v>0</v>
-      </c>
-      <c r="D3" s="24">
-        <v>0</v>
-      </c>
-      <c r="E3" s="24">
-        <v>0</v>
-      </c>
-      <c r="F3" s="24">
-        <v>0</v>
-      </c>
-      <c r="G3" s="24">
-        <v>0</v>
-      </c>
-      <c r="H3" s="24">
-        <v>0</v>
-      </c>
-      <c r="I3" s="24">
-        <v>0</v>
-      </c>
-      <c r="J3" s="25">
-        <v>0</v>
-      </c>
-      <c r="K3" s="25">
-        <v>0</v>
-      </c>
-      <c r="L3" s="25">
-        <v>0</v>
-      </c>
-      <c r="M3" s="25">
-        <v>0</v>
-      </c>
-      <c r="N3" s="25">
-        <v>0</v>
-      </c>
-      <c r="O3" s="24">
-        <v>0</v>
-      </c>
-      <c r="P3" s="24">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="24">
-        <v>0</v>
-      </c>
-      <c r="R3" s="24">
-        <v>0</v>
-      </c>
-      <c r="S3" s="24">
-        <v>0</v>
-      </c>
-      <c r="T3" s="25">
-        <v>0</v>
-      </c>
-      <c r="U3" s="25">
-        <v>0</v>
-      </c>
-      <c r="V3" s="25">
-        <v>0</v>
-      </c>
-      <c r="W3" s="25">
-        <v>0</v>
-      </c>
-      <c r="X3" s="25">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z3" s="24">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="24">
-        <v>1</v>
-      </c>
-      <c r="AB3" s="24">
-        <v>0</v>
-      </c>
-      <c r="AC3" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD3" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE3" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF3" s="25">
-        <v>0</v>
-      </c>
-      <c r="AG3" s="25">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="24">
+      <c r="C3" s="11">
+        <v>0</v>
+      </c>
+      <c r="D3" s="11">
+        <v>0</v>
+      </c>
+      <c r="E3" s="11">
+        <v>0</v>
+      </c>
+      <c r="F3" s="11">
+        <v>0</v>
+      </c>
+      <c r="G3" s="11">
+        <v>0</v>
+      </c>
+      <c r="H3" s="11">
+        <v>0</v>
+      </c>
+      <c r="I3" s="11">
+        <v>0</v>
+      </c>
+      <c r="J3" s="12">
+        <v>0</v>
+      </c>
+      <c r="K3" s="12">
+        <v>0</v>
+      </c>
+      <c r="L3" s="12">
+        <v>0</v>
+      </c>
+      <c r="M3" s="12">
+        <v>0</v>
+      </c>
+      <c r="N3" s="12">
+        <v>0</v>
+      </c>
+      <c r="O3" s="11">
+        <v>0</v>
+      </c>
+      <c r="P3" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="11">
+        <v>0</v>
+      </c>
+      <c r="R3" s="11">
+        <v>0</v>
+      </c>
+      <c r="S3" s="11">
+        <v>0</v>
+      </c>
+      <c r="T3" s="12">
+        <v>0</v>
+      </c>
+      <c r="U3" s="12">
+        <v>0</v>
+      </c>
+      <c r="V3" s="12">
+        <v>0</v>
+      </c>
+      <c r="W3" s="12">
+        <v>0</v>
+      </c>
+      <c r="X3" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB3" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="11">
         <v>0</v>
       </c>
       <c r="AI3" s="8" t="str">
@@ -1884,100 +1875,100 @@
       <c r="B4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="24">
-        <v>0</v>
-      </c>
-      <c r="D4" s="24">
-        <v>0</v>
-      </c>
-      <c r="E4" s="24">
-        <v>0</v>
-      </c>
-      <c r="F4" s="24">
-        <v>0</v>
-      </c>
-      <c r="G4" s="24">
-        <v>0</v>
-      </c>
-      <c r="H4" s="24">
-        <v>0</v>
-      </c>
-      <c r="I4" s="24">
-        <v>0</v>
-      </c>
-      <c r="J4" s="25">
-        <v>1</v>
-      </c>
-      <c r="K4" s="25">
-        <v>0</v>
-      </c>
-      <c r="L4" s="25">
-        <v>0</v>
-      </c>
-      <c r="M4" s="25">
-        <v>0</v>
-      </c>
-      <c r="N4" s="25">
-        <v>1</v>
-      </c>
-      <c r="O4" s="24">
-        <v>1</v>
-      </c>
-      <c r="P4" s="24">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="24">
-        <v>0</v>
-      </c>
-      <c r="R4" s="24">
-        <v>0</v>
-      </c>
-      <c r="S4" s="24">
-        <v>0</v>
-      </c>
-      <c r="T4" s="25">
-        <v>0</v>
-      </c>
-      <c r="U4" s="25">
-        <v>0</v>
-      </c>
-      <c r="V4" s="25">
-        <v>1</v>
-      </c>
-      <c r="W4" s="25">
-        <v>0</v>
-      </c>
-      <c r="X4" s="25">
-        <v>1</v>
-      </c>
-      <c r="Y4" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="24">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="24">
-        <v>1</v>
-      </c>
-      <c r="AB4" s="24">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF4" s="25">
-        <v>0</v>
-      </c>
-      <c r="AG4" s="25">
-        <v>0</v>
-      </c>
-      <c r="AH4" s="24">
+      <c r="C4" s="11">
+        <v>0</v>
+      </c>
+      <c r="D4" s="11">
+        <v>0</v>
+      </c>
+      <c r="E4" s="11">
+        <v>0</v>
+      </c>
+      <c r="F4" s="11">
+        <v>0</v>
+      </c>
+      <c r="G4" s="11">
+        <v>0</v>
+      </c>
+      <c r="H4" s="11">
+        <v>0</v>
+      </c>
+      <c r="I4" s="11">
+        <v>0</v>
+      </c>
+      <c r="J4" s="12">
+        <v>1</v>
+      </c>
+      <c r="K4" s="12">
+        <v>0</v>
+      </c>
+      <c r="L4" s="12">
+        <v>0</v>
+      </c>
+      <c r="M4" s="12">
+        <v>0</v>
+      </c>
+      <c r="N4" s="12">
+        <v>1</v>
+      </c>
+      <c r="O4" s="11">
+        <v>1</v>
+      </c>
+      <c r="P4" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="11">
+        <v>0</v>
+      </c>
+      <c r="R4" s="11">
+        <v>0</v>
+      </c>
+      <c r="S4" s="11">
+        <v>0</v>
+      </c>
+      <c r="T4" s="12">
+        <v>0</v>
+      </c>
+      <c r="U4" s="12">
+        <v>0</v>
+      </c>
+      <c r="V4" s="12">
+        <v>1</v>
+      </c>
+      <c r="W4" s="12">
+        <v>0</v>
+      </c>
+      <c r="X4" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y4" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB4" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="11">
         <v>0</v>
       </c>
       <c r="AI4" s="8" t="str">
@@ -2005,100 +1996,100 @@
       <c r="B5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="26">
-        <v>0</v>
-      </c>
-      <c r="D5" s="26">
-        <v>0</v>
-      </c>
-      <c r="E5" s="26">
-        <v>0</v>
-      </c>
-      <c r="F5" s="26">
-        <v>0</v>
-      </c>
-      <c r="G5" s="26">
-        <v>0</v>
-      </c>
-      <c r="H5" s="26">
-        <v>0</v>
-      </c>
-      <c r="I5" s="26">
-        <v>0</v>
-      </c>
-      <c r="J5" s="26">
-        <v>0</v>
-      </c>
-      <c r="K5" s="26">
-        <v>0</v>
-      </c>
-      <c r="L5" s="26">
-        <v>1</v>
-      </c>
-      <c r="M5" s="26">
-        <v>1</v>
-      </c>
-      <c r="N5" s="26">
-        <v>1</v>
-      </c>
-      <c r="O5" s="24">
-        <v>0</v>
-      </c>
-      <c r="P5" s="24">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="24">
-        <v>0</v>
-      </c>
-      <c r="R5" s="24">
-        <v>0</v>
-      </c>
-      <c r="S5" s="24">
-        <v>1</v>
-      </c>
-      <c r="T5" s="25">
-        <v>0</v>
-      </c>
-      <c r="U5" s="25">
-        <v>0</v>
-      </c>
-      <c r="V5" s="25">
-        <v>0</v>
-      </c>
-      <c r="W5" s="25">
-        <v>1</v>
-      </c>
-      <c r="X5" s="25">
-        <v>1</v>
-      </c>
-      <c r="Y5" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="24">
-        <v>1</v>
-      </c>
-      <c r="AA5" s="24">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="24">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD5" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE5" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF5" s="25">
-        <v>0</v>
-      </c>
-      <c r="AG5" s="25">
-        <v>1</v>
-      </c>
-      <c r="AH5" s="24">
+      <c r="C5" s="13">
+        <v>0</v>
+      </c>
+      <c r="D5" s="13">
+        <v>0</v>
+      </c>
+      <c r="E5" s="13">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13">
+        <v>0</v>
+      </c>
+      <c r="G5" s="13">
+        <v>0</v>
+      </c>
+      <c r="H5" s="13">
+        <v>0</v>
+      </c>
+      <c r="I5" s="13">
+        <v>0</v>
+      </c>
+      <c r="J5" s="13">
+        <v>0</v>
+      </c>
+      <c r="K5" s="13">
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <v>1</v>
+      </c>
+      <c r="M5" s="13">
+        <v>1</v>
+      </c>
+      <c r="N5" s="13">
+        <v>1</v>
+      </c>
+      <c r="O5" s="11">
+        <v>0</v>
+      </c>
+      <c r="P5" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="11">
+        <v>0</v>
+      </c>
+      <c r="R5" s="11">
+        <v>0</v>
+      </c>
+      <c r="S5" s="11">
+        <v>1</v>
+      </c>
+      <c r="T5" s="12">
+        <v>0</v>
+      </c>
+      <c r="U5" s="12">
+        <v>0</v>
+      </c>
+      <c r="V5" s="12">
+        <v>0</v>
+      </c>
+      <c r="W5" s="12">
+        <v>1</v>
+      </c>
+      <c r="X5" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="11">
+        <v>1</v>
+      </c>
+      <c r="AA5" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH5" s="11">
         <v>1</v>
       </c>
       <c r="AI5" s="8" t="str">
@@ -2118,7 +2109,7 @@
         <v>03</v>
       </c>
       <c r="AM5" t="str">
-        <f t="shared" ref="AM4:AM8" si="4">_xlfn.CONCAT("0x",AI5:AL5)</f>
+        <f t="shared" ref="AM5:AM8" si="4">_xlfn.CONCAT("0x",AI5:AL5)</f>
         <v>0x00708D03</v>
       </c>
     </row>
@@ -2126,100 +2117,100 @@
       <c r="B6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="26">
-        <v>1</v>
-      </c>
-      <c r="D6" s="26">
-        <v>1</v>
-      </c>
-      <c r="E6" s="26">
-        <v>1</v>
-      </c>
-      <c r="F6" s="26">
-        <v>1</v>
-      </c>
-      <c r="G6" s="26">
-        <v>1</v>
-      </c>
-      <c r="H6" s="26">
-        <v>1</v>
-      </c>
-      <c r="I6" s="26">
-        <v>1</v>
-      </c>
-      <c r="J6" s="25">
-        <v>1</v>
-      </c>
-      <c r="K6" s="25">
-        <v>0</v>
-      </c>
-      <c r="L6" s="25">
-        <v>1</v>
-      </c>
-      <c r="M6" s="25">
-        <v>0</v>
-      </c>
-      <c r="N6" s="25">
-        <v>1</v>
-      </c>
-      <c r="O6" s="24">
-        <v>1</v>
-      </c>
-      <c r="P6" s="24">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="24">
-        <v>0</v>
-      </c>
-      <c r="R6" s="24">
-        <v>1</v>
-      </c>
-      <c r="S6" s="24">
-        <v>1</v>
-      </c>
-      <c r="T6" s="27">
-        <v>1</v>
-      </c>
-      <c r="U6" s="26">
-        <v>1</v>
-      </c>
-      <c r="V6" s="26">
-        <v>1</v>
-      </c>
-      <c r="W6" s="26">
-        <v>0</v>
-      </c>
-      <c r="X6" s="26">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="24">
-        <v>1</v>
-      </c>
-      <c r="AA6" s="24">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="24">
-        <v>0</v>
-      </c>
-      <c r="AC6" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD6" s="25">
-        <v>1</v>
-      </c>
-      <c r="AE6" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF6" s="25">
-        <v>0</v>
-      </c>
-      <c r="AG6" s="25">
-        <v>0</v>
-      </c>
-      <c r="AH6" s="24">
+      <c r="C6" s="13">
+        <v>1</v>
+      </c>
+      <c r="D6" s="13">
+        <v>1</v>
+      </c>
+      <c r="E6" s="13">
+        <v>1</v>
+      </c>
+      <c r="F6" s="13">
+        <v>1</v>
+      </c>
+      <c r="G6" s="13">
+        <v>1</v>
+      </c>
+      <c r="H6" s="13">
+        <v>1</v>
+      </c>
+      <c r="I6" s="13">
+        <v>1</v>
+      </c>
+      <c r="J6" s="12">
+        <v>1</v>
+      </c>
+      <c r="K6" s="12">
+        <v>0</v>
+      </c>
+      <c r="L6" s="12">
+        <v>1</v>
+      </c>
+      <c r="M6" s="12">
+        <v>0</v>
+      </c>
+      <c r="N6" s="12">
+        <v>1</v>
+      </c>
+      <c r="O6" s="11">
+        <v>1</v>
+      </c>
+      <c r="P6" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="11">
+        <v>0</v>
+      </c>
+      <c r="R6" s="11">
+        <v>1</v>
+      </c>
+      <c r="S6" s="11">
+        <v>1</v>
+      </c>
+      <c r="T6" s="13">
+        <v>1</v>
+      </c>
+      <c r="U6" s="13">
+        <v>1</v>
+      </c>
+      <c r="V6" s="13">
+        <v>1</v>
+      </c>
+      <c r="W6" s="13">
+        <v>0</v>
+      </c>
+      <c r="X6" s="13">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="11">
+        <v>1</v>
+      </c>
+      <c r="AA6" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="12">
+        <v>1</v>
+      </c>
+      <c r="AE6" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="11">
         <v>0</v>
       </c>
       <c r="AI6" s="8" t="str">
@@ -2247,100 +2238,100 @@
       <c r="B7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="26">
-        <v>0</v>
-      </c>
-      <c r="D7" s="26">
-        <v>0</v>
-      </c>
-      <c r="E7" s="26">
-        <v>0</v>
-      </c>
-      <c r="F7" s="26">
-        <v>0</v>
-      </c>
-      <c r="G7" s="26">
-        <v>0</v>
-      </c>
-      <c r="H7" s="26">
-        <v>0</v>
-      </c>
-      <c r="I7" s="26">
-        <v>0</v>
-      </c>
-      <c r="J7" s="26">
-        <v>0</v>
-      </c>
-      <c r="K7" s="26">
-        <v>0</v>
-      </c>
-      <c r="L7" s="26">
-        <v>0</v>
-      </c>
-      <c r="M7" s="26">
-        <v>1</v>
-      </c>
-      <c r="N7" s="26">
-        <v>1</v>
-      </c>
-      <c r="O7" s="24">
-        <v>0</v>
-      </c>
-      <c r="P7" s="24">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="24">
-        <v>0</v>
-      </c>
-      <c r="R7" s="24">
-        <v>1</v>
-      </c>
-      <c r="S7" s="24">
-        <v>0</v>
-      </c>
-      <c r="T7" s="25">
-        <v>0</v>
-      </c>
-      <c r="U7" s="25">
-        <v>1</v>
-      </c>
-      <c r="V7" s="25">
-        <v>1</v>
-      </c>
-      <c r="W7" s="25">
-        <v>1</v>
-      </c>
-      <c r="X7" s="25">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="24">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="24">
-        <v>1</v>
-      </c>
-      <c r="AB7" s="24">
-        <v>1</v>
-      </c>
-      <c r="AC7" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD7" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE7" s="25">
-        <v>1</v>
-      </c>
-      <c r="AF7" s="25">
-        <v>0</v>
-      </c>
-      <c r="AG7" s="25">
-        <v>0</v>
-      </c>
-      <c r="AH7" s="24">
+      <c r="C7" s="13">
+        <v>0</v>
+      </c>
+      <c r="D7" s="13">
+        <v>0</v>
+      </c>
+      <c r="E7" s="13">
+        <v>0</v>
+      </c>
+      <c r="F7" s="13">
+        <v>0</v>
+      </c>
+      <c r="G7" s="13">
+        <v>0</v>
+      </c>
+      <c r="H7" s="13">
+        <v>0</v>
+      </c>
+      <c r="I7" s="13">
+        <v>0</v>
+      </c>
+      <c r="J7" s="13">
+        <v>0</v>
+      </c>
+      <c r="K7" s="13">
+        <v>0</v>
+      </c>
+      <c r="L7" s="13">
+        <v>0</v>
+      </c>
+      <c r="M7" s="13">
+        <v>1</v>
+      </c>
+      <c r="N7" s="13">
+        <v>1</v>
+      </c>
+      <c r="O7" s="11">
+        <v>0</v>
+      </c>
+      <c r="P7" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="11">
+        <v>0</v>
+      </c>
+      <c r="R7" s="11">
+        <v>1</v>
+      </c>
+      <c r="S7" s="11">
+        <v>0</v>
+      </c>
+      <c r="T7" s="12">
+        <v>0</v>
+      </c>
+      <c r="U7" s="12">
+        <v>1</v>
+      </c>
+      <c r="V7" s="12">
+        <v>1</v>
+      </c>
+      <c r="W7" s="12">
+        <v>1</v>
+      </c>
+      <c r="X7" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB7" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC7" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="12">
+        <v>1</v>
+      </c>
+      <c r="AF7" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH7" s="11">
         <v>0</v>
       </c>
       <c r="AI7" s="8" t="str">
@@ -2368,100 +2359,100 @@
       <c r="B8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="26">
-        <v>0</v>
-      </c>
-      <c r="D8" s="26">
-        <v>0</v>
-      </c>
-      <c r="E8" s="26">
-        <v>0</v>
-      </c>
-      <c r="F8" s="26">
-        <v>0</v>
-      </c>
-      <c r="G8" s="26">
-        <v>0</v>
-      </c>
-      <c r="H8" s="26">
-        <v>0</v>
-      </c>
-      <c r="I8" s="26">
-        <v>0</v>
-      </c>
-      <c r="J8" s="26">
-        <v>0</v>
-      </c>
-      <c r="K8" s="26">
-        <v>0</v>
-      </c>
-      <c r="L8" s="26">
-        <v>1</v>
-      </c>
-      <c r="M8" s="26">
-        <v>0</v>
-      </c>
-      <c r="N8" s="26">
-        <v>0</v>
-      </c>
-      <c r="O8" s="29">
-        <v>0</v>
-      </c>
-      <c r="P8" s="29">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="29">
-        <v>0</v>
-      </c>
-      <c r="R8" s="29">
-        <v>1</v>
-      </c>
-      <c r="S8" s="29">
-        <v>0</v>
-      </c>
-      <c r="T8" s="25">
-        <v>1</v>
-      </c>
-      <c r="U8" s="25">
-        <v>0</v>
-      </c>
-      <c r="V8" s="25">
-        <v>0</v>
-      </c>
-      <c r="W8" s="25">
-        <v>1</v>
-      </c>
-      <c r="X8" s="25">
-        <v>1</v>
-      </c>
-      <c r="Y8" s="24">
-        <v>1</v>
-      </c>
-      <c r="Z8" s="24">
-        <v>0</v>
-      </c>
-      <c r="AA8" s="24">
-        <v>0</v>
-      </c>
-      <c r="AB8" s="24">
-        <v>0</v>
-      </c>
-      <c r="AC8" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD8" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE8" s="25">
-        <v>1</v>
-      </c>
-      <c r="AF8" s="25">
-        <v>0</v>
-      </c>
-      <c r="AG8" s="25">
-        <v>1</v>
-      </c>
-      <c r="AH8" s="24">
+      <c r="C8" s="13">
+        <v>0</v>
+      </c>
+      <c r="D8" s="13">
+        <v>0</v>
+      </c>
+      <c r="E8" s="13">
+        <v>0</v>
+      </c>
+      <c r="F8" s="13">
+        <v>0</v>
+      </c>
+      <c r="G8" s="13">
+        <v>0</v>
+      </c>
+      <c r="H8" s="13">
+        <v>0</v>
+      </c>
+      <c r="I8" s="13">
+        <v>0</v>
+      </c>
+      <c r="J8" s="13">
+        <v>0</v>
+      </c>
+      <c r="K8" s="13">
+        <v>0</v>
+      </c>
+      <c r="L8" s="13">
+        <v>1</v>
+      </c>
+      <c r="M8" s="13">
+        <v>0</v>
+      </c>
+      <c r="N8" s="13">
+        <v>0</v>
+      </c>
+      <c r="O8" s="11">
+        <v>0</v>
+      </c>
+      <c r="P8" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="11">
+        <v>0</v>
+      </c>
+      <c r="R8" s="11">
+        <v>1</v>
+      </c>
+      <c r="S8" s="11">
+        <v>0</v>
+      </c>
+      <c r="T8" s="12">
+        <v>1</v>
+      </c>
+      <c r="U8" s="12">
+        <v>0</v>
+      </c>
+      <c r="V8" s="12">
+        <v>0</v>
+      </c>
+      <c r="W8" s="12">
+        <v>1</v>
+      </c>
+      <c r="X8" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="11">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="12">
+        <v>1</v>
+      </c>
+      <c r="AF8" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG8" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH8" s="11">
         <v>0</v>
       </c>
       <c r="AI8" s="8" t="str">
@@ -2489,100 +2480,100 @@
       <c r="B9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="26">
-        <v>0</v>
-      </c>
-      <c r="D9" s="26">
-        <v>0</v>
-      </c>
-      <c r="E9" s="26">
-        <v>0</v>
-      </c>
-      <c r="F9" s="26">
-        <v>0</v>
-      </c>
-      <c r="G9" s="26">
-        <v>0</v>
-      </c>
-      <c r="H9" s="26">
-        <v>0</v>
-      </c>
-      <c r="I9" s="26">
-        <v>0</v>
-      </c>
-      <c r="J9" s="26">
-        <v>0</v>
-      </c>
-      <c r="K9" s="26">
-        <v>0</v>
-      </c>
-      <c r="L9" s="26">
-        <v>0</v>
-      </c>
-      <c r="M9" s="26">
-        <v>0</v>
-      </c>
-      <c r="N9" s="26">
-        <v>0</v>
-      </c>
-      <c r="O9" s="26">
-        <v>0</v>
-      </c>
-      <c r="P9" s="26">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="26">
-        <v>0</v>
-      </c>
-      <c r="R9" s="26">
-        <v>0</v>
-      </c>
-      <c r="S9" s="26">
-        <v>0</v>
-      </c>
-      <c r="T9" s="25">
-        <v>0</v>
-      </c>
-      <c r="U9" s="25">
-        <v>0</v>
-      </c>
-      <c r="V9" s="25">
-        <v>0</v>
-      </c>
-      <c r="W9" s="25">
-        <v>0</v>
-      </c>
-      <c r="X9" s="25">
-        <v>1</v>
-      </c>
-      <c r="Y9" s="26">
-        <v>0</v>
-      </c>
-      <c r="Z9" s="26">
-        <v>1</v>
-      </c>
-      <c r="AA9" s="26">
-        <v>0</v>
-      </c>
-      <c r="AB9" s="26">
-        <v>0</v>
-      </c>
-      <c r="AC9" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD9" s="25">
-        <v>1</v>
-      </c>
-      <c r="AE9" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF9" s="25">
-        <v>0</v>
-      </c>
-      <c r="AG9" s="25">
-        <v>1</v>
-      </c>
-      <c r="AH9" s="24">
+      <c r="C9" s="13">
+        <v>0</v>
+      </c>
+      <c r="D9" s="13">
+        <v>0</v>
+      </c>
+      <c r="E9" s="13">
+        <v>0</v>
+      </c>
+      <c r="F9" s="13">
+        <v>0</v>
+      </c>
+      <c r="G9" s="13">
+        <v>0</v>
+      </c>
+      <c r="H9" s="13">
+        <v>0</v>
+      </c>
+      <c r="I9" s="13">
+        <v>0</v>
+      </c>
+      <c r="J9" s="13">
+        <v>0</v>
+      </c>
+      <c r="K9" s="13">
+        <v>0</v>
+      </c>
+      <c r="L9" s="13">
+        <v>0</v>
+      </c>
+      <c r="M9" s="13">
+        <v>0</v>
+      </c>
+      <c r="N9" s="13">
+        <v>0</v>
+      </c>
+      <c r="O9" s="13">
+        <v>0</v>
+      </c>
+      <c r="P9" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="13">
+        <v>0</v>
+      </c>
+      <c r="R9" s="13">
+        <v>0</v>
+      </c>
+      <c r="S9" s="13">
+        <v>0</v>
+      </c>
+      <c r="T9" s="12">
+        <v>0</v>
+      </c>
+      <c r="U9" s="12">
+        <v>0</v>
+      </c>
+      <c r="V9" s="12">
+        <v>0</v>
+      </c>
+      <c r="W9" s="12">
+        <v>0</v>
+      </c>
+      <c r="X9" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="13">
+        <v>1</v>
+      </c>
+      <c r="Z9" s="13">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="13">
+        <v>1</v>
+      </c>
+      <c r="AB9" s="13">
+        <v>1</v>
+      </c>
+      <c r="AC9" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="12">
+        <v>1</v>
+      </c>
+      <c r="AE9" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF9" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG9" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH9" s="11">
         <v>0</v>
       </c>
       <c r="AI9" s="8" t="str">
@@ -2595,79 +2586,79 @@
       </c>
       <c r="AK9" s="6" t="str">
         <f t="shared" ref="AK9:AK18" si="7">BIN2HEX(_xlfn.CONCAT(S9:Z9),2)</f>
-        <v>05</v>
+        <v>06</v>
       </c>
       <c r="AL9" s="5" t="str">
         <f t="shared" ref="AL9:AL18" si="8">BIN2HEX(_xlfn.CONCAT(AA9:AH9),2)</f>
-        <v>12</v>
+        <v>D2</v>
       </c>
       <c r="AM9" t="str">
         <f t="shared" ref="AM9:AM18" si="9">_xlfn.CONCAT("0x",AI9:AL9)</f>
-        <v>0x00000512</v>
+        <v>0x000006D2</v>
       </c>
     </row>
     <row r="10" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="26">
-        <v>1</v>
-      </c>
-      <c r="D10" s="26">
-        <v>0</v>
-      </c>
-      <c r="E10" s="26">
-        <v>1</v>
-      </c>
-      <c r="F10" s="26">
-        <v>1</v>
-      </c>
-      <c r="G10" s="26">
-        <v>1</v>
-      </c>
-      <c r="H10" s="26">
-        <v>1</v>
-      </c>
-      <c r="I10" s="26">
-        <v>1</v>
-      </c>
-      <c r="J10" s="26">
-        <v>0</v>
-      </c>
-      <c r="K10" s="26">
-        <v>1</v>
-      </c>
-      <c r="L10" s="26">
-        <v>1</v>
-      </c>
-      <c r="M10" s="26">
-        <v>1</v>
-      </c>
-      <c r="N10" s="26">
-        <v>0</v>
-      </c>
-      <c r="O10" s="26">
-        <v>1</v>
-      </c>
-      <c r="P10" s="26">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="26">
-        <v>1</v>
-      </c>
-      <c r="R10" s="26">
-        <v>1</v>
-      </c>
-      <c r="S10" s="26">
-        <v>0</v>
-      </c>
-      <c r="T10" s="26">
-        <v>0</v>
-      </c>
-      <c r="U10" s="26">
-        <v>0</v>
-      </c>
-      <c r="V10" s="26">
+      <c r="C10" s="13">
+        <v>1</v>
+      </c>
+      <c r="D10" s="13">
+        <v>0</v>
+      </c>
+      <c r="E10" s="13">
+        <v>1</v>
+      </c>
+      <c r="F10" s="13">
+        <v>1</v>
+      </c>
+      <c r="G10" s="13">
+        <v>1</v>
+      </c>
+      <c r="H10" s="13">
+        <v>1</v>
+      </c>
+      <c r="I10" s="13">
+        <v>1</v>
+      </c>
+      <c r="J10" s="13">
+        <v>0</v>
+      </c>
+      <c r="K10" s="13">
+        <v>1</v>
+      </c>
+      <c r="L10" s="13">
+        <v>1</v>
+      </c>
+      <c r="M10" s="13">
+        <v>1</v>
+      </c>
+      <c r="N10" s="13">
+        <v>0</v>
+      </c>
+      <c r="O10" s="13">
+        <v>1</v>
+      </c>
+      <c r="P10" s="13">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="13">
+        <v>1</v>
+      </c>
+      <c r="R10" s="13">
+        <v>1</v>
+      </c>
+      <c r="S10" s="13">
+        <v>0</v>
+      </c>
+      <c r="T10" s="13">
+        <v>0</v>
+      </c>
+      <c r="U10" s="13">
+        <v>0</v>
+      </c>
+      <c r="V10" s="13">
         <v>0</v>
       </c>
       <c r="W10" s="3">
@@ -2676,34 +2667,34 @@
       <c r="X10" s="3">
         <v>0</v>
       </c>
-      <c r="Y10" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z10" s="24">
-        <v>0</v>
-      </c>
-      <c r="AA10" s="24">
-        <v>0</v>
-      </c>
-      <c r="AB10" s="24">
-        <v>0</v>
-      </c>
-      <c r="AC10" s="25">
-        <v>1</v>
-      </c>
-      <c r="AD10" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE10" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF10" s="25">
-        <v>0</v>
-      </c>
-      <c r="AG10" s="25">
-        <v>1</v>
-      </c>
-      <c r="AH10" s="24">
+      <c r="Y10" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="12">
+        <v>1</v>
+      </c>
+      <c r="AD10" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF10" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG10" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH10" s="11">
         <v>0</v>
       </c>
       <c r="AI10" s="8" t="str">
@@ -2731,64 +2722,64 @@
       <c r="B11" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="26">
-        <v>0</v>
-      </c>
-      <c r="D11" s="26">
-        <v>0</v>
-      </c>
-      <c r="E11" s="26">
-        <v>0</v>
-      </c>
-      <c r="F11" s="26">
-        <v>0</v>
-      </c>
-      <c r="G11" s="26">
-        <v>0</v>
-      </c>
-      <c r="H11" s="26">
-        <v>0</v>
-      </c>
-      <c r="I11" s="26">
-        <v>0</v>
-      </c>
-      <c r="J11" s="26">
-        <v>0</v>
-      </c>
-      <c r="K11" s="26">
-        <v>0</v>
-      </c>
-      <c r="L11" s="26">
-        <v>0</v>
-      </c>
-      <c r="M11" s="26">
-        <v>0</v>
-      </c>
-      <c r="N11" s="26">
-        <v>0</v>
-      </c>
-      <c r="O11" s="26">
-        <v>0</v>
-      </c>
-      <c r="P11" s="26">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="26">
-        <v>0</v>
-      </c>
-      <c r="R11" s="26">
-        <v>0</v>
-      </c>
-      <c r="S11" s="26">
-        <v>0</v>
-      </c>
-      <c r="T11" s="26">
-        <v>0</v>
-      </c>
-      <c r="U11" s="26">
-        <v>0</v>
-      </c>
-      <c r="V11" s="26">
+      <c r="C11" s="13">
+        <v>0</v>
+      </c>
+      <c r="D11" s="13">
+        <v>0</v>
+      </c>
+      <c r="E11" s="13">
+        <v>0</v>
+      </c>
+      <c r="F11" s="13">
+        <v>0</v>
+      </c>
+      <c r="G11" s="13">
+        <v>0</v>
+      </c>
+      <c r="H11" s="13">
+        <v>0</v>
+      </c>
+      <c r="I11" s="13">
+        <v>0</v>
+      </c>
+      <c r="J11" s="13">
+        <v>0</v>
+      </c>
+      <c r="K11" s="13">
+        <v>0</v>
+      </c>
+      <c r="L11" s="13">
+        <v>0</v>
+      </c>
+      <c r="M11" s="13">
+        <v>0</v>
+      </c>
+      <c r="N11" s="13">
+        <v>0</v>
+      </c>
+      <c r="O11" s="13">
+        <v>0</v>
+      </c>
+      <c r="P11" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="13">
+        <v>0</v>
+      </c>
+      <c r="R11" s="13">
+        <v>0</v>
+      </c>
+      <c r="S11" s="13">
+        <v>0</v>
+      </c>
+      <c r="T11" s="13">
+        <v>0</v>
+      </c>
+      <c r="U11" s="13">
+        <v>0</v>
+      </c>
+      <c r="V11" s="13">
         <v>0</v>
       </c>
       <c r="W11" s="3">
@@ -2797,34 +2788,34 @@
       <c r="X11" s="3">
         <v>0</v>
       </c>
-      <c r="Y11" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z11" s="24">
-        <v>0</v>
-      </c>
-      <c r="AA11" s="24">
-        <v>0</v>
-      </c>
-      <c r="AB11" s="24">
-        <v>1</v>
-      </c>
-      <c r="AC11" s="25">
-        <v>1</v>
-      </c>
-      <c r="AD11" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE11" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF11" s="25">
-        <v>0</v>
-      </c>
-      <c r="AG11" s="25">
-        <v>1</v>
-      </c>
-      <c r="AH11" s="24">
+      <c r="Y11" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC11" s="12">
+        <v>1</v>
+      </c>
+      <c r="AD11" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE11" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF11" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG11" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH11" s="11">
         <v>0</v>
       </c>
       <c r="AI11" s="8" t="str">
@@ -2852,25 +2843,25 @@
       <c r="B12" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="24">
-        <v>0</v>
-      </c>
-      <c r="D12" s="24">
-        <v>0</v>
-      </c>
-      <c r="E12" s="24">
-        <v>0</v>
-      </c>
-      <c r="F12" s="24">
-        <v>0</v>
-      </c>
-      <c r="G12" s="24">
-        <v>0</v>
-      </c>
-      <c r="H12" s="24">
-        <v>0</v>
-      </c>
-      <c r="I12" s="24">
+      <c r="C12" s="11">
+        <v>0</v>
+      </c>
+      <c r="D12" s="11">
+        <v>0</v>
+      </c>
+      <c r="E12" s="11">
+        <v>0</v>
+      </c>
+      <c r="F12" s="11">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11">
+        <v>0</v>
+      </c>
+      <c r="H12" s="11">
+        <v>0</v>
+      </c>
+      <c r="I12" s="11">
         <v>0</v>
       </c>
       <c r="J12" s="3">
@@ -2882,70 +2873,70 @@
       <c r="L12" s="3">
         <v>0</v>
       </c>
-      <c r="M12" s="24">
-        <v>0</v>
-      </c>
-      <c r="N12" s="24">
-        <v>0</v>
-      </c>
-      <c r="O12" s="24">
-        <v>0</v>
-      </c>
-      <c r="P12" s="25">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="25">
-        <v>1</v>
-      </c>
-      <c r="R12" s="25">
-        <v>0</v>
-      </c>
-      <c r="S12" s="24">
-        <v>0</v>
-      </c>
-      <c r="T12" s="24">
-        <v>0</v>
-      </c>
-      <c r="U12" s="24">
-        <v>1</v>
-      </c>
-      <c r="V12" s="25">
-        <v>0</v>
-      </c>
-      <c r="W12" s="25">
-        <v>0</v>
-      </c>
-      <c r="X12" s="25">
-        <v>0</v>
-      </c>
-      <c r="Y12" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z12" s="24">
-        <v>1</v>
-      </c>
-      <c r="AA12" s="24">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="24">
-        <v>1</v>
-      </c>
-      <c r="AC12" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD12" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE12" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF12" s="25">
-        <v>1</v>
-      </c>
-      <c r="AG12" s="25">
-        <v>0</v>
-      </c>
-      <c r="AH12" s="24">
+      <c r="M12" s="11">
+        <v>0</v>
+      </c>
+      <c r="N12" s="11">
+        <v>0</v>
+      </c>
+      <c r="O12" s="11">
+        <v>0</v>
+      </c>
+      <c r="P12" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="12">
+        <v>1</v>
+      </c>
+      <c r="R12" s="12">
+        <v>0</v>
+      </c>
+      <c r="S12" s="11">
+        <v>0</v>
+      </c>
+      <c r="T12" s="11">
+        <v>0</v>
+      </c>
+      <c r="U12" s="11">
+        <v>1</v>
+      </c>
+      <c r="V12" s="12">
+        <v>0</v>
+      </c>
+      <c r="W12" s="12">
+        <v>0</v>
+      </c>
+      <c r="X12" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="11">
+        <v>1</v>
+      </c>
+      <c r="AA12" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC12" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF12" s="12">
+        <v>1</v>
+      </c>
+      <c r="AG12" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH12" s="11">
         <v>0</v>
       </c>
       <c r="AI12" s="8" t="str">
@@ -2973,100 +2964,100 @@
       <c r="B13" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="26">
-        <v>0</v>
-      </c>
-      <c r="D13" s="26">
-        <v>0</v>
-      </c>
-      <c r="E13" s="26">
-        <v>0</v>
-      </c>
-      <c r="F13" s="26">
-        <v>0</v>
-      </c>
-      <c r="G13" s="26">
-        <v>0</v>
-      </c>
-      <c r="H13" s="26">
-        <v>0</v>
-      </c>
-      <c r="I13" s="26">
-        <v>0</v>
-      </c>
-      <c r="J13" s="26">
-        <v>0</v>
-      </c>
-      <c r="K13" s="26">
-        <v>0</v>
-      </c>
-      <c r="L13" s="26">
-        <v>0</v>
-      </c>
-      <c r="M13" s="26">
-        <v>0</v>
-      </c>
-      <c r="N13" s="26">
-        <v>0</v>
-      </c>
-      <c r="O13" s="26">
-        <v>0</v>
-      </c>
-      <c r="P13" s="26">
-        <v>1</v>
-      </c>
-      <c r="Q13" s="26">
-        <v>1</v>
-      </c>
-      <c r="R13" s="26">
-        <v>0</v>
-      </c>
-      <c r="S13" s="24">
-        <v>0</v>
-      </c>
-      <c r="T13" s="24">
-        <v>0</v>
-      </c>
-      <c r="U13" s="24">
-        <v>0</v>
-      </c>
-      <c r="V13" s="25">
-        <v>1</v>
-      </c>
-      <c r="W13" s="25">
-        <v>0</v>
-      </c>
-      <c r="X13" s="25">
-        <v>1</v>
-      </c>
-      <c r="Y13" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z13" s="24">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="24">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="24">
-        <v>0</v>
-      </c>
-      <c r="AC13" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD13" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE13" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF13" s="25">
-        <v>1</v>
-      </c>
-      <c r="AG13" s="25">
-        <v>1</v>
-      </c>
-      <c r="AH13" s="24">
+      <c r="C13" s="13">
+        <v>0</v>
+      </c>
+      <c r="D13" s="13">
+        <v>0</v>
+      </c>
+      <c r="E13" s="13">
+        <v>0</v>
+      </c>
+      <c r="F13" s="13">
+        <v>0</v>
+      </c>
+      <c r="G13" s="13">
+        <v>0</v>
+      </c>
+      <c r="H13" s="13">
+        <v>0</v>
+      </c>
+      <c r="I13" s="13">
+        <v>0</v>
+      </c>
+      <c r="J13" s="13">
+        <v>0</v>
+      </c>
+      <c r="K13" s="13">
+        <v>0</v>
+      </c>
+      <c r="L13" s="13">
+        <v>0</v>
+      </c>
+      <c r="M13" s="13">
+        <v>0</v>
+      </c>
+      <c r="N13" s="13">
+        <v>0</v>
+      </c>
+      <c r="O13" s="13">
+        <v>0</v>
+      </c>
+      <c r="P13" s="13">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="13">
+        <v>1</v>
+      </c>
+      <c r="R13" s="13">
+        <v>0</v>
+      </c>
+      <c r="S13" s="11">
+        <v>0</v>
+      </c>
+      <c r="T13" s="11">
+        <v>0</v>
+      </c>
+      <c r="U13" s="11">
+        <v>0</v>
+      </c>
+      <c r="V13" s="12">
+        <v>1</v>
+      </c>
+      <c r="W13" s="12">
+        <v>0</v>
+      </c>
+      <c r="X13" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y13" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF13" s="12">
+        <v>1</v>
+      </c>
+      <c r="AG13" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH13" s="11">
         <v>0</v>
       </c>
       <c r="AI13" s="8" t="str">
@@ -3094,25 +3085,25 @@
       <c r="B14" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="24">
-        <v>0</v>
-      </c>
-      <c r="D14" s="24">
-        <v>0</v>
-      </c>
-      <c r="E14" s="24">
-        <v>0</v>
-      </c>
-      <c r="F14" s="24">
-        <v>0</v>
-      </c>
-      <c r="G14" s="24">
-        <v>0</v>
-      </c>
-      <c r="H14" s="24">
-        <v>0</v>
-      </c>
-      <c r="I14" s="24">
+      <c r="C14" s="11">
+        <v>0</v>
+      </c>
+      <c r="D14" s="11">
+        <v>0</v>
+      </c>
+      <c r="E14" s="11">
+        <v>0</v>
+      </c>
+      <c r="F14" s="11">
+        <v>0</v>
+      </c>
+      <c r="G14" s="11">
+        <v>0</v>
+      </c>
+      <c r="H14" s="11">
+        <v>0</v>
+      </c>
+      <c r="I14" s="11">
         <v>0</v>
       </c>
       <c r="J14" s="3">
@@ -3124,70 +3115,70 @@
       <c r="L14" s="3">
         <v>1</v>
       </c>
-      <c r="M14" s="24">
-        <v>0</v>
-      </c>
-      <c r="N14" s="24">
-        <v>1</v>
-      </c>
-      <c r="O14" s="24">
-        <v>0</v>
-      </c>
-      <c r="P14" s="25">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="25">
-        <v>0</v>
-      </c>
-      <c r="R14" s="25">
-        <v>1</v>
-      </c>
-      <c r="S14" s="24">
-        <v>1</v>
-      </c>
-      <c r="T14" s="24">
-        <v>0</v>
-      </c>
-      <c r="U14" s="24">
-        <v>1</v>
-      </c>
-      <c r="V14" s="25">
-        <v>0</v>
-      </c>
-      <c r="W14" s="25">
-        <v>0</v>
-      </c>
-      <c r="X14" s="25">
-        <v>0</v>
-      </c>
-      <c r="Y14" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="24">
-        <v>0</v>
-      </c>
-      <c r="AA14" s="24">
-        <v>1</v>
-      </c>
-      <c r="AB14" s="24">
-        <v>0</v>
-      </c>
-      <c r="AC14" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD14" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE14" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF14" s="25">
-        <v>1</v>
-      </c>
-      <c r="AG14" s="25">
-        <v>0</v>
-      </c>
-      <c r="AH14" s="24">
+      <c r="M14" s="11">
+        <v>0</v>
+      </c>
+      <c r="N14" s="11">
+        <v>1</v>
+      </c>
+      <c r="O14" s="11">
+        <v>0</v>
+      </c>
+      <c r="P14" s="12">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="12">
+        <v>0</v>
+      </c>
+      <c r="R14" s="12">
+        <v>1</v>
+      </c>
+      <c r="S14" s="11">
+        <v>1</v>
+      </c>
+      <c r="T14" s="11">
+        <v>0</v>
+      </c>
+      <c r="U14" s="11">
+        <v>1</v>
+      </c>
+      <c r="V14" s="12">
+        <v>0</v>
+      </c>
+      <c r="W14" s="12">
+        <v>0</v>
+      </c>
+      <c r="X14" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB14" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC14" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF14" s="12">
+        <v>1</v>
+      </c>
+      <c r="AG14" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH14" s="11">
         <v>1</v>
       </c>
       <c r="AI14" s="8" t="str">
@@ -3215,100 +3206,100 @@
       <c r="B15" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="26">
-        <v>1</v>
-      </c>
-      <c r="D15" s="26">
-        <v>1</v>
-      </c>
-      <c r="E15" s="26">
-        <v>1</v>
-      </c>
-      <c r="F15" s="26">
-        <v>1</v>
-      </c>
-      <c r="G15" s="26">
-        <v>1</v>
-      </c>
-      <c r="H15" s="26">
-        <v>1</v>
-      </c>
-      <c r="I15" s="26">
-        <v>1</v>
-      </c>
-      <c r="J15" s="26">
-        <v>1</v>
-      </c>
-      <c r="K15" s="26">
-        <v>1</v>
-      </c>
-      <c r="L15" s="26">
-        <v>1</v>
-      </c>
-      <c r="M15" s="26">
-        <v>1</v>
-      </c>
-      <c r="N15" s="26">
-        <v>1</v>
-      </c>
-      <c r="O15" s="26">
-        <v>1</v>
-      </c>
-      <c r="P15" s="26">
-        <v>1</v>
-      </c>
-      <c r="Q15" s="26">
-        <v>1</v>
-      </c>
-      <c r="R15" s="26">
-        <v>0</v>
-      </c>
-      <c r="S15" s="24">
-        <v>0</v>
-      </c>
-      <c r="T15" s="24">
-        <v>1</v>
-      </c>
-      <c r="U15" s="24">
-        <v>1</v>
-      </c>
-      <c r="V15" s="25">
-        <v>0</v>
-      </c>
-      <c r="W15" s="25">
-        <v>0</v>
-      </c>
-      <c r="X15" s="25">
-        <v>1</v>
-      </c>
-      <c r="Y15" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z15" s="24">
-        <v>1</v>
-      </c>
-      <c r="AA15" s="24">
-        <v>0</v>
-      </c>
-      <c r="AB15" s="24">
-        <v>0</v>
-      </c>
-      <c r="AC15" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD15" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE15" s="25">
-        <v>1</v>
-      </c>
-      <c r="AF15" s="25">
-        <v>1</v>
-      </c>
-      <c r="AG15" s="25">
-        <v>0</v>
-      </c>
-      <c r="AH15" s="24">
+      <c r="C15" s="13">
+        <v>1</v>
+      </c>
+      <c r="D15" s="13">
+        <v>1</v>
+      </c>
+      <c r="E15" s="13">
+        <v>1</v>
+      </c>
+      <c r="F15" s="13">
+        <v>1</v>
+      </c>
+      <c r="G15" s="13">
+        <v>1</v>
+      </c>
+      <c r="H15" s="13">
+        <v>1</v>
+      </c>
+      <c r="I15" s="13">
+        <v>1</v>
+      </c>
+      <c r="J15" s="13">
+        <v>1</v>
+      </c>
+      <c r="K15" s="13">
+        <v>1</v>
+      </c>
+      <c r="L15" s="13">
+        <v>1</v>
+      </c>
+      <c r="M15" s="13">
+        <v>1</v>
+      </c>
+      <c r="N15" s="13">
+        <v>1</v>
+      </c>
+      <c r="O15" s="13">
+        <v>1</v>
+      </c>
+      <c r="P15" s="13">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="13">
+        <v>1</v>
+      </c>
+      <c r="R15" s="13">
+        <v>0</v>
+      </c>
+      <c r="S15" s="11">
+        <v>0</v>
+      </c>
+      <c r="T15" s="11">
+        <v>1</v>
+      </c>
+      <c r="U15" s="11">
+        <v>1</v>
+      </c>
+      <c r="V15" s="12">
+        <v>0</v>
+      </c>
+      <c r="W15" s="12">
+        <v>0</v>
+      </c>
+      <c r="X15" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y15" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="11">
+        <v>1</v>
+      </c>
+      <c r="AA15" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB15" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD15" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE15" s="12">
+        <v>1</v>
+      </c>
+      <c r="AF15" s="12">
+        <v>1</v>
+      </c>
+      <c r="AG15" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH15" s="11">
         <v>0</v>
       </c>
       <c r="AI15" s="8" t="str">
@@ -3336,100 +3327,100 @@
       <c r="B16" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="26">
-        <v>1</v>
-      </c>
-      <c r="D16" s="26">
-        <v>1</v>
-      </c>
-      <c r="E16" s="26">
-        <v>1</v>
-      </c>
-      <c r="F16" s="26">
-        <v>1</v>
-      </c>
-      <c r="G16" s="26">
-        <v>1</v>
-      </c>
-      <c r="H16" s="26">
-        <v>1</v>
-      </c>
-      <c r="I16" s="26">
-        <v>1</v>
-      </c>
-      <c r="J16" s="26">
-        <v>1</v>
-      </c>
-      <c r="K16" s="26">
-        <v>1</v>
-      </c>
-      <c r="L16" s="26">
-        <v>1</v>
-      </c>
-      <c r="M16" s="26">
-        <v>1</v>
-      </c>
-      <c r="N16" s="26">
-        <v>1</v>
-      </c>
-      <c r="O16" s="26">
-        <v>1</v>
-      </c>
-      <c r="P16" s="26">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="26">
-        <v>1</v>
-      </c>
-      <c r="R16" s="26">
-        <v>1</v>
-      </c>
-      <c r="S16" s="24">
-        <v>0</v>
-      </c>
-      <c r="T16" s="24">
-        <v>1</v>
-      </c>
-      <c r="U16" s="24">
-        <v>1</v>
-      </c>
-      <c r="V16" s="28">
-        <v>0</v>
-      </c>
-      <c r="W16" s="28">
-        <v>1</v>
-      </c>
-      <c r="X16" s="28">
-        <v>0</v>
-      </c>
-      <c r="Y16" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z16" s="24">
-        <v>0</v>
-      </c>
-      <c r="AA16" s="24">
-        <v>1</v>
-      </c>
-      <c r="AB16" s="24">
-        <v>1</v>
-      </c>
-      <c r="AC16" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD16" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE16" s="25">
-        <v>1</v>
-      </c>
-      <c r="AF16" s="25">
-        <v>1</v>
-      </c>
-      <c r="AG16" s="25">
-        <v>1</v>
-      </c>
-      <c r="AH16" s="24">
+      <c r="C16" s="13">
+        <v>1</v>
+      </c>
+      <c r="D16" s="13">
+        <v>1</v>
+      </c>
+      <c r="E16" s="13">
+        <v>1</v>
+      </c>
+      <c r="F16" s="13">
+        <v>1</v>
+      </c>
+      <c r="G16" s="13">
+        <v>1</v>
+      </c>
+      <c r="H16" s="13">
+        <v>1</v>
+      </c>
+      <c r="I16" s="13">
+        <v>1</v>
+      </c>
+      <c r="J16" s="13">
+        <v>1</v>
+      </c>
+      <c r="K16" s="13">
+        <v>1</v>
+      </c>
+      <c r="L16" s="13">
+        <v>1</v>
+      </c>
+      <c r="M16" s="13">
+        <v>1</v>
+      </c>
+      <c r="N16" s="13">
+        <v>1</v>
+      </c>
+      <c r="O16" s="13">
+        <v>1</v>
+      </c>
+      <c r="P16" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="13">
+        <v>1</v>
+      </c>
+      <c r="R16" s="13">
+        <v>1</v>
+      </c>
+      <c r="S16" s="11">
+        <v>0</v>
+      </c>
+      <c r="T16" s="11">
+        <v>1</v>
+      </c>
+      <c r="U16" s="11">
+        <v>1</v>
+      </c>
+      <c r="V16" s="12">
+        <v>0</v>
+      </c>
+      <c r="W16" s="12">
+        <v>1</v>
+      </c>
+      <c r="X16" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB16" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC16" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD16" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE16" s="12">
+        <v>1</v>
+      </c>
+      <c r="AF16" s="12">
+        <v>1</v>
+      </c>
+      <c r="AG16" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH16" s="11">
         <v>0</v>
       </c>
       <c r="AI16" s="8" t="str">
@@ -3493,19 +3484,19 @@
       <c r="N17" s="3">
         <v>0</v>
       </c>
-      <c r="O17" s="29">
-        <v>1</v>
-      </c>
-      <c r="P17" s="29">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="29">
-        <v>0</v>
-      </c>
-      <c r="R17" s="29">
-        <v>0</v>
-      </c>
-      <c r="S17" s="29">
+      <c r="O17" s="11">
+        <v>1</v>
+      </c>
+      <c r="P17" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="11">
+        <v>0</v>
+      </c>
+      <c r="R17" s="11">
+        <v>0</v>
+      </c>
+      <c r="S17" s="11">
         <v>1</v>
       </c>
       <c r="T17" s="3">
@@ -3514,43 +3505,43 @@
       <c r="U17" s="3">
         <v>0</v>
       </c>
-      <c r="V17" s="28">
-        <v>0</v>
-      </c>
-      <c r="W17" s="28">
-        <v>1</v>
-      </c>
-      <c r="X17" s="28">
-        <v>0</v>
-      </c>
-      <c r="Y17" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z17" s="24">
-        <v>0</v>
-      </c>
-      <c r="AA17" s="24">
-        <v>0</v>
-      </c>
-      <c r="AB17" s="24">
-        <v>0</v>
-      </c>
-      <c r="AC17" s="25">
-        <v>1</v>
-      </c>
-      <c r="AD17" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE17" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF17" s="25">
-        <v>0</v>
-      </c>
-      <c r="AG17" s="25">
-        <v>0</v>
-      </c>
-      <c r="AH17" s="24">
+      <c r="V17" s="12">
+        <v>0</v>
+      </c>
+      <c r="W17" s="12">
+        <v>1</v>
+      </c>
+      <c r="X17" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB17" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC17" s="12">
+        <v>1</v>
+      </c>
+      <c r="AD17" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE17" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF17" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG17" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH17" s="11">
         <v>0</v>
       </c>
       <c r="AI17" s="8" t="str">
@@ -3617,61 +3608,61 @@
       <c r="O18" s="3">
         <v>0</v>
       </c>
-      <c r="P18" s="29">
-        <v>1</v>
-      </c>
-      <c r="Q18" s="29">
-        <v>0</v>
-      </c>
-      <c r="R18" s="29">
+      <c r="P18" s="11">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="11">
+        <v>0</v>
+      </c>
+      <c r="R18" s="11">
         <v>1</v>
       </c>
       <c r="S18" s="3">
         <v>0</v>
       </c>
-      <c r="T18" s="28">
-        <v>0</v>
-      </c>
-      <c r="U18" s="28">
-        <v>1</v>
-      </c>
-      <c r="V18" s="28">
-        <v>1</v>
-      </c>
-      <c r="W18" s="28">
-        <v>1</v>
-      </c>
-      <c r="X18" s="28">
-        <v>0</v>
-      </c>
-      <c r="Y18" s="24">
-        <v>0</v>
-      </c>
-      <c r="Z18" s="24">
-        <v>0</v>
-      </c>
-      <c r="AA18" s="24">
-        <v>0</v>
-      </c>
-      <c r="AB18" s="24">
-        <v>1</v>
-      </c>
-      <c r="AC18" s="25">
-        <v>1</v>
-      </c>
-      <c r="AD18" s="25">
-        <v>0</v>
-      </c>
-      <c r="AE18" s="25">
-        <v>0</v>
-      </c>
-      <c r="AF18" s="25">
-        <v>0</v>
-      </c>
-      <c r="AG18" s="25">
-        <v>0</v>
-      </c>
-      <c r="AH18" s="24">
+      <c r="T18" s="12">
+        <v>0</v>
+      </c>
+      <c r="U18" s="12">
+        <v>1</v>
+      </c>
+      <c r="V18" s="12">
+        <v>1</v>
+      </c>
+      <c r="W18" s="12">
+        <v>1</v>
+      </c>
+      <c r="X18" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB18" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC18" s="12">
+        <v>1</v>
+      </c>
+      <c r="AD18" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE18" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF18" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG18" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH18" s="11">
         <v>0</v>
       </c>
       <c r="AI18" s="8" t="str">

</xml_diff>

<commit_message>
feat(sv): testbench para el datapath
</commit_message>
<xml_diff>
--- a/res/isa.xlsx
+++ b/res/isa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\workbench\repos\CE4301--p2_fobando_isa--\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{120388A2-2551-4D62-8CAE-7210F7BC860E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D8C9AE-62C3-4E28-9AD6-44C33E04427F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{EC7525CD-E51C-4E61-B306-9CBCE090E85A}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="58">
   <si>
     <t>R</t>
   </si>
@@ -193,6 +193,27 @@
   </si>
   <si>
     <t>recv r0, fx</t>
+  </si>
+  <si>
+    <t>movi r0, 15</t>
+  </si>
+  <si>
+    <t>movi r2, -9</t>
+  </si>
+  <si>
+    <t>sub r1, r0, r2</t>
+  </si>
+  <si>
+    <t>mov p0, r1</t>
+  </si>
+  <si>
+    <t>ldw p1,+ 0(zero)</t>
+  </si>
+  <si>
+    <t>muli p2, p1, -1</t>
+  </si>
+  <si>
+    <t>stb p2,+ 3(zero)</t>
   </si>
 </sst>
 </file>
@@ -485,15 +506,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -519,6 +531,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -969,49 +990,49 @@
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="15" t="s">
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="15" t="s">
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="O3" s="16"/>
-      <c r="P3" s="16"/>
-      <c r="Q3" s="16"/>
-      <c r="R3" s="17"/>
-      <c r="S3" s="15" t="s">
+      <c r="O3" s="25"/>
+      <c r="P3" s="25"/>
+      <c r="Q3" s="25"/>
+      <c r="R3" s="26"/>
+      <c r="S3" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="T3" s="16"/>
-      <c r="U3" s="16"/>
-      <c r="V3" s="16"/>
-      <c r="W3" s="17"/>
-      <c r="X3" s="15" t="s">
+      <c r="T3" s="25"/>
+      <c r="U3" s="25"/>
+      <c r="V3" s="25"/>
+      <c r="W3" s="26"/>
+      <c r="X3" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="Y3" s="16"/>
-      <c r="Z3" s="16"/>
-      <c r="AA3" s="17"/>
-      <c r="AB3" s="15" t="s">
+      <c r="Y3" s="25"/>
+      <c r="Z3" s="25"/>
+      <c r="AA3" s="26"/>
+      <c r="AB3" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AC3" s="16"/>
-      <c r="AD3" s="16"/>
-      <c r="AE3" s="16"/>
-      <c r="AF3" s="17"/>
+      <c r="AC3" s="25"/>
+      <c r="AD3" s="25"/>
+      <c r="AE3" s="25"/>
+      <c r="AF3" s="26"/>
       <c r="AG3" s="3" t="s">
         <v>16</v>
       </c>
@@ -1020,47 +1041,47 @@
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="15" t="s">
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-      <c r="R4" s="17"/>
-      <c r="S4" s="15" t="s">
+      <c r="O4" s="25"/>
+      <c r="P4" s="25"/>
+      <c r="Q4" s="25"/>
+      <c r="R4" s="26"/>
+      <c r="S4" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="T4" s="16"/>
-      <c r="U4" s="16"/>
-      <c r="V4" s="16"/>
-      <c r="W4" s="17"/>
-      <c r="X4" s="15" t="s">
+      <c r="T4" s="25"/>
+      <c r="U4" s="25"/>
+      <c r="V4" s="25"/>
+      <c r="W4" s="26"/>
+      <c r="X4" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="Y4" s="16"/>
-      <c r="Z4" s="16"/>
-      <c r="AA4" s="17"/>
-      <c r="AB4" s="15" t="s">
+      <c r="Y4" s="25"/>
+      <c r="Z4" s="25"/>
+      <c r="AA4" s="26"/>
+      <c r="AB4" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AC4" s="16"/>
-      <c r="AD4" s="16"/>
-      <c r="AE4" s="16"/>
-      <c r="AF4" s="17"/>
+      <c r="AC4" s="25"/>
+      <c r="AD4" s="25"/>
+      <c r="AE4" s="25"/>
+      <c r="AF4" s="26"/>
       <c r="AG4" s="3" t="s">
         <v>16</v>
       </c>
@@ -1069,34 +1090,34 @@
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="15" t="s">
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="25"/>
+      <c r="J5" s="25"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="O5" s="16"/>
-      <c r="P5" s="16"/>
-      <c r="Q5" s="16"/>
-      <c r="R5" s="17"/>
-      <c r="S5" s="15" t="s">
+      <c r="O5" s="25"/>
+      <c r="P5" s="25"/>
+      <c r="Q5" s="25"/>
+      <c r="R5" s="26"/>
+      <c r="S5" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="T5" s="16"/>
-      <c r="U5" s="16"/>
-      <c r="V5" s="16"/>
-      <c r="W5" s="17"/>
+      <c r="T5" s="25"/>
+      <c r="U5" s="25"/>
+      <c r="V5" s="25"/>
+      <c r="W5" s="26"/>
       <c r="X5" s="3" t="s">
         <v>19</v>
       </c>
@@ -1109,13 +1130,13 @@
       <c r="AA5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AB5" s="15" t="s">
+      <c r="AB5" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AC5" s="16"/>
-      <c r="AD5" s="16"/>
-      <c r="AE5" s="16"/>
-      <c r="AF5" s="17"/>
+      <c r="AC5" s="25"/>
+      <c r="AD5" s="25"/>
+      <c r="AE5" s="25"/>
+      <c r="AF5" s="26"/>
       <c r="AG5" s="3" t="s">
         <v>16</v>
       </c>
@@ -1124,49 +1145,49 @@
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="15" t="s">
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="15" t="s">
+      <c r="J6" s="25"/>
+      <c r="K6" s="25"/>
+      <c r="L6" s="25"/>
+      <c r="M6" s="26"/>
+      <c r="N6" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="O6" s="16"/>
-      <c r="P6" s="16"/>
-      <c r="Q6" s="16"/>
-      <c r="R6" s="17"/>
-      <c r="S6" s="15" t="s">
+      <c r="O6" s="25"/>
+      <c r="P6" s="25"/>
+      <c r="Q6" s="25"/>
+      <c r="R6" s="26"/>
+      <c r="S6" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="T6" s="16"/>
-      <c r="U6" s="16"/>
-      <c r="V6" s="16"/>
-      <c r="W6" s="17"/>
-      <c r="X6" s="15" t="s">
+      <c r="T6" s="25"/>
+      <c r="U6" s="25"/>
+      <c r="V6" s="25"/>
+      <c r="W6" s="26"/>
+      <c r="X6" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="Y6" s="16"/>
-      <c r="Z6" s="16"/>
-      <c r="AA6" s="17"/>
-      <c r="AB6" s="15" t="s">
+      <c r="Y6" s="25"/>
+      <c r="Z6" s="25"/>
+      <c r="AA6" s="26"/>
+      <c r="AB6" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AC6" s="16"/>
-      <c r="AD6" s="16"/>
-      <c r="AE6" s="16"/>
-      <c r="AF6" s="17"/>
+      <c r="AC6" s="25"/>
+      <c r="AD6" s="25"/>
+      <c r="AE6" s="25"/>
+      <c r="AF6" s="26"/>
       <c r="AG6" s="3" t="s">
         <v>16</v>
       </c>
@@ -1175,45 +1196,45 @@
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="16"/>
-      <c r="Q7" s="16"/>
-      <c r="R7" s="17"/>
-      <c r="S7" s="15" t="s">
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="25"/>
+      <c r="J7" s="25"/>
+      <c r="K7" s="25"/>
+      <c r="L7" s="25"/>
+      <c r="M7" s="25"/>
+      <c r="N7" s="25"/>
+      <c r="O7" s="25"/>
+      <c r="P7" s="25"/>
+      <c r="Q7" s="25"/>
+      <c r="R7" s="26"/>
+      <c r="S7" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="T7" s="16"/>
-      <c r="U7" s="16"/>
-      <c r="V7" s="16"/>
-      <c r="W7" s="17"/>
-      <c r="X7" s="15" t="s">
+      <c r="T7" s="25"/>
+      <c r="U7" s="25"/>
+      <c r="V7" s="25"/>
+      <c r="W7" s="26"/>
+      <c r="X7" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="Y7" s="16"/>
-      <c r="Z7" s="16"/>
-      <c r="AA7" s="17"/>
-      <c r="AB7" s="15" t="s">
+      <c r="Y7" s="25"/>
+      <c r="Z7" s="25"/>
+      <c r="AA7" s="26"/>
+      <c r="AB7" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AC7" s="16"/>
-      <c r="AD7" s="16"/>
-      <c r="AE7" s="16"/>
-      <c r="AF7" s="17"/>
+      <c r="AC7" s="25"/>
+      <c r="AD7" s="25"/>
+      <c r="AE7" s="25"/>
+      <c r="AF7" s="26"/>
       <c r="AG7" s="3" t="s">
         <v>16</v>
       </c>
@@ -1222,47 +1243,47 @@
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="16"/>
-      <c r="S8" s="16"/>
-      <c r="T8" s="16"/>
-      <c r="U8" s="17"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="25"/>
+      <c r="I8" s="25"/>
+      <c r="J8" s="25"/>
+      <c r="K8" s="25"/>
+      <c r="L8" s="25"/>
+      <c r="M8" s="25"/>
+      <c r="N8" s="25"/>
+      <c r="O8" s="25"/>
+      <c r="P8" s="25"/>
+      <c r="Q8" s="25"/>
+      <c r="R8" s="25"/>
+      <c r="S8" s="25"/>
+      <c r="T8" s="25"/>
+      <c r="U8" s="26"/>
       <c r="V8" s="3">
         <v>0</v>
       </c>
       <c r="W8" s="3">
         <v>0</v>
       </c>
-      <c r="X8" s="15" t="s">
+      <c r="X8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="Y8" s="16"/>
-      <c r="Z8" s="16"/>
-      <c r="AA8" s="17"/>
-      <c r="AB8" s="15" t="s">
+      <c r="Y8" s="25"/>
+      <c r="Z8" s="25"/>
+      <c r="AA8" s="26"/>
+      <c r="AB8" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AC8" s="16"/>
-      <c r="AD8" s="16"/>
-      <c r="AE8" s="16"/>
-      <c r="AF8" s="17"/>
+      <c r="AC8" s="25"/>
+      <c r="AD8" s="25"/>
+      <c r="AE8" s="25"/>
+      <c r="AF8" s="26"/>
       <c r="AG8" s="3" t="s">
         <v>16</v>
       </c>
@@ -1271,34 +1292,34 @@
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="16"/>
-      <c r="P9" s="16"/>
-      <c r="Q9" s="17"/>
-      <c r="R9" s="15" t="s">
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="25"/>
+      <c r="J9" s="25"/>
+      <c r="K9" s="25"/>
+      <c r="L9" s="25"/>
+      <c r="M9" s="25"/>
+      <c r="N9" s="25"/>
+      <c r="O9" s="25"/>
+      <c r="P9" s="25"/>
+      <c r="Q9" s="26"/>
+      <c r="R9" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="S9" s="16"/>
-      <c r="T9" s="17"/>
-      <c r="U9" s="15" t="s">
+      <c r="S9" s="25"/>
+      <c r="T9" s="26"/>
+      <c r="U9" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="V9" s="16"/>
-      <c r="W9" s="17"/>
+      <c r="V9" s="25"/>
+      <c r="W9" s="26"/>
       <c r="X9" s="3" t="s">
         <v>19</v>
       </c>
@@ -1311,13 +1332,13 @@
       <c r="AA9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AB9" s="15" t="s">
+      <c r="AB9" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AC9" s="16"/>
-      <c r="AD9" s="16"/>
-      <c r="AE9" s="16"/>
-      <c r="AF9" s="17"/>
+      <c r="AC9" s="25"/>
+      <c r="AD9" s="25"/>
+      <c r="AE9" s="25"/>
+      <c r="AF9" s="26"/>
       <c r="AG9" s="3" t="s">
         <v>16</v>
       </c>
@@ -1326,53 +1347,53 @@
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="15" t="s">
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="J10" s="16"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="15" t="s">
+      <c r="J10" s="25"/>
+      <c r="K10" s="26"/>
+      <c r="L10" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="M10" s="16"/>
-      <c r="N10" s="17"/>
-      <c r="O10" s="15" t="s">
+      <c r="M10" s="25"/>
+      <c r="N10" s="26"/>
+      <c r="O10" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="P10" s="16"/>
-      <c r="Q10" s="17"/>
-      <c r="R10" s="15" t="s">
+      <c r="P10" s="25"/>
+      <c r="Q10" s="26"/>
+      <c r="R10" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="S10" s="16"/>
-      <c r="T10" s="17"/>
-      <c r="U10" s="15" t="s">
+      <c r="S10" s="25"/>
+      <c r="T10" s="26"/>
+      <c r="U10" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="V10" s="16"/>
-      <c r="W10" s="17"/>
-      <c r="X10" s="15" t="s">
+      <c r="V10" s="25"/>
+      <c r="W10" s="26"/>
+      <c r="X10" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="Y10" s="16"/>
-      <c r="Z10" s="16"/>
-      <c r="AA10" s="17"/>
-      <c r="AB10" s="15" t="s">
+      <c r="Y10" s="25"/>
+      <c r="Z10" s="25"/>
+      <c r="AA10" s="26"/>
+      <c r="AB10" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AC10" s="16"/>
-      <c r="AD10" s="16"/>
-      <c r="AE10" s="16"/>
-      <c r="AF10" s="17"/>
+      <c r="AC10" s="25"/>
+      <c r="AD10" s="25"/>
+      <c r="AE10" s="25"/>
+      <c r="AF10" s="26"/>
       <c r="AG10" s="3" t="s">
         <v>16</v>
       </c>
@@ -1381,53 +1402,53 @@
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="16"/>
-      <c r="O11" s="16"/>
-      <c r="P11" s="16"/>
-      <c r="Q11" s="17"/>
-      <c r="R11" s="15" t="s">
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="25"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="25"/>
+      <c r="M11" s="25"/>
+      <c r="N11" s="25"/>
+      <c r="O11" s="25"/>
+      <c r="P11" s="25"/>
+      <c r="Q11" s="26"/>
+      <c r="R11" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="S11" s="16"/>
-      <c r="T11" s="17"/>
-      <c r="U11" s="15" t="s">
+      <c r="S11" s="25"/>
+      <c r="T11" s="26"/>
+      <c r="U11" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="V11" s="16"/>
-      <c r="W11" s="17"/>
-      <c r="X11" s="15" t="s">
+      <c r="V11" s="25"/>
+      <c r="W11" s="26"/>
+      <c r="X11" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="Y11" s="16"/>
-      <c r="Z11" s="16"/>
-      <c r="AA11" s="17"/>
-      <c r="AB11" s="15" t="s">
+      <c r="Y11" s="25"/>
+      <c r="Z11" s="25"/>
+      <c r="AA11" s="26"/>
+      <c r="AB11" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AC11" s="16"/>
-      <c r="AD11" s="16"/>
-      <c r="AE11" s="16"/>
-      <c r="AF11" s="17"/>
+      <c r="AC11" s="25"/>
+      <c r="AD11" s="25"/>
+      <c r="AE11" s="25"/>
+      <c r="AF11" s="26"/>
       <c r="AG11" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="15" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="3">
@@ -1466,43 +1487,43 @@
       <c r="M12" s="3">
         <v>0</v>
       </c>
-      <c r="N12" s="15" t="s">
+      <c r="N12" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="O12" s="16"/>
-      <c r="P12" s="16"/>
-      <c r="Q12" s="16"/>
-      <c r="R12" s="17"/>
+      <c r="O12" s="25"/>
+      <c r="P12" s="25"/>
+      <c r="Q12" s="25"/>
+      <c r="R12" s="26"/>
       <c r="S12" s="3">
         <v>0</v>
       </c>
       <c r="T12" s="3">
         <v>0</v>
       </c>
-      <c r="U12" s="15" t="s">
+      <c r="U12" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="V12" s="16"/>
-      <c r="W12" s="17"/>
-      <c r="X12" s="19" t="s">
+      <c r="V12" s="25"/>
+      <c r="W12" s="26"/>
+      <c r="X12" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="Y12" s="20"/>
-      <c r="Z12" s="20"/>
-      <c r="AA12" s="21"/>
-      <c r="AB12" s="19" t="s">
+      <c r="Y12" s="17"/>
+      <c r="Z12" s="17"/>
+      <c r="AA12" s="18"/>
+      <c r="AB12" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="AC12" s="20"/>
-      <c r="AD12" s="20"/>
-      <c r="AE12" s="20"/>
-      <c r="AF12" s="21"/>
-      <c r="AG12" s="25" t="s">
+      <c r="AC12" s="17"/>
+      <c r="AD12" s="17"/>
+      <c r="AE12" s="17"/>
+      <c r="AF12" s="18"/>
+      <c r="AG12" s="22" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A13" s="18"/>
+      <c r="A13" s="15"/>
       <c r="B13" s="3">
         <v>0</v>
       </c>
@@ -1542,50 +1563,62 @@
       <c r="N13" s="3">
         <v>0</v>
       </c>
-      <c r="O13" s="15" t="s">
+      <c r="O13" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="P13" s="16"/>
-      <c r="Q13" s="17"/>
+      <c r="P13" s="25"/>
+      <c r="Q13" s="26"/>
       <c r="R13" s="9">
         <v>0</v>
       </c>
-      <c r="S13" s="15" t="s">
+      <c r="S13" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="T13" s="16"/>
-      <c r="U13" s="16"/>
-      <c r="V13" s="16"/>
-      <c r="W13" s="17"/>
-      <c r="X13" s="22"/>
-      <c r="Y13" s="23"/>
-      <c r="Z13" s="23"/>
-      <c r="AA13" s="24"/>
-      <c r="AB13" s="22"/>
-      <c r="AC13" s="23"/>
-      <c r="AD13" s="23"/>
-      <c r="AE13" s="23"/>
-      <c r="AF13" s="24"/>
-      <c r="AG13" s="26"/>
+      <c r="T13" s="25"/>
+      <c r="U13" s="25"/>
+      <c r="V13" s="25"/>
+      <c r="W13" s="26"/>
+      <c r="X13" s="19"/>
+      <c r="Y13" s="20"/>
+      <c r="Z13" s="20"/>
+      <c r="AA13" s="21"/>
+      <c r="AB13" s="19"/>
+      <c r="AC13" s="20"/>
+      <c r="AD13" s="20"/>
+      <c r="AE13" s="20"/>
+      <c r="AF13" s="21"/>
+      <c r="AG13" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="X12:AA13"/>
-    <mergeCell ref="AB12:AF13"/>
-    <mergeCell ref="AG12:AG13"/>
-    <mergeCell ref="S13:W13"/>
-    <mergeCell ref="O13:Q13"/>
-    <mergeCell ref="B11:Q11"/>
-    <mergeCell ref="U12:W12"/>
-    <mergeCell ref="N12:R12"/>
-    <mergeCell ref="R11:T11"/>
-    <mergeCell ref="U11:W11"/>
-    <mergeCell ref="X11:AA11"/>
-    <mergeCell ref="AB11:AF11"/>
-    <mergeCell ref="AB9:AF9"/>
-    <mergeCell ref="U9:W9"/>
-    <mergeCell ref="R9:T9"/>
+    <mergeCell ref="AB3:AF3"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="N3:R3"/>
+    <mergeCell ref="S3:W3"/>
+    <mergeCell ref="X3:AA3"/>
+    <mergeCell ref="AB4:AF4"/>
+    <mergeCell ref="B5:M5"/>
+    <mergeCell ref="N5:R5"/>
+    <mergeCell ref="S5:W5"/>
+    <mergeCell ref="AB5:AF5"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="N4:R4"/>
+    <mergeCell ref="S4:W4"/>
+    <mergeCell ref="X4:AA4"/>
+    <mergeCell ref="AB6:AF6"/>
+    <mergeCell ref="X6:AA6"/>
+    <mergeCell ref="I6:M6"/>
+    <mergeCell ref="N6:R6"/>
+    <mergeCell ref="S6:W6"/>
+    <mergeCell ref="AB7:AF7"/>
+    <mergeCell ref="X7:AA7"/>
+    <mergeCell ref="S7:W7"/>
+    <mergeCell ref="B7:R7"/>
+    <mergeCell ref="X8:AA8"/>
+    <mergeCell ref="AB8:AF8"/>
+    <mergeCell ref="B8:U8"/>
     <mergeCell ref="B9:Q9"/>
     <mergeCell ref="X10:AA10"/>
     <mergeCell ref="AB10:AF10"/>
@@ -1595,34 +1628,22 @@
     <mergeCell ref="I10:K10"/>
     <mergeCell ref="B10:H10"/>
     <mergeCell ref="L10:N10"/>
-    <mergeCell ref="AB7:AF7"/>
-    <mergeCell ref="X7:AA7"/>
-    <mergeCell ref="S7:W7"/>
-    <mergeCell ref="B7:R7"/>
-    <mergeCell ref="X8:AA8"/>
-    <mergeCell ref="AB8:AF8"/>
-    <mergeCell ref="B8:U8"/>
-    <mergeCell ref="AB6:AF6"/>
-    <mergeCell ref="X6:AA6"/>
-    <mergeCell ref="I6:M6"/>
-    <mergeCell ref="N6:R6"/>
-    <mergeCell ref="S6:W6"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B4:M4"/>
-    <mergeCell ref="N4:R4"/>
-    <mergeCell ref="S4:W4"/>
-    <mergeCell ref="X4:AA4"/>
-    <mergeCell ref="AB4:AF4"/>
-    <mergeCell ref="B5:M5"/>
-    <mergeCell ref="N5:R5"/>
-    <mergeCell ref="S5:W5"/>
-    <mergeCell ref="AB5:AF5"/>
-    <mergeCell ref="AB3:AF3"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="N3:R3"/>
-    <mergeCell ref="S3:W3"/>
-    <mergeCell ref="X3:AA3"/>
+    <mergeCell ref="X11:AA11"/>
+    <mergeCell ref="AB11:AF11"/>
+    <mergeCell ref="AB9:AF9"/>
+    <mergeCell ref="U9:W9"/>
+    <mergeCell ref="R9:T9"/>
+    <mergeCell ref="B11:Q11"/>
+    <mergeCell ref="U12:W12"/>
+    <mergeCell ref="N12:R12"/>
+    <mergeCell ref="R11:T11"/>
+    <mergeCell ref="U11:W11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="X12:AA13"/>
+    <mergeCell ref="AB12:AF13"/>
+    <mergeCell ref="AG12:AG13"/>
+    <mergeCell ref="S13:W13"/>
+    <mergeCell ref="O13:Q13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1630,7 +1651,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65E70CF8-F0FC-43B5-8B1F-488A2F898887}">
-  <dimension ref="A2:AM26"/>
+  <dimension ref="A2:AM42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="10"/>
@@ -3687,9 +3708,7 @@
       </c>
     </row>
     <row r="19" spans="2:39" x14ac:dyDescent="0.3">
-      <c r="B19" s="2" t="s">
-        <v>34</v>
-      </c>
+      <c r="B19" s="2"/>
       <c r="C19" s="3">
         <v>0</v>
       </c>
@@ -3809,102 +3828,102 @@
     </row>
     <row r="20" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B20" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C20" s="3">
-        <v>0</v>
-      </c>
-      <c r="D20" s="3">
-        <v>0</v>
-      </c>
-      <c r="E20" s="3">
-        <v>0</v>
-      </c>
-      <c r="F20" s="3">
-        <v>0</v>
-      </c>
-      <c r="G20" s="3">
-        <v>0</v>
-      </c>
-      <c r="H20" s="3">
-        <v>0</v>
-      </c>
-      <c r="I20" s="3">
-        <v>0</v>
-      </c>
-      <c r="J20" s="3">
-        <v>0</v>
-      </c>
-      <c r="K20" s="3">
-        <v>0</v>
-      </c>
-      <c r="L20" s="3">
-        <v>0</v>
-      </c>
-      <c r="M20" s="3">
-        <v>0</v>
-      </c>
-      <c r="N20" s="3">
-        <v>0</v>
-      </c>
-      <c r="O20" s="3">
-        <v>0</v>
-      </c>
-      <c r="P20" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="3">
-        <v>0</v>
-      </c>
-      <c r="R20" s="3">
-        <v>0</v>
-      </c>
-      <c r="S20" s="3">
-        <v>0</v>
-      </c>
-      <c r="T20" s="3">
-        <v>0</v>
-      </c>
-      <c r="U20" s="3">
-        <v>0</v>
-      </c>
-      <c r="V20" s="3">
-        <v>0</v>
-      </c>
-      <c r="W20" s="3">
-        <v>0</v>
-      </c>
-      <c r="X20" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y20" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH20" s="3">
+        <v>51</v>
+      </c>
+      <c r="C20" s="13">
+        <v>0</v>
+      </c>
+      <c r="D20" s="13">
+        <v>0</v>
+      </c>
+      <c r="E20" s="13">
+        <v>0</v>
+      </c>
+      <c r="F20" s="13">
+        <v>0</v>
+      </c>
+      <c r="G20" s="13">
+        <v>0</v>
+      </c>
+      <c r="H20" s="13">
+        <v>0</v>
+      </c>
+      <c r="I20" s="13">
+        <v>0</v>
+      </c>
+      <c r="J20" s="13">
+        <v>0</v>
+      </c>
+      <c r="K20" s="13">
+        <v>1</v>
+      </c>
+      <c r="L20" s="13">
+        <v>1</v>
+      </c>
+      <c r="M20" s="13">
+        <v>1</v>
+      </c>
+      <c r="N20" s="13">
+        <v>1</v>
+      </c>
+      <c r="O20" s="11">
+        <v>0</v>
+      </c>
+      <c r="P20" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="11">
+        <v>0</v>
+      </c>
+      <c r="R20" s="11">
+        <v>0</v>
+      </c>
+      <c r="S20" s="11">
+        <v>0</v>
+      </c>
+      <c r="T20" s="12">
+        <v>0</v>
+      </c>
+      <c r="U20" s="12">
+        <v>1</v>
+      </c>
+      <c r="V20" s="12">
+        <v>1</v>
+      </c>
+      <c r="W20" s="12">
+        <v>1</v>
+      </c>
+      <c r="X20" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB20" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD20" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG20" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH20" s="11">
         <v>0</v>
       </c>
       <c r="AI20" s="8" t="str">
@@ -3913,361 +3932,361 @@
       </c>
       <c r="AJ20" s="7" t="str">
         <f t="shared" si="11"/>
-        <v>00</v>
+        <v>F0</v>
       </c>
       <c r="AK20" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>00</v>
+        <v>38</v>
       </c>
       <c r="AL20" s="5" t="str">
         <f t="shared" si="13"/>
-        <v>00</v>
+        <v>82</v>
       </c>
       <c r="AM20" t="str">
         <f t="shared" si="14"/>
-        <v>0x00000000</v>
+        <v>0x00F03882</v>
       </c>
     </row>
     <row r="21" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B21" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="3">
-        <v>0</v>
-      </c>
-      <c r="D21" s="3">
-        <v>0</v>
-      </c>
-      <c r="E21" s="3">
-        <v>0</v>
-      </c>
-      <c r="F21" s="3">
-        <v>0</v>
-      </c>
-      <c r="G21" s="3">
-        <v>0</v>
-      </c>
-      <c r="H21" s="3">
-        <v>0</v>
-      </c>
-      <c r="I21" s="3">
-        <v>0</v>
-      </c>
-      <c r="J21" s="3">
-        <v>0</v>
-      </c>
-      <c r="K21" s="3">
-        <v>0</v>
-      </c>
-      <c r="L21" s="3">
-        <v>0</v>
-      </c>
-      <c r="M21" s="3">
-        <v>0</v>
-      </c>
-      <c r="N21" s="3">
-        <v>0</v>
-      </c>
-      <c r="O21" s="3">
-        <v>0</v>
-      </c>
-      <c r="P21" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="3">
-        <v>0</v>
-      </c>
-      <c r="R21" s="3">
-        <v>0</v>
-      </c>
-      <c r="S21" s="3">
-        <v>0</v>
-      </c>
-      <c r="T21" s="3">
-        <v>0</v>
-      </c>
-      <c r="U21" s="3">
-        <v>0</v>
-      </c>
-      <c r="V21" s="3">
-        <v>0</v>
-      </c>
-      <c r="W21" s="3">
-        <v>0</v>
-      </c>
-      <c r="X21" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y21" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH21" s="3">
+        <v>52</v>
+      </c>
+      <c r="C21" s="13">
+        <v>1</v>
+      </c>
+      <c r="D21" s="13">
+        <v>1</v>
+      </c>
+      <c r="E21" s="13">
+        <v>1</v>
+      </c>
+      <c r="F21" s="13">
+        <v>1</v>
+      </c>
+      <c r="G21" s="13">
+        <v>1</v>
+      </c>
+      <c r="H21" s="13">
+        <v>1</v>
+      </c>
+      <c r="I21" s="13">
+        <v>1</v>
+      </c>
+      <c r="J21" s="13">
+        <v>1</v>
+      </c>
+      <c r="K21" s="13">
+        <v>0</v>
+      </c>
+      <c r="L21" s="13">
+        <v>1</v>
+      </c>
+      <c r="M21" s="13">
+        <v>1</v>
+      </c>
+      <c r="N21" s="13">
+        <v>1</v>
+      </c>
+      <c r="O21" s="11">
+        <v>0</v>
+      </c>
+      <c r="P21" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="11">
+        <v>0</v>
+      </c>
+      <c r="R21" s="11">
+        <v>0</v>
+      </c>
+      <c r="S21" s="11">
+        <v>0</v>
+      </c>
+      <c r="T21" s="12">
+        <v>1</v>
+      </c>
+      <c r="U21" s="12">
+        <v>0</v>
+      </c>
+      <c r="V21" s="12">
+        <v>0</v>
+      </c>
+      <c r="W21" s="12">
+        <v>0</v>
+      </c>
+      <c r="X21" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB21" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC21" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD21" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF21" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG21" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH21" s="11">
         <v>0</v>
       </c>
       <c r="AI21" s="8" t="str">
         <f t="shared" si="10"/>
-        <v>00</v>
+        <v>FF</v>
       </c>
       <c r="AJ21" s="7" t="str">
         <f t="shared" si="11"/>
-        <v>00</v>
+        <v>70</v>
       </c>
       <c r="AK21" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>00</v>
+        <v>40</v>
       </c>
       <c r="AL21" s="5" t="str">
         <f t="shared" si="13"/>
-        <v>00</v>
+        <v>82</v>
       </c>
       <c r="AM21" t="str">
         <f t="shared" si="14"/>
-        <v>0x00000000</v>
+        <v>0xFF704082</v>
       </c>
     </row>
     <row r="22" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B22" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C22" s="3">
-        <v>0</v>
-      </c>
-      <c r="D22" s="3">
-        <v>0</v>
-      </c>
-      <c r="E22" s="3">
-        <v>0</v>
-      </c>
-      <c r="F22" s="3">
-        <v>0</v>
-      </c>
-      <c r="G22" s="3">
-        <v>0</v>
-      </c>
-      <c r="H22" s="3">
-        <v>0</v>
-      </c>
-      <c r="I22" s="3">
-        <v>0</v>
-      </c>
-      <c r="J22" s="3">
-        <v>0</v>
-      </c>
-      <c r="K22" s="3">
-        <v>0</v>
-      </c>
-      <c r="L22" s="3">
-        <v>0</v>
-      </c>
-      <c r="M22" s="3">
-        <v>0</v>
-      </c>
-      <c r="N22" s="3">
-        <v>0</v>
-      </c>
-      <c r="O22" s="3">
-        <v>0</v>
-      </c>
-      <c r="P22" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="3">
-        <v>0</v>
-      </c>
-      <c r="R22" s="3">
-        <v>0</v>
-      </c>
-      <c r="S22" s="3">
-        <v>0</v>
-      </c>
-      <c r="T22" s="3">
-        <v>0</v>
-      </c>
-      <c r="U22" s="3">
-        <v>0</v>
-      </c>
-      <c r="V22" s="3">
-        <v>0</v>
-      </c>
-      <c r="W22" s="3">
-        <v>0</v>
-      </c>
-      <c r="X22" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH22" s="3">
+        <v>53</v>
+      </c>
+      <c r="C22" s="11">
+        <v>0</v>
+      </c>
+      <c r="D22" s="11">
+        <v>0</v>
+      </c>
+      <c r="E22" s="11">
+        <v>0</v>
+      </c>
+      <c r="F22" s="11">
+        <v>0</v>
+      </c>
+      <c r="G22" s="11">
+        <v>0</v>
+      </c>
+      <c r="H22" s="11">
+        <v>0</v>
+      </c>
+      <c r="I22" s="11">
+        <v>0</v>
+      </c>
+      <c r="J22" s="12">
+        <v>1</v>
+      </c>
+      <c r="K22" s="12">
+        <v>0</v>
+      </c>
+      <c r="L22" s="12">
+        <v>0</v>
+      </c>
+      <c r="M22" s="12">
+        <v>0</v>
+      </c>
+      <c r="N22" s="12">
+        <v>0</v>
+      </c>
+      <c r="O22" s="11">
+        <v>0</v>
+      </c>
+      <c r="P22" s="11">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="11">
+        <v>1</v>
+      </c>
+      <c r="R22" s="11">
+        <v>1</v>
+      </c>
+      <c r="S22" s="11">
+        <v>0</v>
+      </c>
+      <c r="T22" s="12">
+        <v>0</v>
+      </c>
+      <c r="U22" s="12">
+        <v>1</v>
+      </c>
+      <c r="V22" s="12">
+        <v>1</v>
+      </c>
+      <c r="W22" s="12">
+        <v>1</v>
+      </c>
+      <c r="X22" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y22" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB22" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC22" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF22" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG22" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH22" s="11">
         <v>0</v>
       </c>
       <c r="AI22" s="8" t="str">
         <f t="shared" si="10"/>
-        <v>00</v>
+        <v>01</v>
       </c>
       <c r="AJ22" s="7" t="str">
         <f t="shared" si="11"/>
-        <v>00</v>
+        <v>07</v>
       </c>
       <c r="AK22" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>00</v>
+        <v>3C</v>
       </c>
       <c r="AL22" s="5" t="str">
         <f t="shared" si="13"/>
-        <v>00</v>
+        <v>C0</v>
       </c>
       <c r="AM22" t="str">
         <f t="shared" si="14"/>
-        <v>0x00000000</v>
+        <v>0x01073CC0</v>
       </c>
     </row>
     <row r="23" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C23" s="3">
-        <v>0</v>
-      </c>
-      <c r="D23" s="3">
-        <v>0</v>
-      </c>
-      <c r="E23" s="3">
-        <v>0</v>
-      </c>
-      <c r="F23" s="3">
-        <v>0</v>
-      </c>
-      <c r="G23" s="3">
-        <v>0</v>
-      </c>
-      <c r="H23" s="3">
-        <v>0</v>
-      </c>
-      <c r="I23" s="3">
-        <v>0</v>
-      </c>
-      <c r="J23" s="3">
-        <v>0</v>
-      </c>
-      <c r="K23" s="3">
-        <v>0</v>
-      </c>
-      <c r="L23" s="3">
-        <v>0</v>
-      </c>
-      <c r="M23" s="3">
-        <v>0</v>
-      </c>
-      <c r="N23" s="3">
-        <v>0</v>
-      </c>
-      <c r="O23" s="3">
-        <v>0</v>
-      </c>
-      <c r="P23" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="3">
-        <v>0</v>
-      </c>
-      <c r="R23" s="3">
-        <v>0</v>
-      </c>
-      <c r="S23" s="3">
-        <v>0</v>
-      </c>
-      <c r="T23" s="3">
-        <v>0</v>
-      </c>
-      <c r="U23" s="3">
-        <v>0</v>
-      </c>
-      <c r="V23" s="3">
-        <v>0</v>
-      </c>
-      <c r="W23" s="3">
-        <v>0</v>
-      </c>
-      <c r="X23" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y23" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH23" s="3">
+        <v>54</v>
+      </c>
+      <c r="C23" s="11">
+        <v>0</v>
+      </c>
+      <c r="D23" s="11">
+        <v>0</v>
+      </c>
+      <c r="E23" s="11">
+        <v>0</v>
+      </c>
+      <c r="F23" s="11">
+        <v>0</v>
+      </c>
+      <c r="G23" s="11">
+        <v>0</v>
+      </c>
+      <c r="H23" s="11">
+        <v>0</v>
+      </c>
+      <c r="I23" s="11">
+        <v>0</v>
+      </c>
+      <c r="J23" s="12">
+        <v>0</v>
+      </c>
+      <c r="K23" s="12">
+        <v>0</v>
+      </c>
+      <c r="L23" s="12">
+        <v>0</v>
+      </c>
+      <c r="M23" s="12">
+        <v>0</v>
+      </c>
+      <c r="N23" s="12">
+        <v>0</v>
+      </c>
+      <c r="O23" s="11">
+        <v>0</v>
+      </c>
+      <c r="P23" s="11">
+        <v>1</v>
+      </c>
+      <c r="Q23" s="11">
+        <v>1</v>
+      </c>
+      <c r="R23" s="11">
+        <v>1</v>
+      </c>
+      <c r="S23" s="11">
+        <v>1</v>
+      </c>
+      <c r="T23" s="12">
+        <v>0</v>
+      </c>
+      <c r="U23" s="12">
+        <v>0</v>
+      </c>
+      <c r="V23" s="12">
+        <v>1</v>
+      </c>
+      <c r="W23" s="12">
+        <v>0</v>
+      </c>
+      <c r="X23" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y23" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA23" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB23" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE23" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF23" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG23" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH23" s="11">
         <v>0</v>
       </c>
       <c r="AI23" s="8" t="str">
@@ -4276,119 +4295,119 @@
       </c>
       <c r="AJ23" s="7" t="str">
         <f t="shared" si="11"/>
-        <v>00</v>
+        <v>07</v>
       </c>
       <c r="AK23" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>00</v>
+        <v>94</v>
       </c>
       <c r="AL23" s="5" t="str">
         <f t="shared" si="13"/>
-        <v>00</v>
+        <v>80</v>
       </c>
       <c r="AM23" t="str">
         <f t="shared" si="14"/>
-        <v>0x00000000</v>
+        <v>0x00079480</v>
       </c>
     </row>
     <row r="24" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B24" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C24" s="3">
-        <v>0</v>
-      </c>
-      <c r="D24" s="3">
-        <v>0</v>
-      </c>
-      <c r="E24" s="3">
-        <v>0</v>
-      </c>
-      <c r="F24" s="3">
-        <v>0</v>
-      </c>
-      <c r="G24" s="3">
-        <v>0</v>
-      </c>
-      <c r="H24" s="3">
-        <v>0</v>
-      </c>
-      <c r="I24" s="3">
-        <v>0</v>
-      </c>
-      <c r="J24" s="3">
-        <v>0</v>
-      </c>
-      <c r="K24" s="3">
-        <v>0</v>
-      </c>
-      <c r="L24" s="3">
-        <v>0</v>
-      </c>
-      <c r="M24" s="3">
-        <v>0</v>
-      </c>
-      <c r="N24" s="3">
-        <v>0</v>
-      </c>
-      <c r="O24" s="3">
-        <v>0</v>
-      </c>
-      <c r="P24" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="3">
-        <v>0</v>
-      </c>
-      <c r="R24" s="3">
-        <v>0</v>
-      </c>
-      <c r="S24" s="3">
-        <v>0</v>
-      </c>
-      <c r="T24" s="3">
-        <v>0</v>
-      </c>
-      <c r="U24" s="3">
-        <v>0</v>
-      </c>
-      <c r="V24" s="3">
-        <v>0</v>
-      </c>
-      <c r="W24" s="3">
-        <v>0</v>
-      </c>
-      <c r="X24" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y24" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH24" s="3">
+        <v>55</v>
+      </c>
+      <c r="C24" s="13">
+        <v>0</v>
+      </c>
+      <c r="D24" s="13">
+        <v>0</v>
+      </c>
+      <c r="E24" s="13">
+        <v>0</v>
+      </c>
+      <c r="F24" s="13">
+        <v>0</v>
+      </c>
+      <c r="G24" s="13">
+        <v>0</v>
+      </c>
+      <c r="H24" s="13">
+        <v>0</v>
+      </c>
+      <c r="I24" s="13">
+        <v>0</v>
+      </c>
+      <c r="J24" s="13">
+        <v>0</v>
+      </c>
+      <c r="K24" s="13">
+        <v>0</v>
+      </c>
+      <c r="L24" s="13">
+        <v>0</v>
+      </c>
+      <c r="M24" s="13">
+        <v>0</v>
+      </c>
+      <c r="N24" s="13">
+        <v>0</v>
+      </c>
+      <c r="O24" s="11">
+        <v>0</v>
+      </c>
+      <c r="P24" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="11">
+        <v>0</v>
+      </c>
+      <c r="R24" s="11">
+        <v>0</v>
+      </c>
+      <c r="S24" s="11">
+        <v>0</v>
+      </c>
+      <c r="T24" s="12">
+        <v>0</v>
+      </c>
+      <c r="U24" s="12">
+        <v>0</v>
+      </c>
+      <c r="V24" s="12">
+        <v>1</v>
+      </c>
+      <c r="W24" s="12">
+        <v>1</v>
+      </c>
+      <c r="X24" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="11">
+        <v>1</v>
+      </c>
+      <c r="Z24" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC24" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD24" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="12">
+        <v>1</v>
+      </c>
+      <c r="AF24" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG24" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="11">
         <v>0</v>
       </c>
       <c r="AI24" s="8" t="str">
@@ -4401,236 +4420,236 @@
       </c>
       <c r="AK24" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>00</v>
+        <v>1A</v>
       </c>
       <c r="AL24" s="5" t="str">
         <f t="shared" si="13"/>
-        <v>00</v>
+        <v>08</v>
       </c>
       <c r="AM24" t="str">
         <f t="shared" si="14"/>
-        <v>0x00000000</v>
+        <v>0x00001A08</v>
       </c>
     </row>
     <row r="25" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B25" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C25" s="3">
-        <v>0</v>
-      </c>
-      <c r="D25" s="3">
-        <v>0</v>
-      </c>
-      <c r="E25" s="3">
-        <v>0</v>
-      </c>
-      <c r="F25" s="3">
-        <v>0</v>
-      </c>
-      <c r="G25" s="3">
-        <v>0</v>
-      </c>
-      <c r="H25" s="3">
-        <v>0</v>
-      </c>
-      <c r="I25" s="3">
-        <v>0</v>
-      </c>
-      <c r="J25" s="3">
-        <v>0</v>
-      </c>
-      <c r="K25" s="3">
-        <v>0</v>
-      </c>
-      <c r="L25" s="3">
-        <v>0</v>
-      </c>
-      <c r="M25" s="3">
-        <v>0</v>
-      </c>
-      <c r="N25" s="3">
-        <v>0</v>
-      </c>
-      <c r="O25" s="3">
-        <v>0</v>
-      </c>
-      <c r="P25" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="3">
-        <v>0</v>
-      </c>
-      <c r="R25" s="3">
-        <v>0</v>
-      </c>
-      <c r="S25" s="3">
-        <v>0</v>
-      </c>
-      <c r="T25" s="3">
-        <v>0</v>
-      </c>
-      <c r="U25" s="3">
-        <v>0</v>
-      </c>
-      <c r="V25" s="3">
-        <v>0</v>
-      </c>
-      <c r="W25" s="3">
-        <v>0</v>
-      </c>
-      <c r="X25" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y25" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z25" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA25" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB25" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC25" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD25" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE25" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF25" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG25" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH25" s="3">
+        <v>56</v>
+      </c>
+      <c r="C25" s="13">
+        <v>1</v>
+      </c>
+      <c r="D25" s="13">
+        <v>1</v>
+      </c>
+      <c r="E25" s="13">
+        <v>1</v>
+      </c>
+      <c r="F25" s="13">
+        <v>1</v>
+      </c>
+      <c r="G25" s="13">
+        <v>1</v>
+      </c>
+      <c r="H25" s="13">
+        <v>1</v>
+      </c>
+      <c r="I25" s="13">
+        <v>1</v>
+      </c>
+      <c r="J25" s="13">
+        <v>1</v>
+      </c>
+      <c r="K25" s="13">
+        <v>1</v>
+      </c>
+      <c r="L25" s="13">
+        <v>1</v>
+      </c>
+      <c r="M25" s="13">
+        <v>1</v>
+      </c>
+      <c r="N25" s="13">
+        <v>1</v>
+      </c>
+      <c r="O25" s="11">
+        <v>0</v>
+      </c>
+      <c r="P25" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="11">
+        <v>1</v>
+      </c>
+      <c r="R25" s="11">
+        <v>1</v>
+      </c>
+      <c r="S25" s="11">
+        <v>1</v>
+      </c>
+      <c r="T25" s="12">
+        <v>0</v>
+      </c>
+      <c r="U25" s="12">
+        <v>0</v>
+      </c>
+      <c r="V25" s="12">
+        <v>1</v>
+      </c>
+      <c r="W25" s="12">
+        <v>1</v>
+      </c>
+      <c r="X25" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y25" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="11">
+        <v>1</v>
+      </c>
+      <c r="AA25" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB25" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC25" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD25" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE25" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF25" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG25" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH25" s="11">
         <v>0</v>
       </c>
       <c r="AI25" s="8" t="str">
         <f t="shared" si="10"/>
-        <v>00</v>
+        <v>FF</v>
       </c>
       <c r="AJ25" s="7" t="str">
         <f t="shared" si="11"/>
-        <v>00</v>
+        <v>F3</v>
       </c>
       <c r="AK25" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>00</v>
+        <v>99</v>
       </c>
       <c r="AL25" s="5" t="str">
         <f t="shared" si="13"/>
-        <v>00</v>
+        <v>02</v>
       </c>
       <c r="AM25" t="str">
         <f t="shared" si="14"/>
-        <v>0x00000000</v>
+        <v>0xFFF39902</v>
       </c>
     </row>
     <row r="26" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B26" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C26" s="3">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3">
-        <v>0</v>
-      </c>
-      <c r="F26" s="3">
-        <v>0</v>
-      </c>
-      <c r="G26" s="3">
-        <v>0</v>
-      </c>
-      <c r="H26" s="3">
-        <v>0</v>
-      </c>
-      <c r="I26" s="3">
-        <v>0</v>
-      </c>
-      <c r="J26" s="3">
-        <v>0</v>
-      </c>
-      <c r="K26" s="3">
-        <v>0</v>
-      </c>
-      <c r="L26" s="3">
-        <v>0</v>
-      </c>
-      <c r="M26" s="3">
-        <v>0</v>
-      </c>
-      <c r="N26" s="3">
-        <v>0</v>
-      </c>
-      <c r="O26" s="3">
-        <v>0</v>
-      </c>
-      <c r="P26" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="3">
-        <v>0</v>
-      </c>
-      <c r="R26" s="3">
-        <v>0</v>
-      </c>
-      <c r="S26" s="3">
-        <v>0</v>
-      </c>
-      <c r="T26" s="3">
-        <v>0</v>
-      </c>
-      <c r="U26" s="3">
-        <v>0</v>
-      </c>
-      <c r="V26" s="3">
-        <v>0</v>
-      </c>
-      <c r="W26" s="3">
-        <v>0</v>
-      </c>
-      <c r="X26" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y26" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z26" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA26" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB26" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC26" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD26" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE26" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF26" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG26" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH26" s="3">
+        <v>57</v>
+      </c>
+      <c r="C26" s="13">
+        <v>0</v>
+      </c>
+      <c r="D26" s="13">
+        <v>0</v>
+      </c>
+      <c r="E26" s="13">
+        <v>0</v>
+      </c>
+      <c r="F26" s="13">
+        <v>0</v>
+      </c>
+      <c r="G26" s="13">
+        <v>0</v>
+      </c>
+      <c r="H26" s="13">
+        <v>0</v>
+      </c>
+      <c r="I26" s="13">
+        <v>0</v>
+      </c>
+      <c r="J26" s="13">
+        <v>0</v>
+      </c>
+      <c r="K26" s="13">
+        <v>0</v>
+      </c>
+      <c r="L26" s="13">
+        <v>0</v>
+      </c>
+      <c r="M26" s="13">
+        <v>1</v>
+      </c>
+      <c r="N26" s="13">
+        <v>1</v>
+      </c>
+      <c r="O26" s="11">
+        <v>0</v>
+      </c>
+      <c r="P26" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="11">
+        <v>0</v>
+      </c>
+      <c r="R26" s="11">
+        <v>0</v>
+      </c>
+      <c r="S26" s="11">
+        <v>0</v>
+      </c>
+      <c r="T26" s="12">
+        <v>0</v>
+      </c>
+      <c r="U26" s="12">
+        <v>0</v>
+      </c>
+      <c r="V26" s="12">
+        <v>1</v>
+      </c>
+      <c r="W26" s="12">
+        <v>1</v>
+      </c>
+      <c r="X26" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y26" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z26" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA26" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB26" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC26" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD26" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE26" s="12">
+        <v>1</v>
+      </c>
+      <c r="AF26" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG26" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH26" s="11">
         <v>0</v>
       </c>
       <c r="AI26" s="8" t="str">
@@ -4639,18 +4658,1906 @@
       </c>
       <c r="AJ26" s="7" t="str">
         <f t="shared" si="11"/>
-        <v>00</v>
+        <v>30</v>
       </c>
       <c r="AK26" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>00</v>
+        <v>1C</v>
       </c>
       <c r="AL26" s="5" t="str">
         <f t="shared" si="13"/>
-        <v>00</v>
+        <v>8A</v>
       </c>
       <c r="AM26" t="str">
         <f t="shared" si="14"/>
+        <v>0x00301C8A</v>
+      </c>
+    </row>
+    <row r="27" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="C27" s="3">
+        <v>0</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0</v>
+      </c>
+      <c r="E27" s="3">
+        <v>0</v>
+      </c>
+      <c r="F27" s="3">
+        <v>0</v>
+      </c>
+      <c r="G27" s="3">
+        <v>0</v>
+      </c>
+      <c r="H27" s="3">
+        <v>0</v>
+      </c>
+      <c r="I27" s="3">
+        <v>0</v>
+      </c>
+      <c r="J27" s="3">
+        <v>0</v>
+      </c>
+      <c r="K27" s="3">
+        <v>0</v>
+      </c>
+      <c r="L27" s="3">
+        <v>0</v>
+      </c>
+      <c r="M27" s="3">
+        <v>0</v>
+      </c>
+      <c r="N27" s="3">
+        <v>0</v>
+      </c>
+      <c r="O27" s="3">
+        <v>0</v>
+      </c>
+      <c r="P27" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="3">
+        <v>0</v>
+      </c>
+      <c r="R27" s="3">
+        <v>0</v>
+      </c>
+      <c r="S27" s="3">
+        <v>0</v>
+      </c>
+      <c r="T27" s="3">
+        <v>0</v>
+      </c>
+      <c r="U27" s="3">
+        <v>0</v>
+      </c>
+      <c r="V27" s="3">
+        <v>0</v>
+      </c>
+      <c r="W27" s="3">
+        <v>0</v>
+      </c>
+      <c r="X27" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC27" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE27" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF27" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG27" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH27" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI27" s="8" t="str">
+        <f t="shared" ref="AI27:AI42" si="15">BIN2HEX(_xlfn.CONCAT(C27:J27),2)</f>
+        <v>00</v>
+      </c>
+      <c r="AJ27" s="7" t="str">
+        <f t="shared" ref="AJ27:AJ42" si="16">BIN2HEX(_xlfn.CONCAT(K27:R27),2)</f>
+        <v>00</v>
+      </c>
+      <c r="AK27" s="6" t="str">
+        <f t="shared" ref="AK27:AK42" si="17">BIN2HEX(_xlfn.CONCAT(S27:Z27),2)</f>
+        <v>00</v>
+      </c>
+      <c r="AL27" s="5" t="str">
+        <f t="shared" ref="AL27:AL42" si="18">BIN2HEX(_xlfn.CONCAT(AA27:AH27),2)</f>
+        <v>00</v>
+      </c>
+      <c r="AM27" t="str">
+        <f t="shared" ref="AM27:AM42" si="19">_xlfn.CONCAT("0x",AI27:AL27)</f>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="28" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="C28" s="3">
+        <v>0</v>
+      </c>
+      <c r="D28" s="3">
+        <v>0</v>
+      </c>
+      <c r="E28" s="3">
+        <v>0</v>
+      </c>
+      <c r="F28" s="3">
+        <v>0</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0</v>
+      </c>
+      <c r="H28" s="3">
+        <v>0</v>
+      </c>
+      <c r="I28" s="3">
+        <v>0</v>
+      </c>
+      <c r="J28" s="3">
+        <v>0</v>
+      </c>
+      <c r="K28" s="3">
+        <v>0</v>
+      </c>
+      <c r="L28" s="3">
+        <v>0</v>
+      </c>
+      <c r="M28" s="3">
+        <v>0</v>
+      </c>
+      <c r="N28" s="3">
+        <v>0</v>
+      </c>
+      <c r="O28" s="3">
+        <v>0</v>
+      </c>
+      <c r="P28" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="3">
+        <v>0</v>
+      </c>
+      <c r="R28" s="3">
+        <v>0</v>
+      </c>
+      <c r="S28" s="3">
+        <v>0</v>
+      </c>
+      <c r="T28" s="3">
+        <v>0</v>
+      </c>
+      <c r="U28" s="3">
+        <v>0</v>
+      </c>
+      <c r="V28" s="3">
+        <v>0</v>
+      </c>
+      <c r="W28" s="3">
+        <v>0</v>
+      </c>
+      <c r="X28" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB28" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC28" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE28" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF28" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG28" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH28" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI28" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ28" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK28" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL28" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM28" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="29" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="C29" s="3">
+        <v>0</v>
+      </c>
+      <c r="D29" s="3">
+        <v>0</v>
+      </c>
+      <c r="E29" s="3">
+        <v>0</v>
+      </c>
+      <c r="F29" s="3">
+        <v>0</v>
+      </c>
+      <c r="G29" s="3">
+        <v>0</v>
+      </c>
+      <c r="H29" s="3">
+        <v>0</v>
+      </c>
+      <c r="I29" s="3">
+        <v>0</v>
+      </c>
+      <c r="J29" s="3">
+        <v>0</v>
+      </c>
+      <c r="K29" s="3">
+        <v>0</v>
+      </c>
+      <c r="L29" s="3">
+        <v>0</v>
+      </c>
+      <c r="M29" s="3">
+        <v>0</v>
+      </c>
+      <c r="N29" s="3">
+        <v>0</v>
+      </c>
+      <c r="O29" s="3">
+        <v>0</v>
+      </c>
+      <c r="P29" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="3">
+        <v>0</v>
+      </c>
+      <c r="R29" s="3">
+        <v>0</v>
+      </c>
+      <c r="S29" s="3">
+        <v>0</v>
+      </c>
+      <c r="T29" s="3">
+        <v>0</v>
+      </c>
+      <c r="U29" s="3">
+        <v>0</v>
+      </c>
+      <c r="V29" s="3">
+        <v>0</v>
+      </c>
+      <c r="W29" s="3">
+        <v>0</v>
+      </c>
+      <c r="X29" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI29" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ29" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK29" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL29" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM29" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="30" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="C30" s="3">
+        <v>0</v>
+      </c>
+      <c r="D30" s="3">
+        <v>0</v>
+      </c>
+      <c r="E30" s="3">
+        <v>0</v>
+      </c>
+      <c r="F30" s="3">
+        <v>0</v>
+      </c>
+      <c r="G30" s="3">
+        <v>0</v>
+      </c>
+      <c r="H30" s="3">
+        <v>0</v>
+      </c>
+      <c r="I30" s="3">
+        <v>0</v>
+      </c>
+      <c r="J30" s="3">
+        <v>0</v>
+      </c>
+      <c r="K30" s="3">
+        <v>0</v>
+      </c>
+      <c r="L30" s="3">
+        <v>0</v>
+      </c>
+      <c r="M30" s="3">
+        <v>0</v>
+      </c>
+      <c r="N30" s="3">
+        <v>0</v>
+      </c>
+      <c r="O30" s="3">
+        <v>0</v>
+      </c>
+      <c r="P30" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="3">
+        <v>0</v>
+      </c>
+      <c r="R30" s="3">
+        <v>0</v>
+      </c>
+      <c r="S30" s="3">
+        <v>0</v>
+      </c>
+      <c r="T30" s="3">
+        <v>0</v>
+      </c>
+      <c r="U30" s="3">
+        <v>0</v>
+      </c>
+      <c r="V30" s="3">
+        <v>0</v>
+      </c>
+      <c r="W30" s="3">
+        <v>0</v>
+      </c>
+      <c r="X30" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI30" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ30" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK30" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL30" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM30" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="31" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="C31" s="3">
+        <v>0</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0</v>
+      </c>
+      <c r="E31" s="3">
+        <v>0</v>
+      </c>
+      <c r="F31" s="3">
+        <v>0</v>
+      </c>
+      <c r="G31" s="3">
+        <v>0</v>
+      </c>
+      <c r="H31" s="3">
+        <v>0</v>
+      </c>
+      <c r="I31" s="3">
+        <v>0</v>
+      </c>
+      <c r="J31" s="3">
+        <v>0</v>
+      </c>
+      <c r="K31" s="3">
+        <v>0</v>
+      </c>
+      <c r="L31" s="3">
+        <v>0</v>
+      </c>
+      <c r="M31" s="3">
+        <v>0</v>
+      </c>
+      <c r="N31" s="3">
+        <v>0</v>
+      </c>
+      <c r="O31" s="3">
+        <v>0</v>
+      </c>
+      <c r="P31" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="3">
+        <v>0</v>
+      </c>
+      <c r="R31" s="3">
+        <v>0</v>
+      </c>
+      <c r="S31" s="3">
+        <v>0</v>
+      </c>
+      <c r="T31" s="3">
+        <v>0</v>
+      </c>
+      <c r="U31" s="3">
+        <v>0</v>
+      </c>
+      <c r="V31" s="3">
+        <v>0</v>
+      </c>
+      <c r="W31" s="3">
+        <v>0</v>
+      </c>
+      <c r="X31" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y31" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI31" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ31" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK31" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL31" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM31" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="32" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="C32" s="3">
+        <v>0</v>
+      </c>
+      <c r="D32" s="3">
+        <v>0</v>
+      </c>
+      <c r="E32" s="3">
+        <v>0</v>
+      </c>
+      <c r="F32" s="3">
+        <v>0</v>
+      </c>
+      <c r="G32" s="3">
+        <v>0</v>
+      </c>
+      <c r="H32" s="3">
+        <v>0</v>
+      </c>
+      <c r="I32" s="3">
+        <v>0</v>
+      </c>
+      <c r="J32" s="3">
+        <v>0</v>
+      </c>
+      <c r="K32" s="3">
+        <v>0</v>
+      </c>
+      <c r="L32" s="3">
+        <v>0</v>
+      </c>
+      <c r="M32" s="3">
+        <v>0</v>
+      </c>
+      <c r="N32" s="3">
+        <v>0</v>
+      </c>
+      <c r="O32" s="3">
+        <v>0</v>
+      </c>
+      <c r="P32" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="3">
+        <v>0</v>
+      </c>
+      <c r="R32" s="3">
+        <v>0</v>
+      </c>
+      <c r="S32" s="3">
+        <v>0</v>
+      </c>
+      <c r="T32" s="3">
+        <v>0</v>
+      </c>
+      <c r="U32" s="3">
+        <v>0</v>
+      </c>
+      <c r="V32" s="3">
+        <v>0</v>
+      </c>
+      <c r="W32" s="3">
+        <v>0</v>
+      </c>
+      <c r="X32" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y32" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z32" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA32" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB32" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC32" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD32" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE32" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF32" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG32" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH32" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI32" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ32" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK32" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL32" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM32" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="33" spans="3:39" x14ac:dyDescent="0.3">
+      <c r="C33" s="3">
+        <v>0</v>
+      </c>
+      <c r="D33" s="3">
+        <v>0</v>
+      </c>
+      <c r="E33" s="3">
+        <v>0</v>
+      </c>
+      <c r="F33" s="3">
+        <v>0</v>
+      </c>
+      <c r="G33" s="3">
+        <v>0</v>
+      </c>
+      <c r="H33" s="3">
+        <v>0</v>
+      </c>
+      <c r="I33" s="3">
+        <v>0</v>
+      </c>
+      <c r="J33" s="3">
+        <v>0</v>
+      </c>
+      <c r="K33" s="3">
+        <v>0</v>
+      </c>
+      <c r="L33" s="3">
+        <v>0</v>
+      </c>
+      <c r="M33" s="3">
+        <v>0</v>
+      </c>
+      <c r="N33" s="3">
+        <v>0</v>
+      </c>
+      <c r="O33" s="3">
+        <v>0</v>
+      </c>
+      <c r="P33" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="3">
+        <v>0</v>
+      </c>
+      <c r="R33" s="3">
+        <v>0</v>
+      </c>
+      <c r="S33" s="3">
+        <v>0</v>
+      </c>
+      <c r="T33" s="3">
+        <v>0</v>
+      </c>
+      <c r="U33" s="3">
+        <v>0</v>
+      </c>
+      <c r="V33" s="3">
+        <v>0</v>
+      </c>
+      <c r="W33" s="3">
+        <v>0</v>
+      </c>
+      <c r="X33" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y33" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI33" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ33" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK33" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL33" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM33" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="34" spans="3:39" x14ac:dyDescent="0.3">
+      <c r="C34" s="3">
+        <v>0</v>
+      </c>
+      <c r="D34" s="3">
+        <v>0</v>
+      </c>
+      <c r="E34" s="3">
+        <v>0</v>
+      </c>
+      <c r="F34" s="3">
+        <v>0</v>
+      </c>
+      <c r="G34" s="3">
+        <v>0</v>
+      </c>
+      <c r="H34" s="3">
+        <v>0</v>
+      </c>
+      <c r="I34" s="3">
+        <v>0</v>
+      </c>
+      <c r="J34" s="3">
+        <v>0</v>
+      </c>
+      <c r="K34" s="3">
+        <v>0</v>
+      </c>
+      <c r="L34" s="3">
+        <v>0</v>
+      </c>
+      <c r="M34" s="3">
+        <v>0</v>
+      </c>
+      <c r="N34" s="3">
+        <v>0</v>
+      </c>
+      <c r="O34" s="3">
+        <v>0</v>
+      </c>
+      <c r="P34" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="3">
+        <v>0</v>
+      </c>
+      <c r="R34" s="3">
+        <v>0</v>
+      </c>
+      <c r="S34" s="3">
+        <v>0</v>
+      </c>
+      <c r="T34" s="3">
+        <v>0</v>
+      </c>
+      <c r="U34" s="3">
+        <v>0</v>
+      </c>
+      <c r="V34" s="3">
+        <v>0</v>
+      </c>
+      <c r="W34" s="3">
+        <v>0</v>
+      </c>
+      <c r="X34" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y34" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI34" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ34" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK34" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL34" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM34" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="35" spans="3:39" x14ac:dyDescent="0.3">
+      <c r="C35" s="3">
+        <v>0</v>
+      </c>
+      <c r="D35" s="3">
+        <v>0</v>
+      </c>
+      <c r="E35" s="3">
+        <v>0</v>
+      </c>
+      <c r="F35" s="3">
+        <v>0</v>
+      </c>
+      <c r="G35" s="3">
+        <v>0</v>
+      </c>
+      <c r="H35" s="3">
+        <v>0</v>
+      </c>
+      <c r="I35" s="3">
+        <v>0</v>
+      </c>
+      <c r="J35" s="3">
+        <v>0</v>
+      </c>
+      <c r="K35" s="3">
+        <v>0</v>
+      </c>
+      <c r="L35" s="3">
+        <v>0</v>
+      </c>
+      <c r="M35" s="3">
+        <v>0</v>
+      </c>
+      <c r="N35" s="3">
+        <v>0</v>
+      </c>
+      <c r="O35" s="3">
+        <v>0</v>
+      </c>
+      <c r="P35" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="3">
+        <v>0</v>
+      </c>
+      <c r="R35" s="3">
+        <v>0</v>
+      </c>
+      <c r="S35" s="3">
+        <v>0</v>
+      </c>
+      <c r="T35" s="3">
+        <v>0</v>
+      </c>
+      <c r="U35" s="3">
+        <v>0</v>
+      </c>
+      <c r="V35" s="3">
+        <v>0</v>
+      </c>
+      <c r="W35" s="3">
+        <v>0</v>
+      </c>
+      <c r="X35" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI35" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ35" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK35" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL35" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM35" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="36" spans="3:39" x14ac:dyDescent="0.3">
+      <c r="C36" s="3">
+        <v>0</v>
+      </c>
+      <c r="D36" s="3">
+        <v>0</v>
+      </c>
+      <c r="E36" s="3">
+        <v>0</v>
+      </c>
+      <c r="F36" s="3">
+        <v>0</v>
+      </c>
+      <c r="G36" s="3">
+        <v>0</v>
+      </c>
+      <c r="H36" s="3">
+        <v>0</v>
+      </c>
+      <c r="I36" s="3">
+        <v>0</v>
+      </c>
+      <c r="J36" s="3">
+        <v>0</v>
+      </c>
+      <c r="K36" s="3">
+        <v>0</v>
+      </c>
+      <c r="L36" s="3">
+        <v>0</v>
+      </c>
+      <c r="M36" s="3">
+        <v>0</v>
+      </c>
+      <c r="N36" s="3">
+        <v>0</v>
+      </c>
+      <c r="O36" s="3">
+        <v>0</v>
+      </c>
+      <c r="P36" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="3">
+        <v>0</v>
+      </c>
+      <c r="R36" s="3">
+        <v>0</v>
+      </c>
+      <c r="S36" s="3">
+        <v>0</v>
+      </c>
+      <c r="T36" s="3">
+        <v>0</v>
+      </c>
+      <c r="U36" s="3">
+        <v>0</v>
+      </c>
+      <c r="V36" s="3">
+        <v>0</v>
+      </c>
+      <c r="W36" s="3">
+        <v>0</v>
+      </c>
+      <c r="X36" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y36" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI36" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ36" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK36" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL36" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM36" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="37" spans="3:39" x14ac:dyDescent="0.3">
+      <c r="C37" s="3">
+        <v>0</v>
+      </c>
+      <c r="D37" s="3">
+        <v>0</v>
+      </c>
+      <c r="E37" s="3">
+        <v>0</v>
+      </c>
+      <c r="F37" s="3">
+        <v>0</v>
+      </c>
+      <c r="G37" s="3">
+        <v>0</v>
+      </c>
+      <c r="H37" s="3">
+        <v>0</v>
+      </c>
+      <c r="I37" s="3">
+        <v>0</v>
+      </c>
+      <c r="J37" s="3">
+        <v>0</v>
+      </c>
+      <c r="K37" s="3">
+        <v>0</v>
+      </c>
+      <c r="L37" s="3">
+        <v>0</v>
+      </c>
+      <c r="M37" s="3">
+        <v>0</v>
+      </c>
+      <c r="N37" s="3">
+        <v>0</v>
+      </c>
+      <c r="O37" s="3">
+        <v>0</v>
+      </c>
+      <c r="P37" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="3">
+        <v>0</v>
+      </c>
+      <c r="R37" s="3">
+        <v>0</v>
+      </c>
+      <c r="S37" s="3">
+        <v>0</v>
+      </c>
+      <c r="T37" s="3">
+        <v>0</v>
+      </c>
+      <c r="U37" s="3">
+        <v>0</v>
+      </c>
+      <c r="V37" s="3">
+        <v>0</v>
+      </c>
+      <c r="W37" s="3">
+        <v>0</v>
+      </c>
+      <c r="X37" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y37" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI37" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ37" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK37" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL37" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM37" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="38" spans="3:39" x14ac:dyDescent="0.3">
+      <c r="C38" s="3">
+        <v>0</v>
+      </c>
+      <c r="D38" s="3">
+        <v>0</v>
+      </c>
+      <c r="E38" s="3">
+        <v>0</v>
+      </c>
+      <c r="F38" s="3">
+        <v>0</v>
+      </c>
+      <c r="G38" s="3">
+        <v>0</v>
+      </c>
+      <c r="H38" s="3">
+        <v>0</v>
+      </c>
+      <c r="I38" s="3">
+        <v>0</v>
+      </c>
+      <c r="J38" s="3">
+        <v>0</v>
+      </c>
+      <c r="K38" s="3">
+        <v>0</v>
+      </c>
+      <c r="L38" s="3">
+        <v>0</v>
+      </c>
+      <c r="M38" s="3">
+        <v>0</v>
+      </c>
+      <c r="N38" s="3">
+        <v>0</v>
+      </c>
+      <c r="O38" s="3">
+        <v>0</v>
+      </c>
+      <c r="P38" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="3">
+        <v>0</v>
+      </c>
+      <c r="R38" s="3">
+        <v>0</v>
+      </c>
+      <c r="S38" s="3">
+        <v>0</v>
+      </c>
+      <c r="T38" s="3">
+        <v>0</v>
+      </c>
+      <c r="U38" s="3">
+        <v>0</v>
+      </c>
+      <c r="V38" s="3">
+        <v>0</v>
+      </c>
+      <c r="W38" s="3">
+        <v>0</v>
+      </c>
+      <c r="X38" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y38" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z38" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA38" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB38" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC38" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD38" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE38" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF38" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG38" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH38" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI38" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ38" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK38" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL38" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM38" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="39" spans="3:39" x14ac:dyDescent="0.3">
+      <c r="C39" s="3">
+        <v>0</v>
+      </c>
+      <c r="D39" s="3">
+        <v>0</v>
+      </c>
+      <c r="E39" s="3">
+        <v>0</v>
+      </c>
+      <c r="F39" s="3">
+        <v>0</v>
+      </c>
+      <c r="G39" s="3">
+        <v>0</v>
+      </c>
+      <c r="H39" s="3">
+        <v>0</v>
+      </c>
+      <c r="I39" s="3">
+        <v>0</v>
+      </c>
+      <c r="J39" s="3">
+        <v>0</v>
+      </c>
+      <c r="K39" s="3">
+        <v>0</v>
+      </c>
+      <c r="L39" s="3">
+        <v>0</v>
+      </c>
+      <c r="M39" s="3">
+        <v>0</v>
+      </c>
+      <c r="N39" s="3">
+        <v>0</v>
+      </c>
+      <c r="O39" s="3">
+        <v>0</v>
+      </c>
+      <c r="P39" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="3">
+        <v>0</v>
+      </c>
+      <c r="R39" s="3">
+        <v>0</v>
+      </c>
+      <c r="S39" s="3">
+        <v>0</v>
+      </c>
+      <c r="T39" s="3">
+        <v>0</v>
+      </c>
+      <c r="U39" s="3">
+        <v>0</v>
+      </c>
+      <c r="V39" s="3">
+        <v>0</v>
+      </c>
+      <c r="W39" s="3">
+        <v>0</v>
+      </c>
+      <c r="X39" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y39" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI39" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ39" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK39" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL39" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM39" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="40" spans="3:39" x14ac:dyDescent="0.3">
+      <c r="C40" s="3">
+        <v>0</v>
+      </c>
+      <c r="D40" s="3">
+        <v>0</v>
+      </c>
+      <c r="E40" s="3">
+        <v>0</v>
+      </c>
+      <c r="F40" s="3">
+        <v>0</v>
+      </c>
+      <c r="G40" s="3">
+        <v>0</v>
+      </c>
+      <c r="H40" s="3">
+        <v>0</v>
+      </c>
+      <c r="I40" s="3">
+        <v>0</v>
+      </c>
+      <c r="J40" s="3">
+        <v>0</v>
+      </c>
+      <c r="K40" s="3">
+        <v>0</v>
+      </c>
+      <c r="L40" s="3">
+        <v>0</v>
+      </c>
+      <c r="M40" s="3">
+        <v>0</v>
+      </c>
+      <c r="N40" s="3">
+        <v>0</v>
+      </c>
+      <c r="O40" s="3">
+        <v>0</v>
+      </c>
+      <c r="P40" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="3">
+        <v>0</v>
+      </c>
+      <c r="R40" s="3">
+        <v>0</v>
+      </c>
+      <c r="S40" s="3">
+        <v>0</v>
+      </c>
+      <c r="T40" s="3">
+        <v>0</v>
+      </c>
+      <c r="U40" s="3">
+        <v>0</v>
+      </c>
+      <c r="V40" s="3">
+        <v>0</v>
+      </c>
+      <c r="W40" s="3">
+        <v>0</v>
+      </c>
+      <c r="X40" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y40" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI40" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ40" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK40" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL40" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM40" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="41" spans="3:39" x14ac:dyDescent="0.3">
+      <c r="C41" s="3">
+        <v>0</v>
+      </c>
+      <c r="D41" s="3">
+        <v>0</v>
+      </c>
+      <c r="E41" s="3">
+        <v>0</v>
+      </c>
+      <c r="F41" s="3">
+        <v>0</v>
+      </c>
+      <c r="G41" s="3">
+        <v>0</v>
+      </c>
+      <c r="H41" s="3">
+        <v>0</v>
+      </c>
+      <c r="I41" s="3">
+        <v>0</v>
+      </c>
+      <c r="J41" s="3">
+        <v>0</v>
+      </c>
+      <c r="K41" s="3">
+        <v>0</v>
+      </c>
+      <c r="L41" s="3">
+        <v>0</v>
+      </c>
+      <c r="M41" s="3">
+        <v>0</v>
+      </c>
+      <c r="N41" s="3">
+        <v>0</v>
+      </c>
+      <c r="O41" s="3">
+        <v>0</v>
+      </c>
+      <c r="P41" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="3">
+        <v>0</v>
+      </c>
+      <c r="R41" s="3">
+        <v>0</v>
+      </c>
+      <c r="S41" s="3">
+        <v>0</v>
+      </c>
+      <c r="T41" s="3">
+        <v>0</v>
+      </c>
+      <c r="U41" s="3">
+        <v>0</v>
+      </c>
+      <c r="V41" s="3">
+        <v>0</v>
+      </c>
+      <c r="W41" s="3">
+        <v>0</v>
+      </c>
+      <c r="X41" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y41" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z41" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA41" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB41" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC41" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD41" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE41" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF41" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG41" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH41" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI41" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ41" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK41" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL41" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM41" t="str">
+        <f t="shared" si="19"/>
+        <v>0x00000000</v>
+      </c>
+    </row>
+    <row r="42" spans="3:39" x14ac:dyDescent="0.3">
+      <c r="C42" s="3">
+        <v>0</v>
+      </c>
+      <c r="D42" s="3">
+        <v>0</v>
+      </c>
+      <c r="E42" s="3">
+        <v>0</v>
+      </c>
+      <c r="F42" s="3">
+        <v>0</v>
+      </c>
+      <c r="G42" s="3">
+        <v>0</v>
+      </c>
+      <c r="H42" s="3">
+        <v>0</v>
+      </c>
+      <c r="I42" s="3">
+        <v>0</v>
+      </c>
+      <c r="J42" s="3">
+        <v>0</v>
+      </c>
+      <c r="K42" s="3">
+        <v>0</v>
+      </c>
+      <c r="L42" s="3">
+        <v>0</v>
+      </c>
+      <c r="M42" s="3">
+        <v>0</v>
+      </c>
+      <c r="N42" s="3">
+        <v>0</v>
+      </c>
+      <c r="O42" s="3">
+        <v>0</v>
+      </c>
+      <c r="P42" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="3">
+        <v>0</v>
+      </c>
+      <c r="R42" s="3">
+        <v>0</v>
+      </c>
+      <c r="S42" s="3">
+        <v>0</v>
+      </c>
+      <c r="T42" s="3">
+        <v>0</v>
+      </c>
+      <c r="U42" s="3">
+        <v>0</v>
+      </c>
+      <c r="V42" s="3">
+        <v>0</v>
+      </c>
+      <c r="W42" s="3">
+        <v>0</v>
+      </c>
+      <c r="X42" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y42" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI42" s="8" t="str">
+        <f t="shared" si="15"/>
+        <v>00</v>
+      </c>
+      <c r="AJ42" s="7" t="str">
+        <f t="shared" si="16"/>
+        <v>00</v>
+      </c>
+      <c r="AK42" s="6" t="str">
+        <f t="shared" si="17"/>
+        <v>00</v>
+      </c>
+      <c r="AL42" s="5" t="str">
+        <f t="shared" si="18"/>
+        <v>00</v>
+      </c>
+      <c r="AM42" t="str">
+        <f t="shared" si="19"/>
         <v>0x00000000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(sv): instrucciones tipo I,R y B funcionales con adelantamiento
Bugs: tipo M(tanto load como store) no adelantan o reciben el adelantamiento adecuado
</commit_message>
<xml_diff>
--- a/res/isa.xlsx
+++ b/res/isa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\workbench\repos\CE4301--p2_fobando_isa--\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D8C9AE-62C3-4E28-9AD6-44C33E04427F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5DE0785-EBA1-4E1E-A31D-F681FC777E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{EC7525CD-E51C-4E61-B306-9CBCE090E85A}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="67">
   <si>
     <t>R</t>
   </si>
@@ -156,9 +156,6 @@
     <t>muli pc, ra, 7</t>
   </si>
   <si>
-    <t>bge r5, r7, -4</t>
-  </si>
-  <si>
     <t>jal ra, 4</t>
   </si>
   <si>
@@ -213,7 +210,37 @@
     <t>muli p2, p1, -1</t>
   </si>
   <si>
-    <t>stb p2,+ 3(zero)</t>
+    <t>sth p2,+ 3(zero)</t>
+  </si>
+  <si>
+    <t>movi r0, 5</t>
+  </si>
+  <si>
+    <t>movi r2, 2</t>
+  </si>
+  <si>
+    <t>addi r1, r1, 1</t>
+  </si>
+  <si>
+    <t>bne r1, r0, -3</t>
+  </si>
+  <si>
+    <t>stw r2,+ 4(zero)</t>
+  </si>
+  <si>
+    <t>stb r1,- -2(zero)</t>
+  </si>
+  <si>
+    <t>mov r1, zero</t>
+  </si>
+  <si>
+    <t>blt r5, r7, -4</t>
+  </si>
+  <si>
+    <t>addi r3, r1, 1</t>
+  </si>
+  <si>
+    <t>mul r3, r3, r2</t>
   </si>
 </sst>
 </file>
@@ -506,6 +533,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -531,15 +567,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -990,49 +1017,49 @@
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="24" t="s">
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="24" t="s">
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="17"/>
+      <c r="N3" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="O3" s="25"/>
-      <c r="P3" s="25"/>
-      <c r="Q3" s="25"/>
-      <c r="R3" s="26"/>
-      <c r="S3" s="24" t="s">
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="17"/>
+      <c r="S3" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="T3" s="25"/>
-      <c r="U3" s="25"/>
-      <c r="V3" s="25"/>
-      <c r="W3" s="26"/>
-      <c r="X3" s="24" t="s">
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
+      <c r="V3" s="16"/>
+      <c r="W3" s="17"/>
+      <c r="X3" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="Y3" s="25"/>
-      <c r="Z3" s="25"/>
-      <c r="AA3" s="26"/>
-      <c r="AB3" s="24" t="s">
+      <c r="Y3" s="16"/>
+      <c r="Z3" s="16"/>
+      <c r="AA3" s="17"/>
+      <c r="AB3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC3" s="25"/>
-      <c r="AD3" s="25"/>
-      <c r="AE3" s="25"/>
-      <c r="AF3" s="26"/>
+      <c r="AC3" s="16"/>
+      <c r="AD3" s="16"/>
+      <c r="AE3" s="16"/>
+      <c r="AF3" s="17"/>
       <c r="AG3" s="3" t="s">
         <v>16</v>
       </c>
@@ -1041,47 +1068,47 @@
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
-      <c r="J4" s="25"/>
-      <c r="K4" s="25"/>
-      <c r="L4" s="25"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="24" t="s">
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="17"/>
+      <c r="N4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="O4" s="25"/>
-      <c r="P4" s="25"/>
-      <c r="Q4" s="25"/>
-      <c r="R4" s="26"/>
-      <c r="S4" s="24" t="s">
+      <c r="O4" s="16"/>
+      <c r="P4" s="16"/>
+      <c r="Q4" s="16"/>
+      <c r="R4" s="17"/>
+      <c r="S4" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="T4" s="25"/>
-      <c r="U4" s="25"/>
-      <c r="V4" s="25"/>
-      <c r="W4" s="26"/>
-      <c r="X4" s="24" t="s">
+      <c r="T4" s="16"/>
+      <c r="U4" s="16"/>
+      <c r="V4" s="16"/>
+      <c r="W4" s="17"/>
+      <c r="X4" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="Y4" s="25"/>
-      <c r="Z4" s="25"/>
-      <c r="AA4" s="26"/>
-      <c r="AB4" s="24" t="s">
+      <c r="Y4" s="16"/>
+      <c r="Z4" s="16"/>
+      <c r="AA4" s="17"/>
+      <c r="AB4" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC4" s="25"/>
-      <c r="AD4" s="25"/>
-      <c r="AE4" s="25"/>
-      <c r="AF4" s="26"/>
+      <c r="AC4" s="16"/>
+      <c r="AD4" s="16"/>
+      <c r="AE4" s="16"/>
+      <c r="AF4" s="17"/>
       <c r="AG4" s="3" t="s">
         <v>16</v>
       </c>
@@ -1090,34 +1117,34 @@
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-      <c r="K5" s="25"/>
-      <c r="L5" s="25"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="24" t="s">
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="17"/>
+      <c r="N5" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="O5" s="25"/>
-      <c r="P5" s="25"/>
-      <c r="Q5" s="25"/>
-      <c r="R5" s="26"/>
-      <c r="S5" s="24" t="s">
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
+      <c r="Q5" s="16"/>
+      <c r="R5" s="17"/>
+      <c r="S5" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="T5" s="25"/>
-      <c r="U5" s="25"/>
-      <c r="V5" s="25"/>
-      <c r="W5" s="26"/>
+      <c r="T5" s="16"/>
+      <c r="U5" s="16"/>
+      <c r="V5" s="16"/>
+      <c r="W5" s="17"/>
       <c r="X5" s="3" t="s">
         <v>19</v>
       </c>
@@ -1130,13 +1157,13 @@
       <c r="AA5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AB5" s="24" t="s">
+      <c r="AB5" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC5" s="25"/>
-      <c r="AD5" s="25"/>
-      <c r="AE5" s="25"/>
-      <c r="AF5" s="26"/>
+      <c r="AC5" s="16"/>
+      <c r="AD5" s="16"/>
+      <c r="AE5" s="16"/>
+      <c r="AF5" s="17"/>
       <c r="AG5" s="3" t="s">
         <v>16</v>
       </c>
@@ -1145,49 +1172,49 @@
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="24" t="s">
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="25"/>
-      <c r="K6" s="25"/>
-      <c r="L6" s="25"/>
-      <c r="M6" s="26"/>
-      <c r="N6" s="24" t="s">
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="O6" s="25"/>
-      <c r="P6" s="25"/>
-      <c r="Q6" s="25"/>
-      <c r="R6" s="26"/>
-      <c r="S6" s="24" t="s">
+      <c r="O6" s="16"/>
+      <c r="P6" s="16"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="T6" s="25"/>
-      <c r="U6" s="25"/>
-      <c r="V6" s="25"/>
-      <c r="W6" s="26"/>
-      <c r="X6" s="24" t="s">
+      <c r="T6" s="16"/>
+      <c r="U6" s="16"/>
+      <c r="V6" s="16"/>
+      <c r="W6" s="17"/>
+      <c r="X6" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="Y6" s="25"/>
-      <c r="Z6" s="25"/>
-      <c r="AA6" s="26"/>
-      <c r="AB6" s="24" t="s">
+      <c r="Y6" s="16"/>
+      <c r="Z6" s="16"/>
+      <c r="AA6" s="17"/>
+      <c r="AB6" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC6" s="25"/>
-      <c r="AD6" s="25"/>
-      <c r="AE6" s="25"/>
-      <c r="AF6" s="26"/>
+      <c r="AC6" s="16"/>
+      <c r="AD6" s="16"/>
+      <c r="AE6" s="16"/>
+      <c r="AF6" s="17"/>
       <c r="AG6" s="3" t="s">
         <v>16</v>
       </c>
@@ -1196,45 +1223,45 @@
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="25"/>
-      <c r="L7" s="25"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="25"/>
-      <c r="Q7" s="25"/>
-      <c r="R7" s="26"/>
-      <c r="S7" s="24" t="s">
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="17"/>
+      <c r="S7" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="T7" s="25"/>
-      <c r="U7" s="25"/>
-      <c r="V7" s="25"/>
-      <c r="W7" s="26"/>
-      <c r="X7" s="24" t="s">
+      <c r="T7" s="16"/>
+      <c r="U7" s="16"/>
+      <c r="V7" s="16"/>
+      <c r="W7" s="17"/>
+      <c r="X7" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="Y7" s="25"/>
-      <c r="Z7" s="25"/>
-      <c r="AA7" s="26"/>
-      <c r="AB7" s="24" t="s">
+      <c r="Y7" s="16"/>
+      <c r="Z7" s="16"/>
+      <c r="AA7" s="17"/>
+      <c r="AB7" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC7" s="25"/>
-      <c r="AD7" s="25"/>
-      <c r="AE7" s="25"/>
-      <c r="AF7" s="26"/>
+      <c r="AC7" s="16"/>
+      <c r="AD7" s="16"/>
+      <c r="AE7" s="16"/>
+      <c r="AF7" s="17"/>
       <c r="AG7" s="3" t="s">
         <v>16</v>
       </c>
@@ -1243,47 +1270,47 @@
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
-      <c r="J8" s="25"/>
-      <c r="K8" s="25"/>
-      <c r="L8" s="25"/>
-      <c r="M8" s="25"/>
-      <c r="N8" s="25"/>
-      <c r="O8" s="25"/>
-      <c r="P8" s="25"/>
-      <c r="Q8" s="25"/>
-      <c r="R8" s="25"/>
-      <c r="S8" s="25"/>
-      <c r="T8" s="25"/>
-      <c r="U8" s="26"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="16"/>
+      <c r="P8" s="16"/>
+      <c r="Q8" s="16"/>
+      <c r="R8" s="16"/>
+      <c r="S8" s="16"/>
+      <c r="T8" s="16"/>
+      <c r="U8" s="17"/>
       <c r="V8" s="3">
         <v>0</v>
       </c>
       <c r="W8" s="3">
         <v>0</v>
       </c>
-      <c r="X8" s="24" t="s">
+      <c r="X8" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="Y8" s="25"/>
-      <c r="Z8" s="25"/>
-      <c r="AA8" s="26"/>
-      <c r="AB8" s="24" t="s">
+      <c r="Y8" s="16"/>
+      <c r="Z8" s="16"/>
+      <c r="AA8" s="17"/>
+      <c r="AB8" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC8" s="25"/>
-      <c r="AD8" s="25"/>
-      <c r="AE8" s="25"/>
-      <c r="AF8" s="26"/>
+      <c r="AC8" s="16"/>
+      <c r="AD8" s="16"/>
+      <c r="AE8" s="16"/>
+      <c r="AF8" s="17"/>
       <c r="AG8" s="3" t="s">
         <v>16</v>
       </c>
@@ -1292,34 +1319,34 @@
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
-      <c r="J9" s="25"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25"/>
-      <c r="M9" s="25"/>
-      <c r="N9" s="25"/>
-      <c r="O9" s="25"/>
-      <c r="P9" s="25"/>
-      <c r="Q9" s="26"/>
-      <c r="R9" s="24" t="s">
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="S9" s="25"/>
-      <c r="T9" s="26"/>
-      <c r="U9" s="24" t="s">
+      <c r="S9" s="16"/>
+      <c r="T9" s="17"/>
+      <c r="U9" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="V9" s="25"/>
-      <c r="W9" s="26"/>
+      <c r="V9" s="16"/>
+      <c r="W9" s="17"/>
       <c r="X9" s="3" t="s">
         <v>19</v>
       </c>
@@ -1332,13 +1359,13 @@
       <c r="AA9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="AB9" s="24" t="s">
+      <c r="AB9" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC9" s="25"/>
-      <c r="AD9" s="25"/>
-      <c r="AE9" s="25"/>
-      <c r="AF9" s="26"/>
+      <c r="AC9" s="16"/>
+      <c r="AD9" s="16"/>
+      <c r="AE9" s="16"/>
+      <c r="AF9" s="17"/>
       <c r="AG9" s="3" t="s">
         <v>16</v>
       </c>
@@ -1347,53 +1374,53 @@
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="24" t="s">
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="J10" s="25"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="24" t="s">
+      <c r="J10" s="16"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="M10" s="25"/>
-      <c r="N10" s="26"/>
-      <c r="O10" s="24" t="s">
+      <c r="M10" s="16"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="P10" s="25"/>
-      <c r="Q10" s="26"/>
-      <c r="R10" s="24" t="s">
+      <c r="P10" s="16"/>
+      <c r="Q10" s="17"/>
+      <c r="R10" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="S10" s="25"/>
-      <c r="T10" s="26"/>
-      <c r="U10" s="24" t="s">
+      <c r="S10" s="16"/>
+      <c r="T10" s="17"/>
+      <c r="U10" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="V10" s="25"/>
-      <c r="W10" s="26"/>
-      <c r="X10" s="24" t="s">
+      <c r="V10" s="16"/>
+      <c r="W10" s="17"/>
+      <c r="X10" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="Y10" s="25"/>
-      <c r="Z10" s="25"/>
-      <c r="AA10" s="26"/>
-      <c r="AB10" s="24" t="s">
+      <c r="Y10" s="16"/>
+      <c r="Z10" s="16"/>
+      <c r="AA10" s="17"/>
+      <c r="AB10" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC10" s="25"/>
-      <c r="AD10" s="25"/>
-      <c r="AE10" s="25"/>
-      <c r="AF10" s="26"/>
+      <c r="AC10" s="16"/>
+      <c r="AD10" s="16"/>
+      <c r="AE10" s="16"/>
+      <c r="AF10" s="17"/>
       <c r="AG10" s="3" t="s">
         <v>16</v>
       </c>
@@ -1402,53 +1429,53 @@
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
-      <c r="M11" s="25"/>
-      <c r="N11" s="25"/>
-      <c r="O11" s="25"/>
-      <c r="P11" s="25"/>
-      <c r="Q11" s="26"/>
-      <c r="R11" s="24" t="s">
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="16"/>
+      <c r="N11" s="16"/>
+      <c r="O11" s="16"/>
+      <c r="P11" s="16"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="S11" s="25"/>
-      <c r="T11" s="26"/>
-      <c r="U11" s="24" t="s">
+      <c r="S11" s="16"/>
+      <c r="T11" s="17"/>
+      <c r="U11" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="V11" s="25"/>
-      <c r="W11" s="26"/>
-      <c r="X11" s="24" t="s">
+      <c r="V11" s="16"/>
+      <c r="W11" s="17"/>
+      <c r="X11" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="Y11" s="25"/>
-      <c r="Z11" s="25"/>
-      <c r="AA11" s="26"/>
-      <c r="AB11" s="24" t="s">
+      <c r="Y11" s="16"/>
+      <c r="Z11" s="16"/>
+      <c r="AA11" s="17"/>
+      <c r="AB11" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="AC11" s="25"/>
-      <c r="AD11" s="25"/>
-      <c r="AE11" s="25"/>
-      <c r="AF11" s="26"/>
+      <c r="AC11" s="16"/>
+      <c r="AD11" s="16"/>
+      <c r="AE11" s="16"/>
+      <c r="AF11" s="17"/>
       <c r="AG11" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="18" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="3">
@@ -1487,43 +1514,43 @@
       <c r="M12" s="3">
         <v>0</v>
       </c>
-      <c r="N12" s="24" t="s">
+      <c r="N12" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="O12" s="25"/>
-      <c r="P12" s="25"/>
-      <c r="Q12" s="25"/>
-      <c r="R12" s="26"/>
+      <c r="O12" s="16"/>
+      <c r="P12" s="16"/>
+      <c r="Q12" s="16"/>
+      <c r="R12" s="17"/>
       <c r="S12" s="3">
         <v>0</v>
       </c>
       <c r="T12" s="3">
         <v>0</v>
       </c>
-      <c r="U12" s="24" t="s">
+      <c r="U12" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="V12" s="25"/>
-      <c r="W12" s="26"/>
-      <c r="X12" s="16" t="s">
+      <c r="V12" s="16"/>
+      <c r="W12" s="17"/>
+      <c r="X12" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="Y12" s="17"/>
-      <c r="Z12" s="17"/>
-      <c r="AA12" s="18"/>
-      <c r="AB12" s="16" t="s">
+      <c r="Y12" s="20"/>
+      <c r="Z12" s="20"/>
+      <c r="AA12" s="21"/>
+      <c r="AB12" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="AC12" s="17"/>
-      <c r="AD12" s="17"/>
-      <c r="AE12" s="17"/>
-      <c r="AF12" s="18"/>
-      <c r="AG12" s="22" t="s">
+      <c r="AC12" s="20"/>
+      <c r="AD12" s="20"/>
+      <c r="AE12" s="20"/>
+      <c r="AF12" s="21"/>
+      <c r="AG12" s="25" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A13" s="15"/>
+      <c r="A13" s="18"/>
       <c r="B13" s="3">
         <v>0</v>
       </c>
@@ -1563,62 +1590,50 @@
       <c r="N13" s="3">
         <v>0</v>
       </c>
-      <c r="O13" s="24" t="s">
+      <c r="O13" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="P13" s="25"/>
-      <c r="Q13" s="26"/>
+      <c r="P13" s="16"/>
+      <c r="Q13" s="17"/>
       <c r="R13" s="9">
         <v>0</v>
       </c>
-      <c r="S13" s="24" t="s">
+      <c r="S13" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="T13" s="25"/>
-      <c r="U13" s="25"/>
-      <c r="V13" s="25"/>
-      <c r="W13" s="26"/>
-      <c r="X13" s="19"/>
-      <c r="Y13" s="20"/>
-      <c r="Z13" s="20"/>
-      <c r="AA13" s="21"/>
-      <c r="AB13" s="19"/>
-      <c r="AC13" s="20"/>
-      <c r="AD13" s="20"/>
-      <c r="AE13" s="20"/>
-      <c r="AF13" s="21"/>
-      <c r="AG13" s="23"/>
+      <c r="T13" s="16"/>
+      <c r="U13" s="16"/>
+      <c r="V13" s="16"/>
+      <c r="W13" s="17"/>
+      <c r="X13" s="22"/>
+      <c r="Y13" s="23"/>
+      <c r="Z13" s="23"/>
+      <c r="AA13" s="24"/>
+      <c r="AB13" s="22"/>
+      <c r="AC13" s="23"/>
+      <c r="AD13" s="23"/>
+      <c r="AE13" s="23"/>
+      <c r="AF13" s="24"/>
+      <c r="AG13" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="AB3:AF3"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="N3:R3"/>
-    <mergeCell ref="S3:W3"/>
-    <mergeCell ref="X3:AA3"/>
-    <mergeCell ref="AB4:AF4"/>
-    <mergeCell ref="B5:M5"/>
-    <mergeCell ref="N5:R5"/>
-    <mergeCell ref="S5:W5"/>
-    <mergeCell ref="AB5:AF5"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B4:M4"/>
-    <mergeCell ref="N4:R4"/>
-    <mergeCell ref="S4:W4"/>
-    <mergeCell ref="X4:AA4"/>
-    <mergeCell ref="AB6:AF6"/>
-    <mergeCell ref="X6:AA6"/>
-    <mergeCell ref="I6:M6"/>
-    <mergeCell ref="N6:R6"/>
-    <mergeCell ref="S6:W6"/>
-    <mergeCell ref="AB7:AF7"/>
-    <mergeCell ref="X7:AA7"/>
-    <mergeCell ref="S7:W7"/>
-    <mergeCell ref="B7:R7"/>
-    <mergeCell ref="X8:AA8"/>
-    <mergeCell ref="AB8:AF8"/>
-    <mergeCell ref="B8:U8"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="X12:AA13"/>
+    <mergeCell ref="AB12:AF13"/>
+    <mergeCell ref="AG12:AG13"/>
+    <mergeCell ref="S13:W13"/>
+    <mergeCell ref="O13:Q13"/>
+    <mergeCell ref="B11:Q11"/>
+    <mergeCell ref="U12:W12"/>
+    <mergeCell ref="N12:R12"/>
+    <mergeCell ref="R11:T11"/>
+    <mergeCell ref="U11:W11"/>
+    <mergeCell ref="X11:AA11"/>
+    <mergeCell ref="AB11:AF11"/>
+    <mergeCell ref="AB9:AF9"/>
+    <mergeCell ref="U9:W9"/>
+    <mergeCell ref="R9:T9"/>
     <mergeCell ref="B9:Q9"/>
     <mergeCell ref="X10:AA10"/>
     <mergeCell ref="AB10:AF10"/>
@@ -1628,22 +1643,34 @@
     <mergeCell ref="I10:K10"/>
     <mergeCell ref="B10:H10"/>
     <mergeCell ref="L10:N10"/>
-    <mergeCell ref="X11:AA11"/>
-    <mergeCell ref="AB11:AF11"/>
-    <mergeCell ref="AB9:AF9"/>
-    <mergeCell ref="U9:W9"/>
-    <mergeCell ref="R9:T9"/>
-    <mergeCell ref="B11:Q11"/>
-    <mergeCell ref="U12:W12"/>
-    <mergeCell ref="N12:R12"/>
-    <mergeCell ref="R11:T11"/>
-    <mergeCell ref="U11:W11"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="X12:AA13"/>
-    <mergeCell ref="AB12:AF13"/>
-    <mergeCell ref="AG12:AG13"/>
-    <mergeCell ref="S13:W13"/>
-    <mergeCell ref="O13:Q13"/>
+    <mergeCell ref="AB7:AF7"/>
+    <mergeCell ref="X7:AA7"/>
+    <mergeCell ref="S7:W7"/>
+    <mergeCell ref="B7:R7"/>
+    <mergeCell ref="X8:AA8"/>
+    <mergeCell ref="AB8:AF8"/>
+    <mergeCell ref="B8:U8"/>
+    <mergeCell ref="AB6:AF6"/>
+    <mergeCell ref="X6:AA6"/>
+    <mergeCell ref="I6:M6"/>
+    <mergeCell ref="N6:R6"/>
+    <mergeCell ref="S6:W6"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="N4:R4"/>
+    <mergeCell ref="S4:W4"/>
+    <mergeCell ref="X4:AA4"/>
+    <mergeCell ref="AB4:AF4"/>
+    <mergeCell ref="B5:M5"/>
+    <mergeCell ref="N5:R5"/>
+    <mergeCell ref="S5:W5"/>
+    <mergeCell ref="AB5:AF5"/>
+    <mergeCell ref="AB3:AF3"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="N3:R3"/>
+    <mergeCell ref="S3:W3"/>
+    <mergeCell ref="X3:AA3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2136,7 +2163,7 @@
     </row>
     <row r="6" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
-        <v>38</v>
+        <v>64</v>
       </c>
       <c r="C6" s="13">
         <v>1</v>
@@ -2257,7 +2284,7 @@
     </row>
     <row r="7" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C7" s="13">
         <v>0</v>
@@ -2378,7 +2405,7 @@
     </row>
     <row r="8" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C8" s="13">
         <v>0</v>
@@ -2499,7 +2526,7 @@
     </row>
     <row r="9" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C9" s="13">
         <v>0</v>
@@ -2620,7 +2647,7 @@
     </row>
     <row r="10" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" s="13">
         <v>1</v>
@@ -2741,7 +2768,7 @@
     </row>
     <row r="11" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C11" s="13">
         <v>0</v>
@@ -2862,7 +2889,7 @@
     </row>
     <row r="12" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B12" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C12" s="11">
         <v>0</v>
@@ -2983,7 +3010,7 @@
     </row>
     <row r="13" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B13" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C13" s="13">
         <v>0</v>
@@ -3104,7 +3131,7 @@
     </row>
     <row r="14" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C14" s="11">
         <v>0</v>
@@ -3225,7 +3252,7 @@
     </row>
     <row r="15" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B15" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C15" s="13">
         <v>1</v>
@@ -3346,7 +3373,7 @@
     </row>
     <row r="16" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B16" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C16" s="13">
         <v>1</v>
@@ -3467,7 +3494,7 @@
     </row>
     <row r="17" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C17" s="3">
         <v>0</v>
@@ -3588,7 +3615,7 @@
     </row>
     <row r="18" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B18" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C18" s="3">
         <v>0</v>
@@ -3828,7 +3855,7 @@
     </row>
     <row r="20" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B20" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C20" s="13">
         <v>0</v>
@@ -3949,7 +3976,7 @@
     </row>
     <row r="21" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B21" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C21" s="13">
         <v>1</v>
@@ -4070,7 +4097,7 @@
     </row>
     <row r="22" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B22" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C22" s="11">
         <v>0</v>
@@ -4191,7 +4218,7 @@
     </row>
     <row r="23" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C23" s="11">
         <v>0</v>
@@ -4312,7 +4339,7 @@
     </row>
     <row r="24" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B24" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C24" s="13">
         <v>0</v>
@@ -4433,7 +4460,7 @@
     </row>
     <row r="25" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B25" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C25" s="13">
         <v>1</v>
@@ -4484,7 +4511,7 @@
         <v>1</v>
       </c>
       <c r="S25" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T25" s="12">
         <v>0</v>
@@ -4499,7 +4526,7 @@
         <v>1</v>
       </c>
       <c r="X25" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y25" s="11">
         <v>0</v>
@@ -4541,7 +4568,7 @@
       </c>
       <c r="AK25" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>99</v>
+        <v>1D</v>
       </c>
       <c r="AL25" s="5" t="str">
         <f t="shared" si="13"/>
@@ -4549,12 +4576,12 @@
       </c>
       <c r="AM25" t="str">
         <f t="shared" si="14"/>
-        <v>0xFFF39902</v>
+        <v>0xFFF31D02</v>
       </c>
     </row>
     <row r="26" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B26" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C26" s="13">
         <v>0</v>
@@ -4626,10 +4653,10 @@
         <v>0</v>
       </c>
       <c r="Z26" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA26" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB26" s="11">
         <v>0</v>
@@ -4662,15 +4689,15 @@
       </c>
       <c r="AK26" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>1C</v>
+        <v>1D</v>
       </c>
       <c r="AL26" s="5" t="str">
         <f t="shared" si="13"/>
-        <v>8A</v>
+        <v>0A</v>
       </c>
       <c r="AM26" t="str">
         <f t="shared" si="14"/>
-        <v>0x00301C8A</v>
+        <v>0x00301D0A</v>
       </c>
     </row>
     <row r="27" spans="2:39" x14ac:dyDescent="0.3">
@@ -4792,100 +4819,103 @@
       </c>
     </row>
     <row r="28" spans="2:39" x14ac:dyDescent="0.3">
-      <c r="C28" s="3">
-        <v>0</v>
-      </c>
-      <c r="D28" s="3">
-        <v>0</v>
-      </c>
-      <c r="E28" s="3">
-        <v>0</v>
-      </c>
-      <c r="F28" s="3">
-        <v>0</v>
-      </c>
-      <c r="G28" s="3">
-        <v>0</v>
-      </c>
-      <c r="H28" s="3">
-        <v>0</v>
-      </c>
-      <c r="I28" s="3">
-        <v>0</v>
-      </c>
-      <c r="J28" s="3">
-        <v>0</v>
-      </c>
-      <c r="K28" s="3">
-        <v>0</v>
-      </c>
-      <c r="L28" s="3">
-        <v>0</v>
-      </c>
-      <c r="M28" s="3">
-        <v>0</v>
-      </c>
-      <c r="N28" s="3">
-        <v>0</v>
-      </c>
-      <c r="O28" s="3">
-        <v>0</v>
-      </c>
-      <c r="P28" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="3">
-        <v>0</v>
-      </c>
-      <c r="R28" s="3">
-        <v>0</v>
-      </c>
-      <c r="S28" s="3">
-        <v>0</v>
-      </c>
-      <c r="T28" s="3">
-        <v>0</v>
-      </c>
-      <c r="U28" s="3">
-        <v>0</v>
-      </c>
-      <c r="V28" s="3">
-        <v>0</v>
-      </c>
-      <c r="W28" s="3">
-        <v>0</v>
-      </c>
-      <c r="X28" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y28" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z28" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA28" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB28" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC28" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD28" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE28" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF28" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG28" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH28" s="3">
+      <c r="B28" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="13">
+        <v>0</v>
+      </c>
+      <c r="D28" s="13">
+        <v>0</v>
+      </c>
+      <c r="E28" s="13">
+        <v>0</v>
+      </c>
+      <c r="F28" s="13">
+        <v>0</v>
+      </c>
+      <c r="G28" s="13">
+        <v>0</v>
+      </c>
+      <c r="H28" s="13">
+        <v>0</v>
+      </c>
+      <c r="I28" s="13">
+        <v>0</v>
+      </c>
+      <c r="J28" s="13">
+        <v>0</v>
+      </c>
+      <c r="K28" s="13">
+        <v>0</v>
+      </c>
+      <c r="L28" s="13">
+        <v>1</v>
+      </c>
+      <c r="M28" s="13">
+        <v>0</v>
+      </c>
+      <c r="N28" s="13">
+        <v>1</v>
+      </c>
+      <c r="O28" s="11">
+        <v>0</v>
+      </c>
+      <c r="P28" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="11">
+        <v>0</v>
+      </c>
+      <c r="R28" s="11">
+        <v>0</v>
+      </c>
+      <c r="S28" s="11">
+        <v>0</v>
+      </c>
+      <c r="T28" s="12">
+        <v>0</v>
+      </c>
+      <c r="U28" s="12">
+        <v>1</v>
+      </c>
+      <c r="V28" s="12">
+        <v>1</v>
+      </c>
+      <c r="W28" s="12">
+        <v>1</v>
+      </c>
+      <c r="X28" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB28" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC28" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE28" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF28" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG28" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH28" s="11">
         <v>0</v>
       </c>
       <c r="AI28" s="8" t="str">
@@ -4894,116 +4924,119 @@
       </c>
       <c r="AJ28" s="7" t="str">
         <f t="shared" si="16"/>
-        <v>00</v>
+        <v>50</v>
       </c>
       <c r="AK28" s="6" t="str">
         <f t="shared" si="17"/>
-        <v>00</v>
+        <v>38</v>
       </c>
       <c r="AL28" s="5" t="str">
         <f t="shared" si="18"/>
-        <v>00</v>
+        <v>82</v>
       </c>
       <c r="AM28" t="str">
         <f t="shared" si="19"/>
-        <v>0x00000000</v>
+        <v>0x00503882</v>
       </c>
     </row>
     <row r="29" spans="2:39" x14ac:dyDescent="0.3">
-      <c r="C29" s="3">
-        <v>0</v>
-      </c>
-      <c r="D29" s="3">
-        <v>0</v>
-      </c>
-      <c r="E29" s="3">
-        <v>0</v>
-      </c>
-      <c r="F29" s="3">
-        <v>0</v>
-      </c>
-      <c r="G29" s="3">
-        <v>0</v>
-      </c>
-      <c r="H29" s="3">
-        <v>0</v>
-      </c>
-      <c r="I29" s="3">
-        <v>0</v>
-      </c>
-      <c r="J29" s="3">
-        <v>0</v>
-      </c>
-      <c r="K29" s="3">
-        <v>0</v>
-      </c>
-      <c r="L29" s="3">
-        <v>0</v>
-      </c>
-      <c r="M29" s="3">
-        <v>0</v>
-      </c>
-      <c r="N29" s="3">
-        <v>0</v>
-      </c>
-      <c r="O29" s="3">
-        <v>0</v>
-      </c>
-      <c r="P29" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="3">
-        <v>0</v>
-      </c>
-      <c r="R29" s="3">
-        <v>0</v>
-      </c>
-      <c r="S29" s="3">
-        <v>0</v>
-      </c>
-      <c r="T29" s="3">
-        <v>0</v>
-      </c>
-      <c r="U29" s="3">
-        <v>0</v>
-      </c>
-      <c r="V29" s="3">
-        <v>0</v>
-      </c>
-      <c r="W29" s="3">
-        <v>0</v>
-      </c>
-      <c r="X29" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y29" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z29" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA29" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB29" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC29" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD29" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE29" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF29" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG29" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH29" s="3">
+      <c r="B29" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" s="11">
+        <v>0</v>
+      </c>
+      <c r="D29" s="11">
+        <v>0</v>
+      </c>
+      <c r="E29" s="11">
+        <v>0</v>
+      </c>
+      <c r="F29" s="11">
+        <v>0</v>
+      </c>
+      <c r="G29" s="11">
+        <v>0</v>
+      </c>
+      <c r="H29" s="11">
+        <v>0</v>
+      </c>
+      <c r="I29" s="11">
+        <v>0</v>
+      </c>
+      <c r="J29" s="12">
+        <v>0</v>
+      </c>
+      <c r="K29" s="12">
+        <v>0</v>
+      </c>
+      <c r="L29" s="12">
+        <v>0</v>
+      </c>
+      <c r="M29" s="12">
+        <v>0</v>
+      </c>
+      <c r="N29" s="12">
+        <v>0</v>
+      </c>
+      <c r="O29" s="11">
+        <v>0</v>
+      </c>
+      <c r="P29" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="11">
+        <v>0</v>
+      </c>
+      <c r="R29" s="11">
+        <v>0</v>
+      </c>
+      <c r="S29" s="11">
+        <v>0</v>
+      </c>
+      <c r="T29" s="12">
+        <v>0</v>
+      </c>
+      <c r="U29" s="12">
+        <v>1</v>
+      </c>
+      <c r="V29" s="12">
+        <v>1</v>
+      </c>
+      <c r="W29" s="12">
+        <v>1</v>
+      </c>
+      <c r="X29" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y29" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA29" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB29" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC29" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE29" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF29" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG29" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH29" s="11">
         <v>0</v>
       </c>
       <c r="AI29" s="8" t="str">
@@ -5016,112 +5049,115 @@
       </c>
       <c r="AK29" s="6" t="str">
         <f t="shared" si="17"/>
-        <v>00</v>
+        <v>3C</v>
       </c>
       <c r="AL29" s="5" t="str">
         <f t="shared" si="18"/>
-        <v>00</v>
+        <v>80</v>
       </c>
       <c r="AM29" t="str">
         <f t="shared" si="19"/>
-        <v>0x00000000</v>
+        <v>0x00003C80</v>
       </c>
     </row>
     <row r="30" spans="2:39" x14ac:dyDescent="0.3">
-      <c r="C30" s="3">
-        <v>0</v>
-      </c>
-      <c r="D30" s="3">
-        <v>0</v>
-      </c>
-      <c r="E30" s="3">
-        <v>0</v>
-      </c>
-      <c r="F30" s="3">
-        <v>0</v>
-      </c>
-      <c r="G30" s="3">
-        <v>0</v>
-      </c>
-      <c r="H30" s="3">
-        <v>0</v>
-      </c>
-      <c r="I30" s="3">
-        <v>0</v>
-      </c>
-      <c r="J30" s="3">
-        <v>0</v>
-      </c>
-      <c r="K30" s="3">
-        <v>0</v>
-      </c>
-      <c r="L30" s="3">
-        <v>0</v>
-      </c>
-      <c r="M30" s="3">
-        <v>0</v>
-      </c>
-      <c r="N30" s="3">
-        <v>0</v>
-      </c>
-      <c r="O30" s="3">
-        <v>0</v>
-      </c>
-      <c r="P30" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="3">
-        <v>0</v>
-      </c>
-      <c r="R30" s="3">
-        <v>0</v>
-      </c>
-      <c r="S30" s="3">
-        <v>0</v>
-      </c>
-      <c r="T30" s="3">
-        <v>0</v>
-      </c>
-      <c r="U30" s="3">
-        <v>0</v>
-      </c>
-      <c r="V30" s="3">
-        <v>0</v>
-      </c>
-      <c r="W30" s="3">
-        <v>0</v>
-      </c>
-      <c r="X30" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y30" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z30" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA30" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB30" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC30" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD30" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE30" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF30" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG30" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH30" s="3">
+      <c r="B30" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="13">
+        <v>0</v>
+      </c>
+      <c r="D30" s="13">
+        <v>0</v>
+      </c>
+      <c r="E30" s="13">
+        <v>0</v>
+      </c>
+      <c r="F30" s="13">
+        <v>0</v>
+      </c>
+      <c r="G30" s="13">
+        <v>0</v>
+      </c>
+      <c r="H30" s="13">
+        <v>0</v>
+      </c>
+      <c r="I30" s="13">
+        <v>0</v>
+      </c>
+      <c r="J30" s="13">
+        <v>0</v>
+      </c>
+      <c r="K30" s="13">
+        <v>0</v>
+      </c>
+      <c r="L30" s="13">
+        <v>0</v>
+      </c>
+      <c r="M30" s="13">
+        <v>1</v>
+      </c>
+      <c r="N30" s="13">
+        <v>0</v>
+      </c>
+      <c r="O30" s="11">
+        <v>0</v>
+      </c>
+      <c r="P30" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="11">
+        <v>0</v>
+      </c>
+      <c r="R30" s="11">
+        <v>0</v>
+      </c>
+      <c r="S30" s="11">
+        <v>0</v>
+      </c>
+      <c r="T30" s="12">
+        <v>1</v>
+      </c>
+      <c r="U30" s="12">
+        <v>0</v>
+      </c>
+      <c r="V30" s="12">
+        <v>0</v>
+      </c>
+      <c r="W30" s="12">
+        <v>0</v>
+      </c>
+      <c r="X30" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB30" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC30" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE30" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF30" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG30" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH30" s="11">
         <v>0</v>
       </c>
       <c r="AI30" s="8" t="str">
@@ -5130,116 +5166,119 @@
       </c>
       <c r="AJ30" s="7" t="str">
         <f t="shared" si="16"/>
-        <v>00</v>
+        <v>20</v>
       </c>
       <c r="AK30" s="6" t="str">
         <f t="shared" si="17"/>
-        <v>00</v>
+        <v>40</v>
       </c>
       <c r="AL30" s="5" t="str">
         <f t="shared" si="18"/>
-        <v>00</v>
+        <v>82</v>
       </c>
       <c r="AM30" t="str">
         <f t="shared" si="19"/>
-        <v>0x00000000</v>
+        <v>0x00204082</v>
       </c>
     </row>
     <row r="31" spans="2:39" x14ac:dyDescent="0.3">
-      <c r="C31" s="3">
-        <v>0</v>
-      </c>
-      <c r="D31" s="3">
-        <v>0</v>
-      </c>
-      <c r="E31" s="3">
-        <v>0</v>
-      </c>
-      <c r="F31" s="3">
-        <v>0</v>
-      </c>
-      <c r="G31" s="3">
-        <v>0</v>
-      </c>
-      <c r="H31" s="3">
-        <v>0</v>
-      </c>
-      <c r="I31" s="3">
-        <v>0</v>
-      </c>
-      <c r="J31" s="3">
-        <v>0</v>
-      </c>
-      <c r="K31" s="3">
-        <v>0</v>
-      </c>
-      <c r="L31" s="3">
-        <v>0</v>
-      </c>
-      <c r="M31" s="3">
-        <v>0</v>
-      </c>
-      <c r="N31" s="3">
-        <v>0</v>
-      </c>
-      <c r="O31" s="3">
-        <v>0</v>
-      </c>
-      <c r="P31" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="3">
-        <v>0</v>
-      </c>
-      <c r="R31" s="3">
-        <v>0</v>
-      </c>
-      <c r="S31" s="3">
-        <v>0</v>
-      </c>
-      <c r="T31" s="3">
-        <v>0</v>
-      </c>
-      <c r="U31" s="3">
-        <v>0</v>
-      </c>
-      <c r="V31" s="3">
-        <v>0</v>
-      </c>
-      <c r="W31" s="3">
-        <v>0</v>
-      </c>
-      <c r="X31" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y31" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z31" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA31" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB31" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC31" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD31" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE31" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF31" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG31" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH31" s="3">
+      <c r="B31" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="13">
+        <v>0</v>
+      </c>
+      <c r="D31" s="13">
+        <v>0</v>
+      </c>
+      <c r="E31" s="13">
+        <v>0</v>
+      </c>
+      <c r="F31" s="13">
+        <v>0</v>
+      </c>
+      <c r="G31" s="13">
+        <v>0</v>
+      </c>
+      <c r="H31" s="13">
+        <v>0</v>
+      </c>
+      <c r="I31" s="13">
+        <v>0</v>
+      </c>
+      <c r="J31" s="13">
+        <v>0</v>
+      </c>
+      <c r="K31" s="13">
+        <v>0</v>
+      </c>
+      <c r="L31" s="13">
+        <v>0</v>
+      </c>
+      <c r="M31" s="13">
+        <v>0</v>
+      </c>
+      <c r="N31" s="13">
+        <v>1</v>
+      </c>
+      <c r="O31" s="11">
+        <v>0</v>
+      </c>
+      <c r="P31" s="11">
+        <v>1</v>
+      </c>
+      <c r="Q31" s="11">
+        <v>1</v>
+      </c>
+      <c r="R31" s="11">
+        <v>1</v>
+      </c>
+      <c r="S31" s="11">
+        <v>1</v>
+      </c>
+      <c r="T31" s="12">
+        <v>1</v>
+      </c>
+      <c r="U31" s="12">
+        <v>0</v>
+      </c>
+      <c r="V31" s="12">
+        <v>0</v>
+      </c>
+      <c r="W31" s="12">
+        <v>0</v>
+      </c>
+      <c r="X31" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y31" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA31" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB31" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG31" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH31" s="11">
         <v>0</v>
       </c>
       <c r="AI31" s="8" t="str">
@@ -5248,129 +5287,132 @@
       </c>
       <c r="AJ31" s="7" t="str">
         <f t="shared" si="16"/>
-        <v>00</v>
+        <v>17</v>
       </c>
       <c r="AK31" s="6" t="str">
         <f t="shared" si="17"/>
-        <v>00</v>
+        <v>C4</v>
       </c>
       <c r="AL31" s="5" t="str">
         <f t="shared" si="18"/>
-        <v>00</v>
+        <v>82</v>
       </c>
       <c r="AM31" t="str">
         <f t="shared" si="19"/>
-        <v>0x00000000</v>
+        <v>0x0017C482</v>
       </c>
     </row>
     <row r="32" spans="2:39" x14ac:dyDescent="0.3">
-      <c r="C32" s="3">
-        <v>0</v>
-      </c>
-      <c r="D32" s="3">
-        <v>0</v>
-      </c>
-      <c r="E32" s="3">
-        <v>0</v>
-      </c>
-      <c r="F32" s="3">
-        <v>0</v>
-      </c>
-      <c r="G32" s="3">
-        <v>0</v>
-      </c>
-      <c r="H32" s="3">
-        <v>0</v>
-      </c>
-      <c r="I32" s="3">
-        <v>0</v>
-      </c>
-      <c r="J32" s="3">
-        <v>0</v>
-      </c>
-      <c r="K32" s="3">
-        <v>0</v>
-      </c>
-      <c r="L32" s="3">
-        <v>0</v>
-      </c>
-      <c r="M32" s="3">
-        <v>0</v>
-      </c>
-      <c r="N32" s="3">
-        <v>0</v>
-      </c>
-      <c r="O32" s="3">
-        <v>0</v>
-      </c>
-      <c r="P32" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="3">
-        <v>0</v>
-      </c>
-      <c r="R32" s="3">
-        <v>0</v>
-      </c>
-      <c r="S32" s="3">
-        <v>0</v>
-      </c>
-      <c r="T32" s="3">
-        <v>0</v>
-      </c>
-      <c r="U32" s="3">
-        <v>0</v>
-      </c>
-      <c r="V32" s="3">
-        <v>0</v>
-      </c>
-      <c r="W32" s="3">
-        <v>0</v>
-      </c>
-      <c r="X32" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y32" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z32" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA32" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB32" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC32" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD32" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE32" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF32" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG32" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH32" s="3">
+      <c r="B32" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" s="11">
+        <v>0</v>
+      </c>
+      <c r="D32" s="11">
+        <v>0</v>
+      </c>
+      <c r="E32" s="11">
+        <v>0</v>
+      </c>
+      <c r="F32" s="11">
+        <v>0</v>
+      </c>
+      <c r="G32" s="11">
+        <v>0</v>
+      </c>
+      <c r="H32" s="11">
+        <v>0</v>
+      </c>
+      <c r="I32" s="11">
+        <v>0</v>
+      </c>
+      <c r="J32" s="12">
+        <v>1</v>
+      </c>
+      <c r="K32" s="12">
+        <v>0</v>
+      </c>
+      <c r="L32" s="12">
+        <v>0</v>
+      </c>
+      <c r="M32" s="12">
+        <v>0</v>
+      </c>
+      <c r="N32" s="12">
+        <v>0</v>
+      </c>
+      <c r="O32" s="11">
+        <v>1</v>
+      </c>
+      <c r="P32" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="11">
+        <v>0</v>
+      </c>
+      <c r="R32" s="11">
+        <v>0</v>
+      </c>
+      <c r="S32" s="11">
+        <v>1</v>
+      </c>
+      <c r="T32" s="12">
+        <v>1</v>
+      </c>
+      <c r="U32" s="12">
+        <v>0</v>
+      </c>
+      <c r="V32" s="12">
+        <v>0</v>
+      </c>
+      <c r="W32" s="12">
+        <v>0</v>
+      </c>
+      <c r="X32" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y32" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z32" s="11">
+        <v>1</v>
+      </c>
+      <c r="AA32" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB32" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC32" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD32" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE32" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF32" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG32" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH32" s="11">
         <v>0</v>
       </c>
       <c r="AI32" s="8" t="str">
         <f t="shared" si="15"/>
-        <v>00</v>
+        <v>01</v>
       </c>
       <c r="AJ32" s="7" t="str">
         <f t="shared" si="16"/>
-        <v>00</v>
+        <v>08</v>
       </c>
       <c r="AK32" s="6" t="str">
         <f t="shared" si="17"/>
-        <v>00</v>
+        <v>C5</v>
       </c>
       <c r="AL32" s="5" t="str">
         <f t="shared" si="18"/>
@@ -5378,104 +5420,107 @@
       </c>
       <c r="AM32" t="str">
         <f t="shared" si="19"/>
-        <v>0x00000000</v>
+        <v>0x0108C500</v>
       </c>
     </row>
-    <row r="33" spans="3:39" x14ac:dyDescent="0.3">
-      <c r="C33" s="3">
-        <v>0</v>
-      </c>
-      <c r="D33" s="3">
-        <v>0</v>
-      </c>
-      <c r="E33" s="3">
-        <v>0</v>
-      </c>
-      <c r="F33" s="3">
-        <v>0</v>
-      </c>
-      <c r="G33" s="3">
-        <v>0</v>
-      </c>
-      <c r="H33" s="3">
-        <v>0</v>
-      </c>
-      <c r="I33" s="3">
-        <v>0</v>
-      </c>
-      <c r="J33" s="3">
-        <v>0</v>
-      </c>
-      <c r="K33" s="3">
-        <v>0</v>
-      </c>
-      <c r="L33" s="3">
-        <v>0</v>
-      </c>
-      <c r="M33" s="3">
-        <v>0</v>
-      </c>
-      <c r="N33" s="3">
-        <v>0</v>
-      </c>
-      <c r="O33" s="3">
-        <v>0</v>
-      </c>
-      <c r="P33" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q33" s="3">
-        <v>0</v>
-      </c>
-      <c r="R33" s="3">
-        <v>0</v>
-      </c>
-      <c r="S33" s="3">
-        <v>0</v>
-      </c>
-      <c r="T33" s="3">
-        <v>0</v>
-      </c>
-      <c r="U33" s="3">
-        <v>0</v>
-      </c>
-      <c r="V33" s="3">
-        <v>0</v>
-      </c>
-      <c r="W33" s="3">
-        <v>0</v>
-      </c>
-      <c r="X33" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y33" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z33" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA33" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB33" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC33" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD33" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE33" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF33" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG33" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH33" s="3">
+    <row r="33" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="B33" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C33" s="13">
+        <v>0</v>
+      </c>
+      <c r="D33" s="13">
+        <v>0</v>
+      </c>
+      <c r="E33" s="13">
+        <v>0</v>
+      </c>
+      <c r="F33" s="13">
+        <v>0</v>
+      </c>
+      <c r="G33" s="13">
+        <v>0</v>
+      </c>
+      <c r="H33" s="13">
+        <v>0</v>
+      </c>
+      <c r="I33" s="13">
+        <v>0</v>
+      </c>
+      <c r="J33" s="13">
+        <v>0</v>
+      </c>
+      <c r="K33" s="13">
+        <v>0</v>
+      </c>
+      <c r="L33" s="13">
+        <v>0</v>
+      </c>
+      <c r="M33" s="13">
+        <v>0</v>
+      </c>
+      <c r="N33" s="13">
+        <v>1</v>
+      </c>
+      <c r="O33" s="11">
+        <v>0</v>
+      </c>
+      <c r="P33" s="11">
+        <v>1</v>
+      </c>
+      <c r="Q33" s="11">
+        <v>1</v>
+      </c>
+      <c r="R33" s="11">
+        <v>1</v>
+      </c>
+      <c r="S33" s="11">
+        <v>1</v>
+      </c>
+      <c r="T33" s="12">
+        <v>0</v>
+      </c>
+      <c r="U33" s="12">
+        <v>1</v>
+      </c>
+      <c r="V33" s="12">
+        <v>1</v>
+      </c>
+      <c r="W33" s="12">
+        <v>1</v>
+      </c>
+      <c r="X33" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y33" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z33" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA33" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB33" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC33" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD33" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE33" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF33" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG33" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH33" s="11">
         <v>0</v>
       </c>
       <c r="AI33" s="8" t="str">
@@ -5484,234 +5529,240 @@
       </c>
       <c r="AJ33" s="7" t="str">
         <f t="shared" si="16"/>
-        <v>00</v>
+        <v>17</v>
       </c>
       <c r="AK33" s="6" t="str">
         <f t="shared" si="17"/>
-        <v>00</v>
+        <v>BC</v>
       </c>
       <c r="AL33" s="5" t="str">
         <f t="shared" si="18"/>
-        <v>00</v>
+        <v>82</v>
       </c>
       <c r="AM33" t="str">
         <f t="shared" si="19"/>
-        <v>0x00000000</v>
+        <v>0x0017BC82</v>
       </c>
     </row>
-    <row r="34" spans="3:39" x14ac:dyDescent="0.3">
-      <c r="C34" s="3">
-        <v>0</v>
-      </c>
-      <c r="D34" s="3">
-        <v>0</v>
-      </c>
-      <c r="E34" s="3">
-        <v>0</v>
-      </c>
-      <c r="F34" s="3">
-        <v>0</v>
-      </c>
-      <c r="G34" s="3">
-        <v>0</v>
-      </c>
-      <c r="H34" s="3">
-        <v>0</v>
-      </c>
-      <c r="I34" s="3">
-        <v>0</v>
-      </c>
-      <c r="J34" s="3">
-        <v>0</v>
-      </c>
-      <c r="K34" s="3">
-        <v>0</v>
-      </c>
-      <c r="L34" s="3">
-        <v>0</v>
-      </c>
-      <c r="M34" s="3">
-        <v>0</v>
-      </c>
-      <c r="N34" s="3">
-        <v>0</v>
-      </c>
-      <c r="O34" s="3">
-        <v>0</v>
-      </c>
-      <c r="P34" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="3">
-        <v>0</v>
-      </c>
-      <c r="R34" s="3">
-        <v>0</v>
-      </c>
-      <c r="S34" s="3">
-        <v>0</v>
-      </c>
-      <c r="T34" s="3">
-        <v>0</v>
-      </c>
-      <c r="U34" s="3">
-        <v>0</v>
-      </c>
-      <c r="V34" s="3">
-        <v>0</v>
-      </c>
-      <c r="W34" s="3">
-        <v>0</v>
-      </c>
-      <c r="X34" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y34" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG34" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH34" s="3">
+    <row r="34" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="B34" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" s="13">
+        <v>1</v>
+      </c>
+      <c r="D34" s="13">
+        <v>1</v>
+      </c>
+      <c r="E34" s="13">
+        <v>1</v>
+      </c>
+      <c r="F34" s="13">
+        <v>1</v>
+      </c>
+      <c r="G34" s="13">
+        <v>1</v>
+      </c>
+      <c r="H34" s="13">
+        <v>1</v>
+      </c>
+      <c r="I34" s="13">
+        <v>1</v>
+      </c>
+      <c r="J34" s="12">
+        <v>0</v>
+      </c>
+      <c r="K34" s="12">
+        <v>1</v>
+      </c>
+      <c r="L34" s="12">
+        <v>1</v>
+      </c>
+      <c r="M34" s="12">
+        <v>1</v>
+      </c>
+      <c r="N34" s="12">
+        <v>0</v>
+      </c>
+      <c r="O34" s="11">
+        <v>0</v>
+      </c>
+      <c r="P34" s="11">
+        <v>1</v>
+      </c>
+      <c r="Q34" s="11">
+        <v>1</v>
+      </c>
+      <c r="R34" s="11">
+        <v>1</v>
+      </c>
+      <c r="S34" s="11">
+        <v>1</v>
+      </c>
+      <c r="T34" s="13">
+        <v>1</v>
+      </c>
+      <c r="U34" s="13">
+        <v>1</v>
+      </c>
+      <c r="V34" s="13">
+        <v>1</v>
+      </c>
+      <c r="W34" s="13">
+        <v>0</v>
+      </c>
+      <c r="X34" s="13">
+        <v>1</v>
+      </c>
+      <c r="Y34" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z34" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA34" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB34" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC34" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD34" s="12">
+        <v>1</v>
+      </c>
+      <c r="AE34" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF34" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG34" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH34" s="11">
         <v>0</v>
       </c>
       <c r="AI34" s="8" t="str">
         <f t="shared" si="15"/>
-        <v>00</v>
+        <v>FE</v>
       </c>
       <c r="AJ34" s="7" t="str">
         <f t="shared" si="16"/>
-        <v>00</v>
+        <v>E7</v>
       </c>
       <c r="AK34" s="6" t="str">
         <f t="shared" si="17"/>
-        <v>00</v>
+        <v>F4</v>
       </c>
       <c r="AL34" s="5" t="str">
         <f t="shared" si="18"/>
-        <v>00</v>
+        <v>90</v>
       </c>
       <c r="AM34" t="str">
         <f t="shared" si="19"/>
-        <v>0x00000000</v>
+        <v>0xFEE7F490</v>
       </c>
     </row>
-    <row r="35" spans="3:39" x14ac:dyDescent="0.3">
-      <c r="C35" s="3">
-        <v>0</v>
-      </c>
-      <c r="D35" s="3">
-        <v>0</v>
-      </c>
-      <c r="E35" s="3">
-        <v>0</v>
-      </c>
-      <c r="F35" s="3">
-        <v>0</v>
-      </c>
-      <c r="G35" s="3">
-        <v>0</v>
-      </c>
-      <c r="H35" s="3">
-        <v>0</v>
-      </c>
-      <c r="I35" s="3">
-        <v>0</v>
-      </c>
-      <c r="J35" s="3">
-        <v>0</v>
-      </c>
-      <c r="K35" s="3">
-        <v>0</v>
-      </c>
-      <c r="L35" s="3">
-        <v>0</v>
-      </c>
-      <c r="M35" s="3">
-        <v>0</v>
-      </c>
-      <c r="N35" s="3">
-        <v>0</v>
-      </c>
-      <c r="O35" s="3">
-        <v>0</v>
-      </c>
-      <c r="P35" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q35" s="3">
-        <v>0</v>
-      </c>
-      <c r="R35" s="3">
-        <v>0</v>
-      </c>
-      <c r="S35" s="3">
-        <v>0</v>
-      </c>
-      <c r="T35" s="3">
-        <v>0</v>
-      </c>
-      <c r="U35" s="3">
-        <v>0</v>
-      </c>
-      <c r="V35" s="3">
-        <v>0</v>
-      </c>
-      <c r="W35" s="3">
-        <v>0</v>
-      </c>
-      <c r="X35" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y35" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z35" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA35" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB35" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC35" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD35" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE35" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF35" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG35" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH35" s="3">
+    <row r="35" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="B35" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" s="13">
+        <v>0</v>
+      </c>
+      <c r="D35" s="13">
+        <v>0</v>
+      </c>
+      <c r="E35" s="13">
+        <v>0</v>
+      </c>
+      <c r="F35" s="13">
+        <v>0</v>
+      </c>
+      <c r="G35" s="13">
+        <v>0</v>
+      </c>
+      <c r="H35" s="13">
+        <v>0</v>
+      </c>
+      <c r="I35" s="13">
+        <v>0</v>
+      </c>
+      <c r="J35" s="13">
+        <v>0</v>
+      </c>
+      <c r="K35" s="13">
+        <v>0</v>
+      </c>
+      <c r="L35" s="13">
+        <v>1</v>
+      </c>
+      <c r="M35" s="13">
+        <v>0</v>
+      </c>
+      <c r="N35" s="13">
+        <v>0</v>
+      </c>
+      <c r="O35" s="11">
+        <v>0</v>
+      </c>
+      <c r="P35" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="11">
+        <v>0</v>
+      </c>
+      <c r="R35" s="11">
+        <v>0</v>
+      </c>
+      <c r="S35" s="11">
+        <v>0</v>
+      </c>
+      <c r="T35" s="12">
+        <v>1</v>
+      </c>
+      <c r="U35" s="12">
+        <v>0</v>
+      </c>
+      <c r="V35" s="12">
+        <v>0</v>
+      </c>
+      <c r="W35" s="12">
+        <v>0</v>
+      </c>
+      <c r="X35" s="12">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="11">
+        <v>1</v>
+      </c>
+      <c r="Z35" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA35" s="11">
+        <v>0</v>
+      </c>
+      <c r="AB35" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC35" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD35" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE35" s="12">
+        <v>1</v>
+      </c>
+      <c r="AF35" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG35" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH35" s="11">
         <v>0</v>
       </c>
       <c r="AI35" s="8" t="str">
@@ -5720,140 +5771,143 @@
       </c>
       <c r="AJ35" s="7" t="str">
         <f t="shared" si="16"/>
-        <v>00</v>
+        <v>40</v>
       </c>
       <c r="AK35" s="6" t="str">
         <f t="shared" si="17"/>
-        <v>00</v>
+        <v>42</v>
       </c>
       <c r="AL35" s="5" t="str">
         <f t="shared" si="18"/>
-        <v>00</v>
+        <v>0A</v>
       </c>
       <c r="AM35" t="str">
         <f t="shared" si="19"/>
-        <v>0x00000000</v>
+        <v>0x0040420A</v>
       </c>
     </row>
-    <row r="36" spans="3:39" x14ac:dyDescent="0.3">
-      <c r="C36" s="3">
-        <v>0</v>
-      </c>
-      <c r="D36" s="3">
-        <v>0</v>
-      </c>
-      <c r="E36" s="3">
-        <v>0</v>
-      </c>
-      <c r="F36" s="3">
-        <v>0</v>
-      </c>
-      <c r="G36" s="3">
-        <v>0</v>
-      </c>
-      <c r="H36" s="3">
-        <v>0</v>
-      </c>
-      <c r="I36" s="3">
-        <v>0</v>
-      </c>
-      <c r="J36" s="3">
-        <v>0</v>
-      </c>
-      <c r="K36" s="3">
-        <v>0</v>
-      </c>
-      <c r="L36" s="3">
-        <v>0</v>
-      </c>
-      <c r="M36" s="3">
-        <v>0</v>
-      </c>
-      <c r="N36" s="3">
-        <v>0</v>
-      </c>
-      <c r="O36" s="3">
-        <v>0</v>
-      </c>
-      <c r="P36" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q36" s="3">
-        <v>0</v>
-      </c>
-      <c r="R36" s="3">
-        <v>0</v>
-      </c>
-      <c r="S36" s="3">
-        <v>0</v>
-      </c>
-      <c r="T36" s="3">
-        <v>0</v>
-      </c>
-      <c r="U36" s="3">
-        <v>0</v>
-      </c>
-      <c r="V36" s="3">
-        <v>0</v>
-      </c>
-      <c r="W36" s="3">
-        <v>0</v>
-      </c>
-      <c r="X36" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y36" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z36" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA36" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB36" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC36" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD36" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE36" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF36" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG36" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH36" s="3">
+    <row r="36" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="B36" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C36" s="13">
+        <v>1</v>
+      </c>
+      <c r="D36" s="13">
+        <v>1</v>
+      </c>
+      <c r="E36" s="13">
+        <v>1</v>
+      </c>
+      <c r="F36" s="13">
+        <v>1</v>
+      </c>
+      <c r="G36" s="13">
+        <v>1</v>
+      </c>
+      <c r="H36" s="13">
+        <v>1</v>
+      </c>
+      <c r="I36" s="13">
+        <v>1</v>
+      </c>
+      <c r="J36" s="13">
+        <v>1</v>
+      </c>
+      <c r="K36" s="13">
+        <v>1</v>
+      </c>
+      <c r="L36" s="13">
+        <v>1</v>
+      </c>
+      <c r="M36" s="13">
+        <v>1</v>
+      </c>
+      <c r="N36" s="13">
+        <v>0</v>
+      </c>
+      <c r="O36" s="11">
+        <v>0</v>
+      </c>
+      <c r="P36" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="11">
+        <v>0</v>
+      </c>
+      <c r="R36" s="11">
+        <v>0</v>
+      </c>
+      <c r="S36" s="11">
+        <v>0</v>
+      </c>
+      <c r="T36" s="12">
+        <v>0</v>
+      </c>
+      <c r="U36" s="12">
+        <v>1</v>
+      </c>
+      <c r="V36" s="12">
+        <v>1</v>
+      </c>
+      <c r="W36" s="12">
+        <v>1</v>
+      </c>
+      <c r="X36" s="12">
+        <v>1</v>
+      </c>
+      <c r="Y36" s="11">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="11">
+        <v>0</v>
+      </c>
+      <c r="AA36" s="11">
+        <v>1</v>
+      </c>
+      <c r="AB36" s="11">
+        <v>1</v>
+      </c>
+      <c r="AC36" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE36" s="12">
+        <v>1</v>
+      </c>
+      <c r="AF36" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG36" s="12">
+        <v>1</v>
+      </c>
+      <c r="AH36" s="11">
         <v>0</v>
       </c>
       <c r="AI36" s="8" t="str">
         <f t="shared" si="15"/>
-        <v>00</v>
+        <v>FF</v>
       </c>
       <c r="AJ36" s="7" t="str">
         <f t="shared" si="16"/>
-        <v>00</v>
+        <v>E0</v>
       </c>
       <c r="AK36" s="6" t="str">
         <f t="shared" si="17"/>
-        <v>00</v>
+        <v>3C</v>
       </c>
       <c r="AL36" s="5" t="str">
         <f t="shared" si="18"/>
-        <v>00</v>
+        <v>CA</v>
       </c>
       <c r="AM36" t="str">
         <f t="shared" si="19"/>
-        <v>0x00000000</v>
+        <v>0xFFE03CCA</v>
       </c>
     </row>
-    <row r="37" spans="3:39" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:39" x14ac:dyDescent="0.3">
       <c r="C37" s="3">
         <v>0</v>
       </c>
@@ -5971,7 +6025,7 @@
         <v>0x00000000</v>
       </c>
     </row>
-    <row r="38" spans="3:39" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:39" x14ac:dyDescent="0.3">
       <c r="C38" s="3">
         <v>0</v>
       </c>
@@ -6089,7 +6143,7 @@
         <v>0x00000000</v>
       </c>
     </row>
-    <row r="39" spans="3:39" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:39" x14ac:dyDescent="0.3">
       <c r="C39" s="3">
         <v>0</v>
       </c>
@@ -6207,7 +6261,7 @@
         <v>0x00000000</v>
       </c>
     </row>
-    <row r="40" spans="3:39" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:39" x14ac:dyDescent="0.3">
       <c r="C40" s="3">
         <v>0</v>
       </c>
@@ -6325,7 +6379,7 @@
         <v>0x00000000</v>
       </c>
     </row>
-    <row r="41" spans="3:39" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:39" x14ac:dyDescent="0.3">
       <c r="C41" s="3">
         <v>0</v>
       </c>
@@ -6443,7 +6497,7 @@
         <v>0x00000000</v>
       </c>
     </row>
-    <row r="42" spans="3:39" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:39" x14ac:dyDescent="0.3">
       <c r="C42" s="3">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
feat(sv): pruebas del datapath con un programa del compilador
</commit_message>
<xml_diff>
--- a/res/isa.xlsx
+++ b/res/isa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\workbench\repos\CE4301--p2_fobando_isa--\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1767F53-2BD2-4D61-A744-BF5ADE48C286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B030CB-2F16-4B4F-98C8-24E7BAE08A6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{EC7525CD-E51C-4E61-B306-9CBCE090E85A}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="89">
   <si>
     <t>R</t>
   </si>
@@ -304,6 +304,9 @@
   </si>
   <si>
     <t xml:space="preserve">muli r2, r0, 2 </t>
+  </si>
+  <si>
+    <t>addi r0, r1, 4</t>
   </si>
 </sst>
 </file>
@@ -6859,7 +6862,7 @@
         <v>81</v>
       </c>
       <c r="AM43" t="str">
-        <f t="shared" ref="AM43:AM49" si="24">_xlfn.CONCAT("0x",AI43:AL43)</f>
+        <f t="shared" ref="AM43:AM47" si="24">_xlfn.CONCAT("0x",AI43:AL43)</f>
         <v>0x00F74081</v>
       </c>
     </row>
@@ -7453,15 +7456,15 @@
         <v>E0</v>
       </c>
       <c r="AK48" s="6" t="str">
-        <f>BIN2HEX(_xlfn.CONCAT(S48:Z48),2)</f>
+        <f t="shared" ref="AK48:AK56" si="26">BIN2HEX(_xlfn.CONCAT(S48:Z48),2)</f>
         <v>38</v>
       </c>
       <c r="AL48" s="5" t="str">
-        <f t="shared" ref="AL48" si="26">BIN2HEX(_xlfn.CONCAT(AA48:AH48),2)</f>
+        <f t="shared" ref="AL48" si="27">BIN2HEX(_xlfn.CONCAT(AA48:AH48),2)</f>
         <v>82</v>
       </c>
       <c r="AM48" t="str">
-        <f>_xlfn.CONCAT("0x",AI48:AL48)</f>
+        <f t="shared" ref="AM48:AM56" si="28">_xlfn.CONCAT("0x",AI48:AL48)</f>
         <v>0xFFE03882</v>
       </c>
     </row>
@@ -7574,7 +7577,7 @@
         <v>00</v>
       </c>
       <c r="AK49" s="6" t="str">
-        <f>BIN2HEX(_xlfn.CONCAT(S49:Z49),2)</f>
+        <f t="shared" si="26"/>
         <v>10</v>
       </c>
       <c r="AL49" s="5" t="str">
@@ -7582,7 +7585,7 @@
         <v>22</v>
       </c>
       <c r="AM49" t="str">
-        <f>_xlfn.CONCAT("0x",AI49:AL49)</f>
+        <f t="shared" si="28"/>
         <v>0x00001022</v>
       </c>
     </row>
@@ -7687,23 +7690,23 @@
         <v>0</v>
       </c>
       <c r="AI50" s="8" t="str">
-        <f t="shared" ref="AI50:AI52" si="27">BIN2HEX(_xlfn.CONCAT(C50:J50),2)</f>
+        <f t="shared" ref="AI50:AI52" si="29">BIN2HEX(_xlfn.CONCAT(C50:J50),2)</f>
         <v>00</v>
       </c>
       <c r="AJ50" s="7" t="str">
-        <f t="shared" ref="AJ50:AJ52" si="28">BIN2HEX(_xlfn.CONCAT(K50:R50),2)</f>
+        <f t="shared" ref="AJ50:AJ52" si="30">BIN2HEX(_xlfn.CONCAT(K50:R50),2)</f>
         <v>07</v>
       </c>
       <c r="AK50" s="6" t="str">
-        <f>BIN2HEX(_xlfn.CONCAT(S50:Z50),2)</f>
+        <f t="shared" si="26"/>
         <v>0C</v>
       </c>
       <c r="AL50" s="5" t="str">
-        <f t="shared" ref="AL50:AL52" si="29">BIN2HEX(_xlfn.CONCAT(AA50:AH50),2)</f>
+        <f t="shared" ref="AL50:AL52" si="31">BIN2HEX(_xlfn.CONCAT(AA50:AH50),2)</f>
         <v>20</v>
       </c>
       <c r="AM50" t="str">
-        <f>_xlfn.CONCAT("0x",AI50:AL50)</f>
+        <f t="shared" si="28"/>
         <v>0x00070C20</v>
       </c>
     </row>
@@ -7808,23 +7811,23 @@
         <v>0</v>
       </c>
       <c r="AI51" s="8" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>00</v>
       </c>
       <c r="AJ51" s="7" t="str">
+        <f t="shared" si="30"/>
+        <v>06</v>
+      </c>
+      <c r="AK51" s="6" t="str">
+        <f t="shared" si="26"/>
+        <v>0D</v>
+      </c>
+      <c r="AL51" s="5" t="str">
+        <f t="shared" si="31"/>
+        <v>0E</v>
+      </c>
+      <c r="AM51" t="str">
         <f t="shared" si="28"/>
-        <v>06</v>
-      </c>
-      <c r="AK51" s="6" t="str">
-        <f>BIN2HEX(_xlfn.CONCAT(S51:Z51),2)</f>
-        <v>0D</v>
-      </c>
-      <c r="AL51" s="5" t="str">
-        <f t="shared" si="29"/>
-        <v>0E</v>
-      </c>
-      <c r="AM51" t="str">
-        <f>_xlfn.CONCAT("0x",AI51:AL51)</f>
         <v>0x00060D0E</v>
       </c>
     </row>
@@ -7929,23 +7932,23 @@
         <v>0</v>
       </c>
       <c r="AI52" s="8" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="29"/>
         <v>00</v>
       </c>
       <c r="AJ52" s="7" t="str">
+        <f t="shared" si="30"/>
+        <v>04</v>
+      </c>
+      <c r="AK52" s="6" t="str">
+        <f t="shared" si="26"/>
+        <v>0C</v>
+      </c>
+      <c r="AL52" s="5" t="str">
+        <f t="shared" si="31"/>
+        <v>8C</v>
+      </c>
+      <c r="AM52" t="str">
         <f t="shared" si="28"/>
-        <v>04</v>
-      </c>
-      <c r="AK52" s="6" t="str">
-        <f>BIN2HEX(_xlfn.CONCAT(S52:Z52),2)</f>
-        <v>0C</v>
-      </c>
-      <c r="AL52" s="5" t="str">
-        <f t="shared" si="29"/>
-        <v>8C</v>
-      </c>
-      <c r="AM52" t="str">
-        <f>_xlfn.CONCAT("0x",AI52:AL52)</f>
         <v>0x00040C8C</v>
       </c>
     </row>
@@ -8058,7 +8061,7 @@
         <v>07</v>
       </c>
       <c r="AK53" s="6" t="str">
-        <f>BIN2HEX(_xlfn.CONCAT(S53:Z53),2)</f>
+        <f t="shared" si="26"/>
         <v>28</v>
       </c>
       <c r="AL53" s="5" t="str">
@@ -8066,7 +8069,7 @@
         <v>86</v>
       </c>
       <c r="AM53" t="str">
-        <f>_xlfn.CONCAT("0x",AI53:AL53)</f>
+        <f t="shared" si="28"/>
         <v>0x00072886</v>
       </c>
     </row>
@@ -8179,7 +8182,7 @@
         <v>03</v>
       </c>
       <c r="AK54" s="6" t="str">
-        <f>BIN2HEX(_xlfn.CONCAT(S54:Z54),2)</f>
+        <f t="shared" si="26"/>
         <v>55</v>
       </c>
       <c r="AL54" s="5" t="str">
@@ -8187,7 +8190,7 @@
         <v>04</v>
       </c>
       <c r="AM54" t="str">
-        <f>_xlfn.CONCAT("0x",AI54:AL54)</f>
+        <f t="shared" si="28"/>
         <v>0x00035504</v>
       </c>
     </row>
@@ -8300,7 +8303,7 @@
         <v>05</v>
       </c>
       <c r="AK55" s="6" t="str">
-        <f>BIN2HEX(_xlfn.CONCAT(S55:Z55),2)</f>
+        <f t="shared" si="26"/>
         <v>3C</v>
       </c>
       <c r="AL55" s="5" t="str">
@@ -8308,7 +8311,7 @@
         <v>60</v>
       </c>
       <c r="AM55" t="str">
-        <f>_xlfn.CONCAT("0x",AI55:AL55)</f>
+        <f t="shared" si="28"/>
         <v>0x00053C60</v>
       </c>
     </row>
@@ -8421,7 +8424,7 @@
         <v>00</v>
       </c>
       <c r="AK56" s="6" t="str">
-        <f>BIN2HEX(_xlfn.CONCAT(S56:Z56),2)</f>
+        <f t="shared" si="26"/>
         <v>00</v>
       </c>
       <c r="AL56" s="5" t="str">
@@ -8429,7 +8432,7 @@
         <v>62</v>
       </c>
       <c r="AM56" t="str">
-        <f>_xlfn.CONCAT("0x",AI56:AL56)</f>
+        <f t="shared" si="28"/>
         <v>0x00000062</v>
       </c>
     </row>
@@ -8531,23 +8534,23 @@
         <v>0</v>
       </c>
       <c r="AI57" s="8" t="str">
-        <f t="shared" ref="AI52:AI62" si="30">BIN2HEX(_xlfn.CONCAT(C57:J57),2)</f>
+        <f t="shared" ref="AI57:AI62" si="32">BIN2HEX(_xlfn.CONCAT(C57:J57),2)</f>
         <v>00</v>
       </c>
       <c r="AJ57" s="7" t="str">
-        <f t="shared" ref="AJ52:AJ62" si="31">BIN2HEX(_xlfn.CONCAT(K57:R57),2)</f>
+        <f t="shared" ref="AJ57:AJ62" si="33">BIN2HEX(_xlfn.CONCAT(K57:R57),2)</f>
         <v>00</v>
       </c>
       <c r="AK57" s="6" t="str">
-        <f t="shared" ref="AK52:AK62" si="32">BIN2HEX(_xlfn.CONCAT(S57:Z57),2)</f>
+        <f t="shared" ref="AK57:AK62" si="34">BIN2HEX(_xlfn.CONCAT(S57:Z57),2)</f>
         <v>00</v>
       </c>
       <c r="AL57" s="5" t="str">
-        <f t="shared" ref="AL52:AL62" si="33">BIN2HEX(_xlfn.CONCAT(AA57:AH57),2)</f>
+        <f t="shared" ref="AL57:AL62" si="35">BIN2HEX(_xlfn.CONCAT(AA57:AH57),2)</f>
         <v>00</v>
       </c>
       <c r="AM57" t="str">
-        <f t="shared" ref="AM50:AM62" si="34">_xlfn.CONCAT("0x",AI57:AL57)</f>
+        <f t="shared" ref="AM57:AM62" si="36">_xlfn.CONCAT("0x",AI57:AL57)</f>
         <v>0x00000000</v>
       </c>
     </row>
@@ -8652,23 +8655,23 @@
         <v>0</v>
       </c>
       <c r="AI58" s="8" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>00</v>
       </c>
       <c r="AJ58" s="7" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>30</v>
       </c>
       <c r="AK58" s="6" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>38</v>
       </c>
       <c r="AL58" s="5" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>82</v>
       </c>
       <c r="AM58" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>0x00303882</v>
       </c>
     </row>
@@ -8773,23 +8776,23 @@
         <v>0</v>
       </c>
       <c r="AI59" s="8" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>00</v>
       </c>
       <c r="AJ59" s="7" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>00</v>
       </c>
       <c r="AK59" s="6" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>04</v>
       </c>
       <c r="AL59" s="5" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>52</v>
       </c>
       <c r="AM59" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>0x00000452</v>
       </c>
     </row>
@@ -8837,13 +8840,13 @@
         <v>0</v>
       </c>
       <c r="P60" s="17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q60" s="17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R60" s="17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S60" s="17">
         <v>0</v>
@@ -8861,7 +8864,7 @@
         <v>1</v>
       </c>
       <c r="X60" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y60" s="14">
         <v>0</v>
@@ -8894,24 +8897,24 @@
         <v>0</v>
       </c>
       <c r="AI60" s="8" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>00</v>
       </c>
       <c r="AJ60" s="7" t="str">
-        <f t="shared" si="31"/>
-        <v>40</v>
+        <f t="shared" si="33"/>
+        <v>47</v>
       </c>
       <c r="AK60" s="6" t="str">
-        <f t="shared" si="32"/>
-        <v>38</v>
+        <f t="shared" si="34"/>
+        <v>3C</v>
       </c>
       <c r="AL60" s="5" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>82</v>
       </c>
       <c r="AM60" t="str">
-        <f t="shared" si="34"/>
-        <v>0x00403882</v>
+        <f t="shared" si="36"/>
+        <v>0x00473C82</v>
       </c>
     </row>
     <row r="61" spans="2:39" x14ac:dyDescent="0.3">
@@ -9015,23 +9018,23 @@
         <v>0</v>
       </c>
       <c r="AI61" s="8" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>00</v>
       </c>
       <c r="AJ61" s="7" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>41</v>
       </c>
       <c r="AK61" s="6" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>8C</v>
       </c>
       <c r="AL61" s="5" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>82</v>
       </c>
       <c r="AM61" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>0x00418C82</v>
       </c>
     </row>
@@ -9136,23 +9139,23 @@
         <v>0</v>
       </c>
       <c r="AI62" s="8" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>00</v>
       </c>
       <c r="AJ62" s="7" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>57</v>
       </c>
       <c r="AK62" s="6" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="34"/>
         <v>40</v>
       </c>
       <c r="AL62" s="5" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="35"/>
         <v>82</v>
       </c>
       <c r="AM62" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="36"/>
         <v>0x00574082</v>
       </c>
     </row>
@@ -9257,23 +9260,23 @@
         <v>0</v>
       </c>
       <c r="AI63" s="8" t="str">
-        <f t="shared" ref="AI63:AI66" si="35">BIN2HEX(_xlfn.CONCAT(C63:J63),2)</f>
+        <f t="shared" ref="AI63:AI66" si="37">BIN2HEX(_xlfn.CONCAT(C63:J63),2)</f>
         <v>00</v>
       </c>
       <c r="AJ63" s="7" t="str">
-        <f t="shared" ref="AJ63:AJ66" si="36">BIN2HEX(_xlfn.CONCAT(K63:R63),2)</f>
+        <f t="shared" ref="AJ63:AJ66" si="38">BIN2HEX(_xlfn.CONCAT(K63:R63),2)</f>
         <v>27</v>
       </c>
       <c r="AK63" s="6" t="str">
-        <f t="shared" ref="AK63:AK66" si="37">BIN2HEX(_xlfn.CONCAT(S63:Z63),2)</f>
+        <f t="shared" ref="AK63:AK66" si="39">BIN2HEX(_xlfn.CONCAT(S63:Z63),2)</f>
         <v>41</v>
       </c>
       <c r="AL63" s="5" t="str">
-        <f t="shared" ref="AL63:AL66" si="38">BIN2HEX(_xlfn.CONCAT(AA63:AH63),2)</f>
+        <f t="shared" ref="AL63:AL66" si="40">BIN2HEX(_xlfn.CONCAT(AA63:AH63),2)</f>
         <v>02</v>
       </c>
       <c r="AM63" t="str">
-        <f t="shared" ref="AM63:AM66" si="39">_xlfn.CONCAT("0x",AI63:AL63)</f>
+        <f t="shared" ref="AM63:AM66" si="41">_xlfn.CONCAT("0x",AI63:AL63)</f>
         <v>0x00274102</v>
       </c>
     </row>
@@ -9375,259 +9378,262 @@
         <v>0</v>
       </c>
       <c r="AI64" s="8" t="str">
-        <f t="shared" si="35"/>
-        <v>00</v>
-      </c>
-      <c r="AJ64" s="7" t="str">
-        <f t="shared" si="36"/>
-        <v>00</v>
-      </c>
-      <c r="AK64" s="6" t="str">
         <f t="shared" si="37"/>
         <v>00</v>
       </c>
-      <c r="AL64" s="5" t="str">
+      <c r="AJ64" s="7" t="str">
         <f t="shared" si="38"/>
         <v>00</v>
       </c>
+      <c r="AK64" s="6" t="str">
+        <f t="shared" si="39"/>
+        <v>00</v>
+      </c>
+      <c r="AL64" s="5" t="str">
+        <f t="shared" si="40"/>
+        <v>00</v>
+      </c>
       <c r="AM64" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v>0x00000000</v>
       </c>
     </row>
-    <row r="65" spans="3:39" x14ac:dyDescent="0.3">
-      <c r="C65" s="3">
-        <v>0</v>
-      </c>
-      <c r="D65" s="3">
-        <v>0</v>
-      </c>
-      <c r="E65" s="3">
-        <v>0</v>
-      </c>
-      <c r="F65" s="3">
-        <v>0</v>
-      </c>
-      <c r="G65" s="3">
-        <v>0</v>
-      </c>
-      <c r="H65" s="3">
-        <v>0</v>
-      </c>
-      <c r="I65" s="3">
-        <v>0</v>
-      </c>
-      <c r="J65" s="3">
-        <v>0</v>
-      </c>
-      <c r="K65" s="3">
-        <v>0</v>
-      </c>
-      <c r="L65" s="3">
-        <v>0</v>
-      </c>
-      <c r="M65" s="3">
-        <v>0</v>
-      </c>
-      <c r="N65" s="3">
-        <v>0</v>
-      </c>
-      <c r="O65" s="3">
-        <v>0</v>
-      </c>
-      <c r="P65" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q65" s="3">
-        <v>0</v>
-      </c>
-      <c r="R65" s="3">
-        <v>0</v>
-      </c>
-      <c r="S65" s="3">
-        <v>0</v>
-      </c>
-      <c r="T65" s="3">
-        <v>0</v>
-      </c>
-      <c r="U65" s="3">
-        <v>0</v>
-      </c>
-      <c r="V65" s="3">
-        <v>0</v>
-      </c>
-      <c r="W65" s="3">
-        <v>0</v>
-      </c>
-      <c r="X65" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y65" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z65" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA65" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB65" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC65" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD65" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE65" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF65" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG65" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH65" s="3">
+    <row r="65" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="B65" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C65" s="12">
+        <v>0</v>
+      </c>
+      <c r="D65" s="12">
+        <v>0</v>
+      </c>
+      <c r="E65" s="12">
+        <v>0</v>
+      </c>
+      <c r="F65" s="12">
+        <v>0</v>
+      </c>
+      <c r="G65" s="12">
+        <v>0</v>
+      </c>
+      <c r="H65" s="12">
+        <v>0</v>
+      </c>
+      <c r="I65" s="12">
+        <v>0</v>
+      </c>
+      <c r="J65" s="12">
+        <v>0</v>
+      </c>
+      <c r="K65" s="12">
+        <v>0</v>
+      </c>
+      <c r="L65" s="12">
+        <v>1</v>
+      </c>
+      <c r="M65" s="12">
+        <v>0</v>
+      </c>
+      <c r="N65" s="12">
+        <v>0</v>
+      </c>
+      <c r="O65" s="17">
+        <v>0</v>
+      </c>
+      <c r="P65" s="17">
+        <v>1</v>
+      </c>
+      <c r="Q65" s="17">
+        <v>1</v>
+      </c>
+      <c r="R65" s="17">
+        <v>1</v>
+      </c>
+      <c r="S65" s="17">
+        <v>1</v>
+      </c>
+      <c r="T65" s="15">
+        <v>0</v>
+      </c>
+      <c r="U65" s="15">
+        <v>1</v>
+      </c>
+      <c r="V65" s="15">
+        <v>1</v>
+      </c>
+      <c r="W65" s="15">
+        <v>1</v>
+      </c>
+      <c r="X65" s="15">
+        <v>0</v>
+      </c>
+      <c r="Y65" s="14">
+        <v>0</v>
+      </c>
+      <c r="Z65" s="14">
+        <v>0</v>
+      </c>
+      <c r="AA65" s="14">
+        <v>1</v>
+      </c>
+      <c r="AB65" s="14">
+        <v>0</v>
+      </c>
+      <c r="AC65" s="13">
+        <v>0</v>
+      </c>
+      <c r="AD65" s="13">
+        <v>0</v>
+      </c>
+      <c r="AE65" s="13">
+        <v>0</v>
+      </c>
+      <c r="AF65" s="13">
+        <v>0</v>
+      </c>
+      <c r="AG65" s="13">
+        <v>1</v>
+      </c>
+      <c r="AH65" s="16">
         <v>0</v>
       </c>
       <c r="AI65" s="8" t="str">
-        <f t="shared" si="35"/>
-        <v>00</v>
-      </c>
-      <c r="AJ65" s="7" t="str">
-        <f t="shared" si="36"/>
-        <v>00</v>
-      </c>
-      <c r="AK65" s="6" t="str">
         <f t="shared" si="37"/>
         <v>00</v>
       </c>
+      <c r="AJ65" s="7" t="str">
+        <f t="shared" si="38"/>
+        <v>47</v>
+      </c>
+      <c r="AK65" s="6" t="str">
+        <f t="shared" si="39"/>
+        <v>B8</v>
+      </c>
       <c r="AL65" s="5" t="str">
+        <f t="shared" si="40"/>
+        <v>82</v>
+      </c>
+      <c r="AM65" t="str">
+        <f t="shared" si="41"/>
+        <v>0x0047B882</v>
+      </c>
+    </row>
+    <row r="66" spans="2:39" x14ac:dyDescent="0.3">
+      <c r="C66" s="3">
+        <v>0</v>
+      </c>
+      <c r="D66" s="3">
+        <v>0</v>
+      </c>
+      <c r="E66" s="3">
+        <v>0</v>
+      </c>
+      <c r="F66" s="3">
+        <v>0</v>
+      </c>
+      <c r="G66" s="3">
+        <v>0</v>
+      </c>
+      <c r="H66" s="3">
+        <v>0</v>
+      </c>
+      <c r="I66" s="3">
+        <v>0</v>
+      </c>
+      <c r="J66" s="3">
+        <v>0</v>
+      </c>
+      <c r="K66" s="3">
+        <v>0</v>
+      </c>
+      <c r="L66" s="3">
+        <v>0</v>
+      </c>
+      <c r="M66" s="3">
+        <v>0</v>
+      </c>
+      <c r="N66" s="3">
+        <v>0</v>
+      </c>
+      <c r="O66" s="3">
+        <v>0</v>
+      </c>
+      <c r="P66" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q66" s="3">
+        <v>0</v>
+      </c>
+      <c r="R66" s="3">
+        <v>0</v>
+      </c>
+      <c r="S66" s="3">
+        <v>0</v>
+      </c>
+      <c r="T66" s="3">
+        <v>0</v>
+      </c>
+      <c r="U66" s="3">
+        <v>0</v>
+      </c>
+      <c r="V66" s="3">
+        <v>0</v>
+      </c>
+      <c r="W66" s="3">
+        <v>0</v>
+      </c>
+      <c r="X66" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y66" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI66" s="8" t="str">
+        <f t="shared" si="37"/>
+        <v>00</v>
+      </c>
+      <c r="AJ66" s="7" t="str">
         <f t="shared" si="38"/>
         <v>00</v>
       </c>
-      <c r="AM65" t="str">
+      <c r="AK66" s="6" t="str">
         <f t="shared" si="39"/>
-        <v>0x00000000</v>
-      </c>
-    </row>
-    <row r="66" spans="3:39" x14ac:dyDescent="0.3">
-      <c r="C66" s="3">
-        <v>0</v>
-      </c>
-      <c r="D66" s="3">
-        <v>0</v>
-      </c>
-      <c r="E66" s="3">
-        <v>0</v>
-      </c>
-      <c r="F66" s="3">
-        <v>0</v>
-      </c>
-      <c r="G66" s="3">
-        <v>0</v>
-      </c>
-      <c r="H66" s="3">
-        <v>0</v>
-      </c>
-      <c r="I66" s="3">
-        <v>0</v>
-      </c>
-      <c r="J66" s="3">
-        <v>0</v>
-      </c>
-      <c r="K66" s="3">
-        <v>0</v>
-      </c>
-      <c r="L66" s="3">
-        <v>0</v>
-      </c>
-      <c r="M66" s="3">
-        <v>0</v>
-      </c>
-      <c r="N66" s="3">
-        <v>0</v>
-      </c>
-      <c r="O66" s="3">
-        <v>0</v>
-      </c>
-      <c r="P66" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q66" s="3">
-        <v>0</v>
-      </c>
-      <c r="R66" s="3">
-        <v>0</v>
-      </c>
-      <c r="S66" s="3">
-        <v>0</v>
-      </c>
-      <c r="T66" s="3">
-        <v>0</v>
-      </c>
-      <c r="U66" s="3">
-        <v>0</v>
-      </c>
-      <c r="V66" s="3">
-        <v>0</v>
-      </c>
-      <c r="W66" s="3">
-        <v>0</v>
-      </c>
-      <c r="X66" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y66" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z66" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA66" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB66" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC66" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD66" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE66" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF66" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG66" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH66" s="3">
-        <v>0</v>
-      </c>
-      <c r="AI66" s="8" t="str">
-        <f t="shared" si="35"/>
         <v>00</v>
       </c>
-      <c r="AJ66" s="7" t="str">
-        <f t="shared" si="36"/>
+      <c r="AL66" s="5" t="str">
+        <f t="shared" si="40"/>
         <v>00</v>
       </c>
-      <c r="AK66" s="6" t="str">
-        <f t="shared" si="37"/>
-        <v>00</v>
-      </c>
-      <c r="AL66" s="5" t="str">
-        <f t="shared" si="38"/>
-        <v>00</v>
-      </c>
       <c r="AM66" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="41"/>
         <v>0x00000000</v>
       </c>
     </row>

</xml_diff>